<commit_message>
Set fixed talla curve S12 XL18 2XL13 and LA VELA 350 und
- Fixed production curve: S 12%, M 25%, L 32%, XL 18%, 2XL 13%
- LA VELA store allocation fixed at 350 units minimum
- Remaining units distributed to other stores by sales weight

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SHORT_PLAYA_CAB_Cantidades_Sugeridas_Proyecciones.xlsx
+++ b/SHORT_PLAYA_CAB_Cantidades_Sugeridas_Proyecciones.xlsx
@@ -23,7 +23,7 @@
     <t>CANTIDADES POR COLORES</t>
   </si>
   <si>
-    <t>SHORT PLAYA CAB liso · Sin 3XL · Curva tallas = ventas globales CAB · Habano/Azul Verdoso/Azul Pizzarra al 70% tela · ≤50 und → solo M, L, XL · Sin sublimado</t>
+    <t>SHORT PLAYA CAB · S12 M25 L32 XL18 2XL13 · LA VELA 350 und · Habano/Azul Verdoso/Azul Pizzarra 70% tela · ≤50 und → M/L/XL</t>
   </si>
   <si>
     <t>Rango producción: 802 – 856 und</t>
@@ -110,7 +110,7 @@
     <t>SHORT PLAYA CAB — CANTIDADES POR TALLA (MÍN / MÁX)</t>
   </si>
   <si>
-    <t>Curva referencia ventas globales CAB liso: S 12.5% · M 25.2% · L 32.3% · XL 14.6% · 2XL 15.4%</t>
+    <t>Curva fija: S 12% · M 25% · L 32% · XL 18% · 2XL 13%</t>
   </si>
   <si>
     <t>Talla</t>
@@ -182,7 +182,7 @@
     <t>SHORT PLAYA CAB — DISTRIBUCIÓN POR TIENDA Y TALLA</t>
   </si>
   <si>
-    <t>★ LA VELA / TOLON · MGTA playa priorizada (VELA 1,5× GRIETA)</t>
+    <t>★ LA VELA = 350 und mín · resto tiendas por peso ventas</t>
   </si>
   <si>
     <t>Tienda</t>
@@ -754,7 +754,7 @@
         <v>11</v>
       </c>
       <c r="B7">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C7">
         <v>47</v>
@@ -763,10 +763,10 @@
         <v>60</v>
       </c>
       <c r="E7">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="F7">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="G7">
         <v>187</v>
@@ -777,19 +777,19 @@
         <v>12</v>
       </c>
       <c r="B8">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C8">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D8">
         <v>49</v>
       </c>
       <c r="E8">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F8">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="G8">
         <v>153</v>
@@ -800,7 +800,7 @@
         <v>13</v>
       </c>
       <c r="B9">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C9">
         <v>38</v>
@@ -809,10 +809,10 @@
         <v>49</v>
       </c>
       <c r="E9">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="F9">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="G9">
         <v>152</v>
@@ -823,7 +823,7 @@
         <v>14</v>
       </c>
       <c r="B10">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C10">
         <v>25</v>
@@ -832,10 +832,10 @@
         <v>33</v>
       </c>
       <c r="E10">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F10">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G10">
         <v>101</v>
@@ -846,7 +846,7 @@
         <v>15</v>
       </c>
       <c r="B11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C11">
         <v>22</v>
@@ -855,10 +855,10 @@
         <v>28</v>
       </c>
       <c r="E11">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F11">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G11">
         <v>86</v>
@@ -875,10 +875,10 @@
         <v>13</v>
       </c>
       <c r="D12">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E12">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -898,10 +898,10 @@
         <v>13</v>
       </c>
       <c r="D13">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E13">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -921,10 +921,10 @@
         <v>11</v>
       </c>
       <c r="D14">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E14">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F14">
         <v>0</v>
@@ -944,10 +944,10 @@
         <v>5</v>
       </c>
       <c r="D15">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F15">
         <v>0</v>
@@ -961,19 +961,19 @@
         <v>20</v>
       </c>
       <c r="B16" s="3">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="C16" s="3">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D16" s="3">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="E16" s="3">
-        <v>124</v>
+        <v>152</v>
       </c>
       <c r="F16" s="3">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="G16" s="3">
         <v>802</v>
@@ -1012,19 +1012,19 @@
         <v>22</v>
       </c>
       <c r="B20">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C20">
         <v>50</v>
       </c>
       <c r="D20">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E20">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="F20">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="G20">
         <v>199</v>
@@ -1041,13 +1041,13 @@
         <v>41</v>
       </c>
       <c r="D21">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E21">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F21">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="G21">
         <v>163</v>
@@ -1058,7 +1058,7 @@
         <v>24</v>
       </c>
       <c r="B22">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C22">
         <v>41</v>
@@ -1067,10 +1067,10 @@
         <v>52</v>
       </c>
       <c r="E22">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F22">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="G22">
         <v>162</v>
@@ -1090,10 +1090,10 @@
         <v>35</v>
       </c>
       <c r="E23">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F23">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G23">
         <v>108</v>
@@ -1104,19 +1104,19 @@
         <v>15</v>
       </c>
       <c r="B24">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C24">
         <v>23</v>
       </c>
       <c r="D24">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E24">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F24">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G24">
         <v>92</v>
@@ -1133,10 +1133,10 @@
         <v>14</v>
       </c>
       <c r="D25">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E25">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -1156,10 +1156,10 @@
         <v>14</v>
       </c>
       <c r="D26">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E26">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F26">
         <v>0</v>
@@ -1176,13 +1176,13 @@
         <v>0</v>
       </c>
       <c r="C27">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D27">
         <v>15</v>
       </c>
       <c r="E27">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F27">
         <v>0</v>
@@ -1199,13 +1199,13 @@
         <v>0</v>
       </c>
       <c r="C28">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D28">
         <v>7</v>
       </c>
       <c r="E28">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F28">
         <v>0</v>
@@ -1219,19 +1219,19 @@
         <v>20</v>
       </c>
       <c r="B29" s="3">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C29" s="3">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D29" s="3">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="E29" s="3">
-        <v>132</v>
+        <v>162</v>
       </c>
       <c r="F29" s="3">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="G29" s="3">
         <v>856</v>
@@ -1276,13 +1276,13 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>0.125</v>
+        <v>0.12</v>
       </c>
       <c r="C5">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D5">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1290,13 +1290,13 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>0.252</v>
+        <v>0.25</v>
       </c>
       <c r="C6">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D6">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1304,13 +1304,13 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>0.323</v>
+        <v>0.32</v>
       </c>
       <c r="C7">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="D7">
-        <v>294</v>
+        <v>287</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1318,13 +1318,13 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>0.146</v>
+        <v>0.18</v>
       </c>
       <c r="C8">
-        <v>124</v>
+        <v>152</v>
       </c>
       <c r="D8">
-        <v>132</v>
+        <v>162</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1332,13 +1332,13 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>0.154</v>
+        <v>0.13</v>
       </c>
       <c r="C9">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="D9">
-        <v>112</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -1403,10 +1403,10 @@
         <v>5</v>
       </c>
       <c r="B6">
+        <v>22</v>
+      </c>
+      <c r="C6">
         <v>24</v>
-      </c>
-      <c r="C6">
-        <v>25</v>
       </c>
       <c r="D6">
         <v>3.1</v>
@@ -1446,7 +1446,7 @@
         <v>60</v>
       </c>
       <c r="C8">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D8">
         <v>7.3</v>
@@ -1463,10 +1463,10 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="C9">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="D9">
         <v>3.5</v>
@@ -1483,10 +1483,10 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C10">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="D10">
         <v>3.8</v>
@@ -1542,7 +1542,7 @@
         <v>5</v>
       </c>
       <c r="B15">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C15">
         <v>20</v>
@@ -1562,7 +1562,7 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C16">
         <v>41</v>
@@ -1585,7 +1585,7 @@
         <v>49</v>
       </c>
       <c r="C17">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D17">
         <v>7.7</v>
@@ -1602,10 +1602,10 @@
         <v>8</v>
       </c>
       <c r="B18">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C18">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="D18">
         <v>4.6</v>
@@ -1622,10 +1622,10 @@
         <v>9</v>
       </c>
       <c r="B19">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C19">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D19">
         <v>4</v>
@@ -1681,10 +1681,10 @@
         <v>5</v>
       </c>
       <c r="B24">
+        <v>18</v>
+      </c>
+      <c r="C24">
         <v>19</v>
-      </c>
-      <c r="C24">
-        <v>20</v>
       </c>
       <c r="D24">
         <v>4.2</v>
@@ -1741,10 +1741,10 @@
         <v>8</v>
       </c>
       <c r="B27">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C27">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="D27">
         <v>5.4</v>
@@ -1761,10 +1761,10 @@
         <v>9</v>
       </c>
       <c r="B28">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C28">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D28">
         <v>5.2</v>
@@ -1820,7 +1820,7 @@
         <v>5</v>
       </c>
       <c r="B33">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C33">
         <v>13</v>
@@ -1880,10 +1880,10 @@
         <v>8</v>
       </c>
       <c r="B36">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C36">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D36">
         <v>5.2</v>
@@ -1900,10 +1900,10 @@
         <v>9</v>
       </c>
       <c r="B37">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C37">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D37">
         <v>2.7</v>
@@ -1959,10 +1959,10 @@
         <v>5</v>
       </c>
       <c r="B42">
+        <v>10</v>
+      </c>
+      <c r="C42">
         <v>11</v>
-      </c>
-      <c r="C42">
-        <v>12</v>
       </c>
       <c r="D42">
         <v>2.5</v>
@@ -2002,7 +2002,7 @@
         <v>28</v>
       </c>
       <c r="C44">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D44">
         <v>7.7</v>
@@ -2019,10 +2019,10 @@
         <v>8</v>
       </c>
       <c r="B45">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C45">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D45">
         <v>4.8</v>
@@ -2039,10 +2039,10 @@
         <v>9</v>
       </c>
       <c r="B46">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C46">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D46">
         <v>2.5</v>
@@ -2118,10 +2118,10 @@
         <v>7</v>
       </c>
       <c r="B52">
+        <v>16</v>
+      </c>
+      <c r="C52">
         <v>17</v>
-      </c>
-      <c r="C52">
-        <v>19</v>
       </c>
       <c r="D52">
         <v>0</v>
@@ -2138,10 +2138,10 @@
         <v>8</v>
       </c>
       <c r="B53">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C53">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D53">
         <v>0.2</v>
@@ -2217,10 +2217,10 @@
         <v>7</v>
       </c>
       <c r="B59">
+        <v>16</v>
+      </c>
+      <c r="C59">
         <v>17</v>
-      </c>
-      <c r="C59">
-        <v>19</v>
       </c>
       <c r="D59">
         <v>0</v>
@@ -2237,10 +2237,10 @@
         <v>8</v>
       </c>
       <c r="B60">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C60">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D60">
         <v>0</v>
@@ -2299,7 +2299,7 @@
         <v>11</v>
       </c>
       <c r="C65">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D65">
         <v>0.2</v>
@@ -2316,7 +2316,7 @@
         <v>7</v>
       </c>
       <c r="B66">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C66">
         <v>15</v>
@@ -2336,10 +2336,10 @@
         <v>8</v>
       </c>
       <c r="B67">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C67">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D67">
         <v>0.2</v>
@@ -2398,7 +2398,7 @@
         <v>5</v>
       </c>
       <c r="C72">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D72">
         <v>0</v>
@@ -2415,7 +2415,7 @@
         <v>7</v>
       </c>
       <c r="B73">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C73">
         <v>7</v>
@@ -2435,10 +2435,10 @@
         <v>8</v>
       </c>
       <c r="B74">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C74">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D74">
         <v>0</v>
@@ -2551,37 +2551,37 @@
         <v>56</v>
       </c>
       <c r="B6">
+        <v>13</v>
+      </c>
+      <c r="C6">
+        <v>14</v>
+      </c>
+      <c r="D6">
+        <v>27</v>
+      </c>
+      <c r="E6">
+        <v>30</v>
+      </c>
+      <c r="F6">
+        <v>35</v>
+      </c>
+      <c r="G6">
+        <v>38</v>
+      </c>
+      <c r="H6">
+        <v>20</v>
+      </c>
+      <c r="I6">
+        <v>21</v>
+      </c>
+      <c r="J6">
+        <v>14</v>
+      </c>
+      <c r="K6">
         <v>15</v>
       </c>
-      <c r="C6">
-        <v>16</v>
-      </c>
-      <c r="D6">
-        <v>38</v>
-      </c>
-      <c r="E6">
-        <v>41</v>
-      </c>
-      <c r="F6">
-        <v>49</v>
-      </c>
-      <c r="G6">
-        <v>52</v>
-      </c>
-      <c r="H6">
-        <v>22</v>
-      </c>
-      <c r="I6">
-        <v>23</v>
-      </c>
-      <c r="J6">
-        <v>19</v>
-      </c>
-      <c r="K6">
-        <v>20</v>
-      </c>
       <c r="L6">
-        <v>143</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -2589,37 +2589,37 @@
         <v>57</v>
       </c>
       <c r="B7">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="C7">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="D7">
-        <v>57</v>
+        <v>88</v>
       </c>
       <c r="E7">
-        <v>61</v>
+        <v>93</v>
       </c>
       <c r="F7">
-        <v>73</v>
+        <v>112</v>
       </c>
       <c r="G7">
-        <v>78</v>
+        <v>119</v>
       </c>
       <c r="H7">
-        <v>33</v>
+        <v>63</v>
       </c>
       <c r="I7">
-        <v>35</v>
+        <v>67</v>
       </c>
       <c r="J7">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="K7">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="L7">
-        <v>214</v>
+        <v>350</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -2627,37 +2627,37 @@
         <v>58</v>
       </c>
       <c r="B8">
+        <v>13</v>
+      </c>
+      <c r="C8">
+        <v>14</v>
+      </c>
+      <c r="D8">
+        <v>27</v>
+      </c>
+      <c r="E8">
+        <v>29</v>
+      </c>
+      <c r="F8">
+        <v>34</v>
+      </c>
+      <c r="G8">
+        <v>37</v>
+      </c>
+      <c r="H8">
+        <v>19</v>
+      </c>
+      <c r="I8">
+        <v>20</v>
+      </c>
+      <c r="J8">
+        <v>14</v>
+      </c>
+      <c r="K8">
         <v>15</v>
       </c>
-      <c r="C8">
-        <v>16</v>
-      </c>
-      <c r="D8">
-        <v>37</v>
-      </c>
-      <c r="E8">
-        <v>40</v>
-      </c>
-      <c r="F8">
-        <v>48</v>
-      </c>
-      <c r="G8">
-        <v>51</v>
-      </c>
-      <c r="H8">
-        <v>22</v>
-      </c>
-      <c r="I8">
-        <v>23</v>
-      </c>
-      <c r="J8">
-        <v>18</v>
-      </c>
-      <c r="K8">
-        <v>19</v>
-      </c>
       <c r="L8">
-        <v>140</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -2665,37 +2665,37 @@
         <v>59</v>
       </c>
       <c r="B9">
+        <v>12</v>
+      </c>
+      <c r="C9">
+        <v>13</v>
+      </c>
+      <c r="D9">
+        <v>26</v>
+      </c>
+      <c r="E9">
+        <v>27</v>
+      </c>
+      <c r="F9">
+        <v>33</v>
+      </c>
+      <c r="G9">
+        <v>35</v>
+      </c>
+      <c r="H9">
+        <v>18</v>
+      </c>
+      <c r="I9">
+        <v>20</v>
+      </c>
+      <c r="J9">
+        <v>13</v>
+      </c>
+      <c r="K9">
         <v>14</v>
       </c>
-      <c r="C9">
-        <v>15</v>
-      </c>
-      <c r="D9">
-        <v>35</v>
-      </c>
-      <c r="E9">
-        <v>38</v>
-      </c>
-      <c r="F9">
-        <v>45</v>
-      </c>
-      <c r="G9">
-        <v>49</v>
-      </c>
-      <c r="H9">
-        <v>20</v>
-      </c>
-      <c r="I9">
-        <v>22</v>
-      </c>
-      <c r="J9">
-        <v>17</v>
-      </c>
-      <c r="K9">
-        <v>18</v>
-      </c>
       <c r="L9">
-        <v>131</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -2703,37 +2703,37 @@
         <v>60</v>
       </c>
       <c r="B10">
+        <v>12</v>
+      </c>
+      <c r="C10">
+        <v>13</v>
+      </c>
+      <c r="D10">
+        <v>26</v>
+      </c>
+      <c r="E10">
+        <v>28</v>
+      </c>
+      <c r="F10">
+        <v>33</v>
+      </c>
+      <c r="G10">
+        <v>35</v>
+      </c>
+      <c r="H10">
+        <v>18</v>
+      </c>
+      <c r="I10">
+        <v>20</v>
+      </c>
+      <c r="J10">
+        <v>13</v>
+      </c>
+      <c r="K10">
         <v>14</v>
       </c>
-      <c r="C10">
-        <v>15</v>
-      </c>
-      <c r="D10">
-        <v>35</v>
-      </c>
-      <c r="E10">
-        <v>38</v>
-      </c>
-      <c r="F10">
-        <v>46</v>
-      </c>
-      <c r="G10">
-        <v>49</v>
-      </c>
-      <c r="H10">
-        <v>21</v>
-      </c>
-      <c r="I10">
-        <v>22</v>
-      </c>
-      <c r="J10">
-        <v>17</v>
-      </c>
-      <c r="K10">
-        <v>19</v>
-      </c>
       <c r="L10">
-        <v>133</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -2744,19 +2744,19 @@
         <v>1</v>
       </c>
       <c r="C11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>3</v>
+      </c>
+      <c r="F11">
         <v>4</v>
       </c>
-      <c r="E11">
+      <c r="G11">
         <v>4</v>
-      </c>
-      <c r="F11">
-        <v>5</v>
-      </c>
-      <c r="G11">
-        <v>5</v>
       </c>
       <c r="H11">
         <v>2</v>
@@ -2765,13 +2765,13 @@
         <v>2</v>
       </c>
       <c r="J11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L11">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -2779,22 +2779,22 @@
         <v>62</v>
       </c>
       <c r="B12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C12">
         <v>3</v>
       </c>
       <c r="D12">
+        <v>5</v>
+      </c>
+      <c r="E12">
+        <v>5</v>
+      </c>
+      <c r="F12">
         <v>7</v>
       </c>
-      <c r="E12">
-        <v>8</v>
-      </c>
-      <c r="F12">
-        <v>9</v>
-      </c>
       <c r="G12">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H12">
         <v>4</v>
@@ -2803,13 +2803,13 @@
         <v>4</v>
       </c>
       <c r="J12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L12">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -2817,34 +2817,34 @@
         <v>35</v>
       </c>
       <c r="B13" s="3">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="C13" s="3">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D13" s="3">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="E13" s="3">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="F13" s="3">
-        <v>275</v>
+        <v>258</v>
       </c>
       <c r="G13" s="3">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="H13" s="3">
-        <v>124</v>
+        <v>144</v>
       </c>
       <c r="I13" s="3">
-        <v>132</v>
+        <v>162</v>
       </c>
       <c r="J13" s="3">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="K13" s="3">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="L13" s="3">
         <v>802</v>

</xml_diff>

<commit_message>
Raise main fabric use to 90%, add S/XL to small batches, add LA VELA sheet
Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SHORT_PLAYA_CAB_Cantidades_Sugeridas_Proyecciones.xlsx
+++ b/SHORT_PLAYA_CAB_Cantidades_Sugeridas_Proyecciones.xlsx
@@ -10,26 +10,27 @@
     <sheet name="Cantidades por Colores" sheetId="1" r:id="rId1"/>
     <sheet name="Producción por Talla" sheetId="2" r:id="rId2"/>
     <sheet name="Producción Color × Talla" sheetId="3" r:id="rId3"/>
-    <sheet name="Distribución por Tienda" sheetId="4" r:id="rId4"/>
-    <sheet name="Uso de Tela Short Playa" sheetId="5" r:id="rId5"/>
+    <sheet name="Producción LA VELA" sheetId="4" r:id="rId4"/>
+    <sheet name="Distribución por Tienda" sheetId="5" r:id="rId5"/>
+    <sheet name="Uso de Tela Short Playa" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="113">
   <si>
     <t>CANTIDADES POR COLORES</t>
   </si>
   <si>
-    <t>SHORT PLAYA CAB · S12 M25 L32 XL18 2XL13 · LA VELA 350 und · Habano/Azul Verdoso/Azul Pizzarra 70% tela · ≤50 und → M/L/XL</t>
-  </si>
-  <si>
-    <t>Rango producción: 802 – 856 und</t>
-  </si>
-  <si>
-    <t>MÍNIMO — 802 und</t>
+    <t>SHORT PLAYA CAB · S12 M25 L32 XL18 2XL13 · LA VELA 350 und · Habano/Azul Verdoso/Azul Pizzarra 90% tela · ≤50 und → S10 M24 L30 XL16 2XL20</t>
+  </si>
+  <si>
+    <t>Rango producción: 941 – 1002 und</t>
+  </si>
+  <si>
+    <t>MÍNIMO — 941 und</t>
   </si>
   <si>
     <t>SHORT PLAYA CAB</t>
@@ -53,13 +54,13 @@
     <t>Tot</t>
   </si>
   <si>
-    <t>Marron · tela Habano (70%)</t>
-  </si>
-  <si>
-    <t>Azul Verdoso · tela Azul Verdoso (70%)</t>
-  </si>
-  <si>
-    <t>Azul Pizarra · tela Azul Pizzarra (70%)</t>
+    <t>Marron · tela Habano (90%)</t>
+  </si>
+  <si>
+    <t>Azul Verdoso · tela Azul Verdoso (90%)</t>
+  </si>
+  <si>
+    <t>Azul Pizarra · tela Azul Pizzarra (90%)</t>
   </si>
   <si>
     <t>Verde Pino · tela Verde Pino</t>
@@ -68,22 +69,22 @@
     <t>Cereza · tela Rojo</t>
   </si>
   <si>
-    <t>Verde Oliva · tela Verde Oliva · M/L/XL</t>
-  </si>
-  <si>
-    <t>Gris Azulado · tela Gris Azulado · M/L/XL</t>
-  </si>
-  <si>
-    <t>Azul Marino · tela Azul Marino · M/L/XL</t>
-  </si>
-  <si>
-    <t>Aguamarina · tela Aguamarina · M/L/XL</t>
+    <t>Verde Oliva · tela Verde Oliva · lote chico</t>
+  </si>
+  <si>
+    <t>Gris Azulado · tela Gris Azulado · lote chico</t>
+  </si>
+  <si>
+    <t>Azul Marino · tela Azul Marino · lote chico</t>
+  </si>
+  <si>
+    <t>Aguamarina · tela Aguamarina · lote chico</t>
   </si>
   <si>
     <t>TOTAL GENERAL</t>
   </si>
   <si>
-    <t>MÁXIMO — 856 und (tope)</t>
+    <t>MÁXIMO — 1002 und (tope)</t>
   </si>
   <si>
     <t>Marron · tela Habano</t>
@@ -131,10 +132,10 @@
     <t>SHORT PLAYA CAB — PRODUCCIÓN POR COLOR Y TALLA</t>
   </si>
   <si>
-    <t>Rango global: 802 – 856 und · Rotación últimos 6 meses × 1.25</t>
-  </si>
-  <si>
-    <t>Short Playa · Marron [PRODUCCIÓN · Tela Habano (140.58 m usados = 70% de 200.83 m)]</t>
+    <t>Rango global: 941 – 1002 und · Rotación últimos 6 meses × 1.25</t>
+  </si>
+  <si>
+    <t>Short Playa · Marron [PRODUCCIÓN · Tela Habano (180.75 m usados = 90% de 200.83 m)]</t>
   </si>
   <si>
     <t>Mín</t>
@@ -155,10 +156,10 @@
     <t>TOTAL color</t>
   </si>
   <si>
-    <t>Short Playa · Azul Verdoso [PRODUCCIÓN · Tela Azul Verdoso (114.76 m usados = 70% de 163.94 m)]</t>
-  </si>
-  <si>
-    <t>Short Playa · Azul Pizarra [PRODUCCIÓN · Tela Azul Pizzarra (114.31 m usados = 70% de 163.30 m)]</t>
+    <t>Short Playa · Azul Verdoso [PRODUCCIÓN · Tela Azul Verdoso (147.55 m usados = 90% de 163.94 m)]</t>
+  </si>
+  <si>
+    <t>Short Playa · Azul Pizarra [PRODUCCIÓN · Tela Azul Pizzarra (146.97 m usados = 90% de 163.30 m)]</t>
   </si>
   <si>
     <t>Short Playa · Verde Pino [PRODUCCIÓN · Tela Verde Pino (76.33 m usados)]</t>
@@ -167,16 +168,82 @@
     <t>Short Playa · Cereza [PRODUCCIÓN · Tela Rojo (65.00 m usados)]</t>
   </si>
   <si>
-    <t>Short Playa · Verde Oliva [PRODUCCIÓN · Tela Verde Oliva (29.13 m usados) · solo M/L/XL]</t>
-  </si>
-  <si>
-    <t>Short Playa · Gris Azulado [PRODUCCIÓN · Tela Gris Azulado (28.67 m usados) · solo M/L/XL]</t>
-  </si>
-  <si>
-    <t>Short Playa · Azul Marino [PRODUCCIÓN · Tela Azul Marino (24.25 m usados) · solo M/L/XL]</t>
-  </si>
-  <si>
-    <t>Short Playa · Aguamarina [PRODUCCIÓN · Tela Aguamarina (11.50 m usados) · solo M/L/XL]</t>
+    <t>Short Playa · Verde Oliva [PRODUCCIÓN · Tela Verde Oliva (29.13 m usados) · curva lote chico S10 M24 L30 XL16 2XL20]</t>
+  </si>
+  <si>
+    <t>Short Playa · Gris Azulado [PRODUCCIÓN · Tela Gris Azulado (28.67 m usados) · curva lote chico S10 M24 L30 XL16 2XL20]</t>
+  </si>
+  <si>
+    <t>Short Playa · Azul Marino [PRODUCCIÓN · Tela Azul Marino (24.25 m usados) · curva lote chico S10 M24 L30 XL16 2XL20]</t>
+  </si>
+  <si>
+    <t>Short Playa · Aguamarina [PRODUCCIÓN · Tela Aguamarina (11.50 m usados) · curva lote chico S10 M24 L30 XL16 2XL20]</t>
+  </si>
+  <si>
+    <t>SHORT PLAYA CAB — PRODUCCIÓN LA VELA ★ (350 und)</t>
+  </si>
+  <si>
+    <t>Desglose color × talla para playa · prioridad por rotación y stock crítico VELA</t>
+  </si>
+  <si>
+    <t>Color</t>
+  </si>
+  <si>
+    <t>Tela</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Azul Pizarra</t>
+  </si>
+  <si>
+    <t>Azul Pizzarra</t>
+  </si>
+  <si>
+    <t>Azul Verdoso</t>
+  </si>
+  <si>
+    <t>Cereza</t>
+  </si>
+  <si>
+    <t>Rojo</t>
+  </si>
+  <si>
+    <t>Marron</t>
+  </si>
+  <si>
+    <t>Habano</t>
+  </si>
+  <si>
+    <t>Verde Pino</t>
+  </si>
+  <si>
+    <t>Azul Marino</t>
+  </si>
+  <si>
+    <t>Gris Azulado</t>
+  </si>
+  <si>
+    <t>Verde Oliva</t>
+  </si>
+  <si>
+    <t>Aguamarina</t>
+  </si>
+  <si>
+    <t>TOTAL VELA</t>
+  </si>
+  <si>
+    <t>Detalle línea a línea:</t>
+  </si>
+  <si>
+    <t>Und</t>
+  </si>
+  <si>
+    <t>Nota</t>
+  </si>
+  <si>
+    <t>lote chico</t>
   </si>
   <si>
     <t>SHORT PLAYA CAB — DISTRIBUCIÓN POR TIENDA Y TALLA</t>
@@ -212,10 +279,7 @@
     <t>SHORT PLAYA CAB — TELA EXISTENTE A AGOTAR (100%)</t>
   </si>
   <si>
-    <t>Consumo: 0.75 m/pieza · Habano/Azul Verdoso/Azul Pizzarra al 70% · ≤50 und → M/L/XL</t>
-  </si>
-  <si>
-    <t>Tela</t>
+    <t>Consumo: 0.75 m/pieza · Habano/Azul Verdoso/Azul Pizzarra al 90% · ≤50 und → S10 M24 L30 XL16 2XL20</t>
   </si>
   <si>
     <t>Producto</t>
@@ -245,91 +309,55 @@
     <t>Notas</t>
   </si>
   <si>
-    <t>Habano</t>
-  </si>
-  <si>
     <t>Short Playa · Marron</t>
   </si>
   <si>
-    <t>70%</t>
+    <t>90%</t>
   </si>
   <si>
     <t>Curva global ventas · Tela HABANO</t>
   </si>
   <si>
-    <t>Azul Verdoso</t>
-  </si>
-  <si>
     <t>Short Playa · Azul Verdoso</t>
   </si>
   <si>
     <t>Curva global ventas</t>
   </si>
   <si>
-    <t>Azul Pizzarra</t>
-  </si>
-  <si>
     <t>Short Playa · Azul Pizarra</t>
   </si>
   <si>
     <t>Curva global ventas · Tela AZUL PIZZARRA</t>
   </si>
   <si>
-    <t>Verde Pino</t>
-  </si>
-  <si>
     <t>Short Playa · Verde Pino</t>
   </si>
   <si>
     <t>100%</t>
   </si>
   <si>
-    <t>Rojo</t>
-  </si>
-  <si>
     <t>Short Playa · Cereza</t>
   </si>
   <si>
     <t>Curva global ventas · Tela ROJO</t>
   </si>
   <si>
-    <t>Verde Oliva</t>
-  </si>
-  <si>
     <t>Short Playa · Verde Oliva</t>
   </si>
   <si>
-    <t>Curva global ventas · Tela escasa → M/L/XL</t>
-  </si>
-  <si>
-    <t>Gris Azulado</t>
+    <t>Curva global ventas · Lote chico → todas las tallas</t>
   </si>
   <si>
     <t>Short Playa · Gris Azulado</t>
   </si>
   <si>
-    <t>Azul Marino</t>
-  </si>
-  <si>
     <t>Short Playa · Azul Marino</t>
   </si>
   <si>
-    <t>Aguamarina</t>
-  </si>
-  <si>
     <t>Short Playa · Aguamarina</t>
   </si>
   <si>
     <t>Resumen tela stock vs usada:</t>
-  </si>
-  <si>
-    <t>Marron</t>
-  </si>
-  <si>
-    <t>Azul Pizarra</t>
-  </si>
-  <si>
-    <t>Cereza</t>
   </si>
 </sst>
 </file>
@@ -754,22 +782,22 @@
         <v>11</v>
       </c>
       <c r="B7">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C7">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="D7">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="E7">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="F7">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="G7">
-        <v>187</v>
+        <v>240</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -777,22 +805,22 @@
         <v>12</v>
       </c>
       <c r="B8">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C8">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="D8">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="E8">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="F8">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="G8">
-        <v>153</v>
+        <v>196</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -800,22 +828,22 @@
         <v>13</v>
       </c>
       <c r="B9">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C9">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="D9">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="E9">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="F9">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="G9">
-        <v>152</v>
+        <v>195</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -869,19 +897,19 @@
         <v>16</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C12">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D12">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E12">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G12">
         <v>38</v>
@@ -892,19 +920,19 @@
         <v>17</v>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C13">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D13">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E13">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G13">
         <v>38</v>
@@ -915,19 +943,19 @@
         <v>18</v>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C14">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D14">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E14">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G14">
         <v>32</v>
@@ -938,19 +966,19 @@
         <v>19</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C15">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D15">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G15">
         <v>15</v>
@@ -961,22 +989,22 @@
         <v>20</v>
       </c>
       <c r="B16" s="3">
-        <v>80</v>
+        <v>112</v>
       </c>
       <c r="C16" s="3">
-        <v>212</v>
+        <v>235</v>
       </c>
       <c r="D16" s="3">
-        <v>270</v>
+        <v>299</v>
       </c>
       <c r="E16" s="3">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="F16" s="3">
-        <v>88</v>
+        <v>130</v>
       </c>
       <c r="G16" s="3">
-        <v>802</v>
+        <v>941</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -1012,22 +1040,22 @@
         <v>22</v>
       </c>
       <c r="B20">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="C20">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="D20">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="E20">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="F20">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="G20">
-        <v>199</v>
+        <v>255</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -1035,22 +1063,22 @@
         <v>23</v>
       </c>
       <c r="B21">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C21">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="D21">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="E21">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="F21">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="G21">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -1058,22 +1086,22 @@
         <v>24</v>
       </c>
       <c r="B22">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C22">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="D22">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="E22">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="F22">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="G22">
-        <v>162</v>
+        <v>207</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -1127,19 +1155,19 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C25">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D25">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E25">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F25">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G25">
         <v>41</v>
@@ -1150,19 +1178,19 @@
         <v>26</v>
       </c>
       <c r="B26">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C26">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D26">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E26">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F26">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G26">
         <v>41</v>
@@ -1173,19 +1201,19 @@
         <v>27</v>
       </c>
       <c r="B27">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C27">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D27">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E27">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G27">
         <v>34</v>
@@ -1196,19 +1224,19 @@
         <v>28</v>
       </c>
       <c r="B28">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C28">
+        <v>4</v>
+      </c>
+      <c r="D28">
         <v>5</v>
       </c>
-      <c r="D28">
-        <v>7</v>
-      </c>
       <c r="E28">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F28">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G28">
         <v>16</v>
@@ -1219,22 +1247,22 @@
         <v>20</v>
       </c>
       <c r="B29" s="3">
-        <v>87</v>
+        <v>117</v>
       </c>
       <c r="C29" s="3">
-        <v>226</v>
+        <v>250</v>
       </c>
       <c r="D29" s="3">
-        <v>287</v>
+        <v>318</v>
       </c>
       <c r="E29" s="3">
-        <v>162</v>
+        <v>178</v>
       </c>
       <c r="F29" s="3">
-        <v>94</v>
+        <v>139</v>
       </c>
       <c r="G29" s="3">
-        <v>856</v>
+        <v>1002</v>
       </c>
     </row>
   </sheetData>
@@ -1279,10 +1307,10 @@
         <v>0.12</v>
       </c>
       <c r="C5">
-        <v>80</v>
+        <v>112</v>
       </c>
       <c r="D5">
-        <v>87</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1293,10 +1321,10 @@
         <v>0.25</v>
       </c>
       <c r="C6">
-        <v>212</v>
+        <v>235</v>
       </c>
       <c r="D6">
-        <v>226</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1307,10 +1335,10 @@
         <v>0.32</v>
       </c>
       <c r="C7">
-        <v>270</v>
+        <v>299</v>
       </c>
       <c r="D7">
-        <v>287</v>
+        <v>318</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1321,10 +1349,10 @@
         <v>0.18</v>
       </c>
       <c r="C8">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="D8">
-        <v>162</v>
+        <v>178</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1335,10 +1363,10 @@
         <v>0.13</v>
       </c>
       <c r="C9">
-        <v>88</v>
+        <v>130</v>
       </c>
       <c r="D9">
-        <v>94</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -1347,10 +1375,10 @@
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3">
-        <v>802</v>
+        <v>941</v>
       </c>
       <c r="D10" s="3">
-        <v>856</v>
+        <v>1002</v>
       </c>
     </row>
   </sheetData>
@@ -1360,7 +1388,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F83"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1403,10 +1431,10 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C6">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D6">
         <v>3.1</v>
@@ -1423,10 +1451,10 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="C7">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="D7">
         <v>5.8</v>
@@ -1443,10 +1471,10 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="C8">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="D8">
         <v>7.3</v>
@@ -1463,10 +1491,10 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="C9">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D9">
         <v>3.5</v>
@@ -1483,10 +1511,10 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C10">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="D10">
         <v>3.8</v>
@@ -1503,10 +1531,10 @@
         <v>44</v>
       </c>
       <c r="B11" s="3">
-        <v>187</v>
+        <v>240</v>
       </c>
       <c r="C11" s="3">
-        <v>199</v>
+        <v>255</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
@@ -1542,10 +1570,10 @@
         <v>5</v>
       </c>
       <c r="B15">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C15">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D15">
         <v>2.1</v>
@@ -1562,10 +1590,10 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="C16">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="D16">
         <v>4</v>
@@ -1582,10 +1610,10 @@
         <v>7</v>
       </c>
       <c r="B17">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="C17">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="D17">
         <v>7.7</v>
@@ -1602,10 +1630,10 @@
         <v>8</v>
       </c>
       <c r="B18">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C18">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="D18">
         <v>4.6</v>
@@ -1622,10 +1650,10 @@
         <v>9</v>
       </c>
       <c r="B19">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C19">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D19">
         <v>4</v>
@@ -1642,10 +1670,10 @@
         <v>44</v>
       </c>
       <c r="B20" s="3">
-        <v>153</v>
+        <v>196</v>
       </c>
       <c r="C20" s="3">
-        <v>163</v>
+        <v>208</v>
       </c>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
@@ -1681,10 +1709,10 @@
         <v>5</v>
       </c>
       <c r="B24">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C24">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="D24">
         <v>4.2</v>
@@ -1701,10 +1729,10 @@
         <v>6</v>
       </c>
       <c r="B25">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="C25">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="D25">
         <v>4.8</v>
@@ -1721,10 +1749,10 @@
         <v>7</v>
       </c>
       <c r="B26">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="C26">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="D26">
         <v>7.3</v>
@@ -1741,10 +1769,10 @@
         <v>8</v>
       </c>
       <c r="B27">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="C27">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="D27">
         <v>5.4</v>
@@ -1761,10 +1789,10 @@
         <v>9</v>
       </c>
       <c r="B28">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C28">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D28">
         <v>5.2</v>
@@ -1781,10 +1809,10 @@
         <v>44</v>
       </c>
       <c r="B29" s="3">
-        <v>152</v>
+        <v>195</v>
       </c>
       <c r="C29" s="3">
-        <v>162</v>
+        <v>207</v>
       </c>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
@@ -2095,13 +2123,13 @@
     </row>
     <row r="51" spans="1:6">
       <c r="A51" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B51">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="C51">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="D51">
         <v>0</v>
@@ -2115,13 +2143,13 @@
     </row>
     <row r="52" spans="1:6">
       <c r="A52" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B52">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C52">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="D52">
         <v>0</v>
@@ -2135,112 +2163,112 @@
     </row>
     <row r="53" spans="1:6">
       <c r="A53" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B53">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C53">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D53">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="E53">
         <v>0</v>
       </c>
       <c r="F53">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54" t="s">
+        <v>8</v>
+      </c>
+      <c r="B54">
+        <v>6</v>
+      </c>
+      <c r="C54">
+        <v>7</v>
+      </c>
+      <c r="D54">
+        <v>0.2</v>
+      </c>
+      <c r="E54">
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:6">
-      <c r="A54" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B54" s="3">
-        <v>38</v>
-      </c>
-      <c r="C54" s="3">
-        <v>41</v>
-      </c>
-      <c r="D54" s="3"/>
-      <c r="E54" s="3"/>
-      <c r="F54" s="3"/>
+      <c r="F54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55" t="s">
+        <v>9</v>
+      </c>
+      <c r="B55">
+        <v>8</v>
+      </c>
+      <c r="C55">
+        <v>8</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55">
+        <v>0</v>
+      </c>
+      <c r="F55">
+        <v>99</v>
+      </c>
     </row>
     <row r="56" spans="1:6">
       <c r="A56" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B56" s="3">
+        <v>38</v>
+      </c>
+      <c r="C56" s="3">
+        <v>41</v>
+      </c>
+      <c r="D56" s="3"/>
+      <c r="E56" s="3"/>
+      <c r="F56" s="3"/>
+    </row>
+    <row r="58" spans="1:6">
+      <c r="A58" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="57" spans="1:6">
-      <c r="A57" s="4" t="s">
+    <row r="59" spans="1:6">
+      <c r="A59" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B57" s="4" t="s">
+      <c r="B59" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C57" s="4" t="s">
+      <c r="C59" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D57" s="4" t="s">
+      <c r="D59" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="E57" s="4" t="s">
+      <c r="E59" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="F57" s="4" t="s">
+      <c r="F59" s="4" t="s">
         <v>43</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6">
-      <c r="A58" t="s">
-        <v>6</v>
-      </c>
-      <c r="B58">
-        <v>13</v>
-      </c>
-      <c r="C58">
-        <v>14</v>
-      </c>
-      <c r="D58">
-        <v>0.6</v>
-      </c>
-      <c r="E58">
-        <v>0</v>
-      </c>
-      <c r="F58">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6">
-      <c r="A59" t="s">
-        <v>7</v>
-      </c>
-      <c r="B59">
-        <v>16</v>
-      </c>
-      <c r="C59">
-        <v>17</v>
-      </c>
-      <c r="D59">
-        <v>0</v>
-      </c>
-      <c r="E59">
-        <v>0</v>
-      </c>
-      <c r="F59">
-        <v>99</v>
       </c>
     </row>
     <row r="60" spans="1:6">
       <c r="A60" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B60">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C60">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D60">
         <v>0</v>
@@ -2253,166 +2281,207 @@
       </c>
     </row>
     <row r="61" spans="1:6">
-      <c r="A61" s="3" t="s">
+      <c r="A61" t="s">
+        <v>6</v>
+      </c>
+      <c r="B61">
+        <v>9</v>
+      </c>
+      <c r="C61">
+        <v>10</v>
+      </c>
+      <c r="D61">
+        <v>0.6</v>
+      </c>
+      <c r="E61">
+        <v>0</v>
+      </c>
+      <c r="F61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
+      <c r="A62" t="s">
+        <v>7</v>
+      </c>
+      <c r="B62">
+        <v>11</v>
+      </c>
+      <c r="C62">
+        <v>12</v>
+      </c>
+      <c r="D62">
+        <v>0</v>
+      </c>
+      <c r="E62">
+        <v>0</v>
+      </c>
+      <c r="F62">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="A63" t="s">
+        <v>8</v>
+      </c>
+      <c r="B63">
+        <v>6</v>
+      </c>
+      <c r="C63">
+        <v>7</v>
+      </c>
+      <c r="D63">
+        <v>0</v>
+      </c>
+      <c r="E63">
+        <v>0</v>
+      </c>
+      <c r="F63">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
+      <c r="A64" t="s">
+        <v>9</v>
+      </c>
+      <c r="B64">
+        <v>8</v>
+      </c>
+      <c r="C64">
+        <v>8</v>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+      <c r="E64">
+        <v>0</v>
+      </c>
+      <c r="F64">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
+      <c r="A65" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B61" s="3">
+      <c r="B65" s="3">
         <v>38</v>
       </c>
-      <c r="C61" s="3">
+      <c r="C65" s="3">
         <v>41</v>
       </c>
-      <c r="D61" s="3"/>
-      <c r="E61" s="3"/>
-      <c r="F61" s="3"/>
-    </row>
-    <row r="63" spans="1:6">
-      <c r="A63" s="3" t="s">
+      <c r="D65" s="3"/>
+      <c r="E65" s="3"/>
+      <c r="F65" s="3"/>
+    </row>
+    <row r="67" spans="1:6">
+      <c r="A67" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="64" spans="1:6">
-      <c r="A64" s="4" t="s">
+    <row r="68" spans="1:6">
+      <c r="A68" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B64" s="4" t="s">
+      <c r="B68" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C64" s="4" t="s">
+      <c r="C68" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D64" s="4" t="s">
+      <c r="D68" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="E64" s="4" t="s">
+      <c r="E68" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="F64" s="4" t="s">
+      <c r="F68" s="4" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="65" spans="1:6">
-      <c r="A65" t="s">
+    <row r="69" spans="1:6">
+      <c r="A69" t="s">
+        <v>5</v>
+      </c>
+      <c r="B69">
+        <v>3</v>
+      </c>
+      <c r="C69">
+        <v>3</v>
+      </c>
+      <c r="D69">
+        <v>0</v>
+      </c>
+      <c r="E69">
+        <v>0</v>
+      </c>
+      <c r="F69">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6">
+      <c r="A70" t="s">
         <v>6</v>
       </c>
-      <c r="B65">
-        <v>11</v>
-      </c>
-      <c r="C65">
-        <v>11</v>
-      </c>
-      <c r="D65">
+      <c r="B70">
+        <v>8</v>
+      </c>
+      <c r="C70">
+        <v>8</v>
+      </c>
+      <c r="D70">
         <v>0.2</v>
       </c>
-      <c r="E65">
+      <c r="E70">
         <v>0</v>
       </c>
-      <c r="F65">
+      <c r="F70">
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:6">
-      <c r="A66" t="s">
+    <row r="71" spans="1:6">
+      <c r="A71" t="s">
         <v>7</v>
       </c>
-      <c r="B66">
-        <v>13</v>
-      </c>
-      <c r="C66">
-        <v>15</v>
-      </c>
-      <c r="D66">
+      <c r="B71">
+        <v>10</v>
+      </c>
+      <c r="C71">
+        <v>10</v>
+      </c>
+      <c r="D71">
         <v>0.6</v>
       </c>
-      <c r="E66">
+      <c r="E71">
         <v>0</v>
       </c>
-      <c r="F66">
+      <c r="F71">
         <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6">
-      <c r="A67" t="s">
-        <v>8</v>
-      </c>
-      <c r="B67">
-        <v>8</v>
-      </c>
-      <c r="C67">
-        <v>8</v>
-      </c>
-      <c r="D67">
-        <v>0.2</v>
-      </c>
-      <c r="E67">
-        <v>0</v>
-      </c>
-      <c r="F67">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6">
-      <c r="A68" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B68" s="3">
-        <v>32</v>
-      </c>
-      <c r="C68" s="3">
-        <v>34</v>
-      </c>
-      <c r="D68" s="3"/>
-      <c r="E68" s="3"/>
-      <c r="F68" s="3"/>
-    </row>
-    <row r="70" spans="1:6">
-      <c r="A70" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6">
-      <c r="A71" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B71" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C71" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D71" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E71" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="F71" s="4" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="72" spans="1:6">
       <c r="A72" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B72">
         <v>5</v>
       </c>
       <c r="C72">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D72">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="E72">
         <v>0</v>
       </c>
       <c r="F72">
-        <v>99</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73" spans="1:6">
       <c r="A73" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B73">
         <v>6</v>
@@ -2421,48 +2490,167 @@
         <v>7</v>
       </c>
       <c r="D73">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="E73">
         <v>0</v>
       </c>
       <c r="F73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6">
+      <c r="A74" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B74" s="3">
+        <v>32</v>
+      </c>
+      <c r="C74" s="3">
+        <v>34</v>
+      </c>
+      <c r="D74" s="3"/>
+      <c r="E74" s="3"/>
+      <c r="F74" s="3"/>
+    </row>
+    <row r="76" spans="1:6">
+      <c r="A76" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6">
+      <c r="A77" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D77" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E77" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F77" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6">
+      <c r="A78" t="s">
+        <v>5</v>
+      </c>
+      <c r="B78">
+        <v>2</v>
+      </c>
+      <c r="C78">
+        <v>2</v>
+      </c>
+      <c r="D78">
+        <v>0</v>
+      </c>
+      <c r="E78">
+        <v>0</v>
+      </c>
+      <c r="F78">
         <v>99</v>
       </c>
     </row>
-    <row r="74" spans="1:6">
-      <c r="A74" t="s">
+    <row r="79" spans="1:6">
+      <c r="A79" t="s">
+        <v>6</v>
+      </c>
+      <c r="B79">
+        <v>4</v>
+      </c>
+      <c r="C79">
+        <v>4</v>
+      </c>
+      <c r="D79">
+        <v>0</v>
+      </c>
+      <c r="E79">
+        <v>0</v>
+      </c>
+      <c r="F79">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6">
+      <c r="A80" t="s">
+        <v>7</v>
+      </c>
+      <c r="B80">
+        <v>4</v>
+      </c>
+      <c r="C80">
+        <v>5</v>
+      </c>
+      <c r="D80">
+        <v>0</v>
+      </c>
+      <c r="E80">
+        <v>0</v>
+      </c>
+      <c r="F80">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6">
+      <c r="A81" t="s">
         <v>8</v>
       </c>
-      <c r="B74">
-        <v>4</v>
-      </c>
-      <c r="C74">
-        <v>4</v>
-      </c>
-      <c r="D74">
+      <c r="B81">
+        <v>2</v>
+      </c>
+      <c r="C81">
+        <v>2</v>
+      </c>
+      <c r="D81">
         <v>0</v>
       </c>
-      <c r="E74">
+      <c r="E81">
         <v>0</v>
       </c>
-      <c r="F74">
+      <c r="F81">
         <v>99</v>
       </c>
     </row>
-    <row r="75" spans="1:6">
-      <c r="A75" s="3" t="s">
+    <row r="82" spans="1:6">
+      <c r="A82" t="s">
+        <v>9</v>
+      </c>
+      <c r="B82">
+        <v>3</v>
+      </c>
+      <c r="C82">
+        <v>3</v>
+      </c>
+      <c r="D82">
+        <v>0</v>
+      </c>
+      <c r="E82">
+        <v>0</v>
+      </c>
+      <c r="F82">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6">
+      <c r="A83" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B75" s="3">
+      <c r="B83" s="3">
         <v>15</v>
       </c>
-      <c r="C75" s="3">
+      <c r="C83" s="3">
         <v>16</v>
       </c>
-      <c r="D75" s="3"/>
-      <c r="E75" s="3"/>
-      <c r="F75" s="3"/>
+      <c r="D83" s="3"/>
+      <c r="E83" s="3"/>
+      <c r="F83" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2471,286 +2659,216 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:8">
       <c r="A2" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:8">
       <c r="A4" s="4" t="s">
         <v>55</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="4"/>
       <c r="D4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="4"/>
+      <c r="E4" s="4" t="s">
+        <v>7</v>
+      </c>
       <c r="F4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5">
         <v>7</v>
       </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4" t="s">
+      <c r="D5">
+        <v>14</v>
+      </c>
+      <c r="E5">
+        <v>18</v>
+      </c>
+      <c r="F5">
+        <v>10</v>
+      </c>
+      <c r="G5">
         <v>8</v>
       </c>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4" t="s">
+      <c r="H5">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6">
+        <v>7</v>
+      </c>
+      <c r="D6">
+        <v>14</v>
+      </c>
+      <c r="E6">
+        <v>18</v>
+      </c>
+      <c r="F6">
+        <v>10</v>
+      </c>
+      <c r="G6">
+        <v>7</v>
+      </c>
+      <c r="H6">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7">
+        <v>6</v>
+      </c>
+      <c r="D7">
+        <v>14</v>
+      </c>
+      <c r="E7">
+        <v>18</v>
+      </c>
+      <c r="F7">
+        <v>10</v>
+      </c>
+      <c r="G7">
+        <v>7</v>
+      </c>
+      <c r="H7">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8">
+        <v>6</v>
+      </c>
+      <c r="D8">
+        <v>13</v>
+      </c>
+      <c r="E8">
+        <v>17</v>
+      </c>
+      <c r="F8">
+        <v>10</v>
+      </c>
+      <c r="G8">
+        <v>7</v>
+      </c>
+      <c r="H8">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9">
+        <v>6</v>
+      </c>
+      <c r="D9">
+        <v>13</v>
+      </c>
+      <c r="E9">
+        <v>17</v>
+      </c>
+      <c r="F9">
         <v>9</v>
       </c>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="L5" s="4"/>
-    </row>
-    <row r="6" spans="1:12">
-      <c r="A6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B6">
-        <v>13</v>
-      </c>
-      <c r="C6">
-        <v>14</v>
-      </c>
-      <c r="D6">
-        <v>27</v>
-      </c>
-      <c r="E6">
+      <c r="G9">
+        <v>7</v>
+      </c>
+      <c r="H9">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10">
+        <v>7</v>
+      </c>
+      <c r="E10">
+        <v>9</v>
+      </c>
+      <c r="F10">
+        <v>5</v>
+      </c>
+      <c r="G10">
+        <v>6</v>
+      </c>
+      <c r="H10">
         <v>30</v>
       </c>
-      <c r="F6">
-        <v>35</v>
-      </c>
-      <c r="G6">
-        <v>38</v>
-      </c>
-      <c r="H6">
-        <v>20</v>
-      </c>
-      <c r="I6">
-        <v>21</v>
-      </c>
-      <c r="J6">
-        <v>14</v>
-      </c>
-      <c r="K6">
-        <v>15</v>
-      </c>
-      <c r="L6">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
-      <c r="A7" t="s">
-        <v>57</v>
-      </c>
-      <c r="B7">
-        <v>42</v>
-      </c>
-      <c r="C7">
-        <v>44</v>
-      </c>
-      <c r="D7">
-        <v>88</v>
-      </c>
-      <c r="E7">
-        <v>93</v>
-      </c>
-      <c r="F7">
-        <v>112</v>
-      </c>
-      <c r="G7">
-        <v>119</v>
-      </c>
-      <c r="H7">
-        <v>63</v>
-      </c>
-      <c r="I7">
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" t="s">
         <v>67</v>
       </c>
-      <c r="J7">
-        <v>45</v>
-      </c>
-      <c r="K7">
-        <v>48</v>
-      </c>
-      <c r="L7">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
-      <c r="A8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B8">
-        <v>13</v>
-      </c>
-      <c r="C8">
-        <v>14</v>
-      </c>
-      <c r="D8">
-        <v>27</v>
-      </c>
-      <c r="E8">
-        <v>29</v>
-      </c>
-      <c r="F8">
-        <v>34</v>
-      </c>
-      <c r="G8">
-        <v>37</v>
-      </c>
-      <c r="H8">
-        <v>19</v>
-      </c>
-      <c r="I8">
-        <v>20</v>
-      </c>
-      <c r="J8">
-        <v>14</v>
-      </c>
-      <c r="K8">
-        <v>15</v>
-      </c>
-      <c r="L8">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
-      <c r="A9" t="s">
-        <v>59</v>
-      </c>
-      <c r="B9">
-        <v>12</v>
-      </c>
-      <c r="C9">
-        <v>13</v>
-      </c>
-      <c r="D9">
-        <v>26</v>
-      </c>
-      <c r="E9">
-        <v>27</v>
-      </c>
-      <c r="F9">
-        <v>33</v>
-      </c>
-      <c r="G9">
-        <v>35</v>
-      </c>
-      <c r="H9">
-        <v>18</v>
-      </c>
-      <c r="I9">
-        <v>20</v>
-      </c>
-      <c r="J9">
-        <v>13</v>
-      </c>
-      <c r="K9">
-        <v>14</v>
-      </c>
-      <c r="L9">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
-      <c r="A10" t="s">
-        <v>60</v>
-      </c>
-      <c r="B10">
-        <v>12</v>
-      </c>
-      <c r="C10">
-        <v>13</v>
-      </c>
-      <c r="D10">
-        <v>26</v>
-      </c>
-      <c r="E10">
-        <v>28</v>
-      </c>
-      <c r="F10">
-        <v>33</v>
-      </c>
-      <c r="G10">
-        <v>35</v>
-      </c>
-      <c r="H10">
-        <v>18</v>
-      </c>
-      <c r="I10">
-        <v>20</v>
-      </c>
-      <c r="J10">
-        <v>13</v>
-      </c>
-      <c r="K10">
-        <v>14</v>
-      </c>
-      <c r="L10">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12">
-      <c r="A11" t="s">
-        <v>61</v>
-      </c>
-      <c r="B11">
-        <v>1</v>
+      <c r="B11" t="s">
+        <v>67</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E11">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F11">
         <v>4</v>
@@ -2759,95 +2877,795 @@
         <v>4</v>
       </c>
       <c r="H11">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B12" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12">
         <v>2</v>
       </c>
-      <c r="I11">
+      <c r="D12">
+        <v>4</v>
+      </c>
+      <c r="E12">
+        <v>4</v>
+      </c>
+      <c r="F12">
         <v>2</v>
       </c>
-      <c r="J11">
+      <c r="G12">
+        <v>3</v>
+      </c>
+      <c r="H12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13">
         <v>1</v>
       </c>
-      <c r="K11">
+      <c r="D13">
+        <v>3</v>
+      </c>
+      <c r="E13">
+        <v>3</v>
+      </c>
+      <c r="F13">
+        <v>2</v>
+      </c>
+      <c r="G13">
+        <v>2</v>
+      </c>
+      <c r="H13">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3">
+        <v>40</v>
+      </c>
+      <c r="D14" s="3">
+        <v>87</v>
+      </c>
+      <c r="E14" s="3">
+        <v>110</v>
+      </c>
+      <c r="F14" s="3">
+        <v>62</v>
+      </c>
+      <c r="G14" s="3">
+        <v>51</v>
+      </c>
+      <c r="H14" s="3">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" t="s">
+        <v>58</v>
+      </c>
+      <c r="B18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" t="s">
+        <v>58</v>
+      </c>
+      <c r="B19" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" t="s">
+        <v>6</v>
+      </c>
+      <c r="D20">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" t="s">
+        <v>58</v>
+      </c>
+      <c r="B21" t="s">
+        <v>59</v>
+      </c>
+      <c r="C21" t="s">
+        <v>5</v>
+      </c>
+      <c r="D21">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" t="s">
+        <v>58</v>
+      </c>
+      <c r="B22" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" t="s">
+        <v>60</v>
+      </c>
+      <c r="B23" t="s">
+        <v>60</v>
+      </c>
+      <c r="C23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" t="s">
+        <v>60</v>
+      </c>
+      <c r="B24" t="s">
+        <v>60</v>
+      </c>
+      <c r="C24" t="s">
+        <v>7</v>
+      </c>
+      <c r="D24">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" t="s">
+        <v>60</v>
+      </c>
+      <c r="B25" t="s">
+        <v>60</v>
+      </c>
+      <c r="C25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" t="s">
+        <v>60</v>
+      </c>
+      <c r="B26" t="s">
+        <v>60</v>
+      </c>
+      <c r="C26" t="s">
+        <v>5</v>
+      </c>
+      <c r="D26">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" t="s">
+        <v>60</v>
+      </c>
+      <c r="B27" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" t="s">
+        <v>61</v>
+      </c>
+      <c r="B28" t="s">
+        <v>62</v>
+      </c>
+      <c r="C28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" t="s">
+        <v>61</v>
+      </c>
+      <c r="B29" t="s">
+        <v>62</v>
+      </c>
+      <c r="C29" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" t="s">
+        <v>61</v>
+      </c>
+      <c r="B30" t="s">
+        <v>62</v>
+      </c>
+      <c r="C30" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" t="s">
+        <v>61</v>
+      </c>
+      <c r="B31" t="s">
+        <v>62</v>
+      </c>
+      <c r="C31" t="s">
+        <v>5</v>
+      </c>
+      <c r="D31">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" t="s">
+        <v>61</v>
+      </c>
+      <c r="B32" t="s">
+        <v>62</v>
+      </c>
+      <c r="C32" t="s">
+        <v>8</v>
+      </c>
+      <c r="D32">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" t="s">
+        <v>63</v>
+      </c>
+      <c r="B33" t="s">
+        <v>64</v>
+      </c>
+      <c r="C33" t="s">
+        <v>9</v>
+      </c>
+      <c r="D33">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" t="s">
+        <v>63</v>
+      </c>
+      <c r="B34" t="s">
+        <v>64</v>
+      </c>
+      <c r="C34" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" t="s">
+        <v>63</v>
+      </c>
+      <c r="B35" t="s">
+        <v>64</v>
+      </c>
+      <c r="C35" t="s">
+        <v>6</v>
+      </c>
+      <c r="D35">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36" t="s">
+        <v>63</v>
+      </c>
+      <c r="B36" t="s">
+        <v>64</v>
+      </c>
+      <c r="C36" t="s">
+        <v>5</v>
+      </c>
+      <c r="D36">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" t="s">
+        <v>63</v>
+      </c>
+      <c r="B37" t="s">
+        <v>64</v>
+      </c>
+      <c r="C37" t="s">
+        <v>8</v>
+      </c>
+      <c r="D37">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38" t="s">
+        <v>65</v>
+      </c>
+      <c r="B38" t="s">
+        <v>65</v>
+      </c>
+      <c r="C38" t="s">
+        <v>9</v>
+      </c>
+      <c r="D38">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
+      <c r="A39" t="s">
+        <v>65</v>
+      </c>
+      <c r="B39" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40" t="s">
+        <v>65</v>
+      </c>
+      <c r="B40" t="s">
+        <v>65</v>
+      </c>
+      <c r="C40" t="s">
+        <v>6</v>
+      </c>
+      <c r="D40">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41" t="s">
+        <v>65</v>
+      </c>
+      <c r="B41" t="s">
+        <v>65</v>
+      </c>
+      <c r="C41" t="s">
+        <v>5</v>
+      </c>
+      <c r="D41">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42" t="s">
+        <v>65</v>
+      </c>
+      <c r="C42" t="s">
+        <v>8</v>
+      </c>
+      <c r="D42">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43" t="s">
+        <v>66</v>
+      </c>
+      <c r="B43" t="s">
+        <v>66</v>
+      </c>
+      <c r="C43" t="s">
+        <v>9</v>
+      </c>
+      <c r="D43">
+        <v>6</v>
+      </c>
+      <c r="E43" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44" t="s">
+        <v>66</v>
+      </c>
+      <c r="B44" t="s">
+        <v>66</v>
+      </c>
+      <c r="C44" t="s">
+        <v>7</v>
+      </c>
+      <c r="D44">
+        <v>9</v>
+      </c>
+      <c r="E44" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45" t="s">
+        <v>66</v>
+      </c>
+      <c r="B45" t="s">
+        <v>66</v>
+      </c>
+      <c r="C45" t="s">
+        <v>6</v>
+      </c>
+      <c r="D45">
+        <v>7</v>
+      </c>
+      <c r="E45" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="A46" t="s">
+        <v>66</v>
+      </c>
+      <c r="B46" t="s">
+        <v>66</v>
+      </c>
+      <c r="C46" t="s">
+        <v>5</v>
+      </c>
+      <c r="D46">
+        <v>3</v>
+      </c>
+      <c r="E46" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
+      <c r="A47" t="s">
+        <v>66</v>
+      </c>
+      <c r="B47" t="s">
+        <v>66</v>
+      </c>
+      <c r="C47" t="s">
+        <v>8</v>
+      </c>
+      <c r="D47">
+        <v>5</v>
+      </c>
+      <c r="E47" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5">
+      <c r="A48" t="s">
+        <v>67</v>
+      </c>
+      <c r="B48" t="s">
+        <v>67</v>
+      </c>
+      <c r="C48" t="s">
+        <v>9</v>
+      </c>
+      <c r="D48">
+        <v>4</v>
+      </c>
+      <c r="E48" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5">
+      <c r="A49" t="s">
+        <v>67</v>
+      </c>
+      <c r="B49" t="s">
+        <v>67</v>
+      </c>
+      <c r="C49" t="s">
+        <v>7</v>
+      </c>
+      <c r="D49">
+        <v>6</v>
+      </c>
+      <c r="E49" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5">
+      <c r="A50" t="s">
+        <v>67</v>
+      </c>
+      <c r="B50" t="s">
+        <v>67</v>
+      </c>
+      <c r="C50" t="s">
+        <v>6</v>
+      </c>
+      <c r="D50">
+        <v>5</v>
+      </c>
+      <c r="E50" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5">
+      <c r="A51" t="s">
+        <v>67</v>
+      </c>
+      <c r="B51" t="s">
+        <v>67</v>
+      </c>
+      <c r="C51" t="s">
+        <v>5</v>
+      </c>
+      <c r="D51">
+        <v>2</v>
+      </c>
+      <c r="E51" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5">
+      <c r="A52" t="s">
+        <v>67</v>
+      </c>
+      <c r="B52" t="s">
+        <v>67</v>
+      </c>
+      <c r="C52" t="s">
+        <v>8</v>
+      </c>
+      <c r="D52">
+        <v>4</v>
+      </c>
+      <c r="E52" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5">
+      <c r="A53" t="s">
+        <v>68</v>
+      </c>
+      <c r="B53" t="s">
+        <v>68</v>
+      </c>
+      <c r="C53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D53">
+        <v>3</v>
+      </c>
+      <c r="E53" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5">
+      <c r="A54" t="s">
+        <v>68</v>
+      </c>
+      <c r="B54" t="s">
+        <v>68</v>
+      </c>
+      <c r="C54" t="s">
+        <v>7</v>
+      </c>
+      <c r="D54">
+        <v>4</v>
+      </c>
+      <c r="E54" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5">
+      <c r="A55" t="s">
+        <v>68</v>
+      </c>
+      <c r="B55" t="s">
+        <v>68</v>
+      </c>
+      <c r="C55" t="s">
+        <v>6</v>
+      </c>
+      <c r="D55">
+        <v>4</v>
+      </c>
+      <c r="E55" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5">
+      <c r="A56" t="s">
+        <v>68</v>
+      </c>
+      <c r="B56" t="s">
+        <v>68</v>
+      </c>
+      <c r="C56" t="s">
+        <v>5</v>
+      </c>
+      <c r="D56">
+        <v>2</v>
+      </c>
+      <c r="E56" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
+      <c r="A57" t="s">
+        <v>68</v>
+      </c>
+      <c r="B57" t="s">
+        <v>68</v>
+      </c>
+      <c r="C57" t="s">
+        <v>8</v>
+      </c>
+      <c r="D57">
+        <v>2</v>
+      </c>
+      <c r="E57" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
+      <c r="A58" t="s">
+        <v>69</v>
+      </c>
+      <c r="B58" t="s">
+        <v>69</v>
+      </c>
+      <c r="C58" t="s">
+        <v>9</v>
+      </c>
+      <c r="D58">
+        <v>2</v>
+      </c>
+      <c r="E58" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5">
+      <c r="A59" t="s">
+        <v>69</v>
+      </c>
+      <c r="B59" t="s">
+        <v>69</v>
+      </c>
+      <c r="C59" t="s">
+        <v>7</v>
+      </c>
+      <c r="D59">
+        <v>3</v>
+      </c>
+      <c r="E59" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5">
+      <c r="A60" t="s">
+        <v>69</v>
+      </c>
+      <c r="B60" t="s">
+        <v>69</v>
+      </c>
+      <c r="C60" t="s">
+        <v>6</v>
+      </c>
+      <c r="D60">
+        <v>3</v>
+      </c>
+      <c r="E60" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
+      <c r="A61" t="s">
+        <v>69</v>
+      </c>
+      <c r="B61" t="s">
+        <v>69</v>
+      </c>
+      <c r="C61" t="s">
+        <v>5</v>
+      </c>
+      <c r="D61">
         <v>1</v>
       </c>
-      <c r="L11">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12">
-      <c r="A12" t="s">
-        <v>62</v>
-      </c>
-      <c r="B12">
+      <c r="E61" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5">
+      <c r="A62" t="s">
+        <v>69</v>
+      </c>
+      <c r="B62" t="s">
+        <v>69</v>
+      </c>
+      <c r="C62" t="s">
+        <v>8</v>
+      </c>
+      <c r="D62">
         <v>2</v>
       </c>
-      <c r="C12">
-        <v>3</v>
-      </c>
-      <c r="D12">
-        <v>5</v>
-      </c>
-      <c r="E12">
-        <v>5</v>
-      </c>
-      <c r="F12">
-        <v>7</v>
-      </c>
-      <c r="G12">
-        <v>7</v>
-      </c>
-      <c r="H12">
-        <v>4</v>
-      </c>
-      <c r="I12">
-        <v>4</v>
-      </c>
-      <c r="J12">
-        <v>3</v>
-      </c>
-      <c r="K12">
-        <v>3</v>
-      </c>
-      <c r="L12">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12">
-      <c r="A13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="3">
-        <v>95</v>
-      </c>
-      <c r="C13" s="3">
-        <v>87</v>
-      </c>
-      <c r="D13" s="3">
-        <v>202</v>
-      </c>
-      <c r="E13" s="3">
-        <v>226</v>
-      </c>
-      <c r="F13" s="3">
-        <v>258</v>
-      </c>
-      <c r="G13" s="3">
-        <v>287</v>
-      </c>
-      <c r="H13" s="3">
-        <v>144</v>
-      </c>
-      <c r="I13" s="3">
-        <v>162</v>
-      </c>
-      <c r="J13" s="3">
-        <v>103</v>
-      </c>
-      <c r="K13" s="3">
-        <v>94</v>
-      </c>
-      <c r="L13" s="3">
-        <v>802</v>
+      <c r="E62" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -2857,156 +3675,542 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="L5" s="4"/>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B6">
+        <v>17</v>
+      </c>
+      <c r="C6">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>36</v>
+      </c>
+      <c r="E6">
+        <v>38</v>
+      </c>
+      <c r="F6">
+        <v>46</v>
+      </c>
+      <c r="G6">
+        <v>49</v>
+      </c>
+      <c r="H6">
+        <v>26</v>
+      </c>
+      <c r="I6">
+        <v>28</v>
+      </c>
+      <c r="J6">
+        <v>18</v>
+      </c>
+      <c r="K6">
+        <v>20</v>
+      </c>
+      <c r="L6">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B7">
+        <v>42</v>
+      </c>
+      <c r="C7">
+        <v>44</v>
+      </c>
+      <c r="D7">
+        <v>88</v>
+      </c>
+      <c r="E7">
+        <v>93</v>
+      </c>
+      <c r="F7">
+        <v>112</v>
+      </c>
+      <c r="G7">
+        <v>119</v>
+      </c>
+      <c r="H7">
+        <v>63</v>
+      </c>
+      <c r="I7">
+        <v>67</v>
+      </c>
+      <c r="J7">
+        <v>45</v>
+      </c>
+      <c r="K7">
+        <v>48</v>
+      </c>
+      <c r="L7">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" t="s">
+        <v>80</v>
+      </c>
+      <c r="B8">
+        <v>17</v>
+      </c>
+      <c r="C8">
+        <v>18</v>
+      </c>
+      <c r="D8">
+        <v>35</v>
+      </c>
+      <c r="E8">
+        <v>37</v>
+      </c>
+      <c r="F8">
+        <v>45</v>
+      </c>
+      <c r="G8">
+        <v>48</v>
+      </c>
+      <c r="H8">
+        <v>25</v>
+      </c>
+      <c r="I8">
+        <v>27</v>
+      </c>
+      <c r="J8">
+        <v>18</v>
+      </c>
+      <c r="K8">
+        <v>19</v>
+      </c>
+      <c r="L8">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>81</v>
+      </c>
+      <c r="B9">
+        <v>16</v>
+      </c>
+      <c r="C9">
+        <v>17</v>
+      </c>
+      <c r="D9">
+        <v>33</v>
+      </c>
+      <c r="E9">
+        <v>36</v>
+      </c>
+      <c r="F9">
+        <v>43</v>
+      </c>
+      <c r="G9">
+        <v>45</v>
+      </c>
+      <c r="H9">
+        <v>24</v>
+      </c>
+      <c r="I9">
+        <v>26</v>
+      </c>
+      <c r="J9">
+        <v>17</v>
+      </c>
+      <c r="K9">
+        <v>18</v>
+      </c>
+      <c r="L9">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>82</v>
+      </c>
+      <c r="B10">
+        <v>16</v>
+      </c>
+      <c r="C10">
+        <v>17</v>
+      </c>
+      <c r="D10">
+        <v>34</v>
+      </c>
+      <c r="E10">
+        <v>36</v>
+      </c>
+      <c r="F10">
+        <v>43</v>
+      </c>
+      <c r="G10">
+        <v>46</v>
+      </c>
+      <c r="H10">
+        <v>24</v>
+      </c>
+      <c r="I10">
+        <v>26</v>
+      </c>
+      <c r="J10">
+        <v>17</v>
+      </c>
+      <c r="K10">
+        <v>18</v>
+      </c>
+      <c r="L10">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>83</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>4</v>
+      </c>
+      <c r="F11">
+        <v>4</v>
+      </c>
+      <c r="G11">
+        <v>5</v>
+      </c>
+      <c r="H11">
+        <v>3</v>
+      </c>
+      <c r="I11">
+        <v>2</v>
+      </c>
+      <c r="J11">
+        <v>2</v>
+      </c>
+      <c r="K11">
+        <v>2</v>
+      </c>
+      <c r="L11">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>4</v>
+      </c>
+      <c r="D12">
+        <v>7</v>
+      </c>
+      <c r="E12">
+        <v>7</v>
+      </c>
+      <c r="F12">
+        <v>9</v>
+      </c>
+      <c r="G12">
+        <v>9</v>
+      </c>
+      <c r="H12">
+        <v>5</v>
+      </c>
+      <c r="I12">
+        <v>5</v>
+      </c>
+      <c r="J12">
+        <v>3</v>
+      </c>
+      <c r="K12">
+        <v>4</v>
+      </c>
+      <c r="L12">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="3">
+        <v>113</v>
+      </c>
+      <c r="C13" s="3">
+        <v>117</v>
+      </c>
+      <c r="D13" s="3">
+        <v>236</v>
+      </c>
+      <c r="E13" s="3">
+        <v>250</v>
+      </c>
+      <c r="F13" s="3">
+        <v>302</v>
+      </c>
+      <c r="G13" s="3">
+        <v>318</v>
+      </c>
+      <c r="H13" s="3">
+        <v>170</v>
+      </c>
+      <c r="I13" s="3">
+        <v>178</v>
+      </c>
+      <c r="J13" s="3">
+        <v>120</v>
+      </c>
+      <c r="K13" s="3">
+        <v>139</v>
+      </c>
+      <c r="L13" s="3">
+        <v>941</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="2" t="s">
-        <v>64</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="4" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>66</v>
+        <v>87</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>67</v>
+        <v>88</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>68</v>
+        <v>89</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>70</v>
+        <v>91</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>71</v>
+        <v>92</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>73</v>
+        <v>94</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>74</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="B5" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="C5" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="D5">
         <v>200.83</v>
       </c>
       <c r="E5">
-        <v>140.58</v>
+        <v>180.75</v>
       </c>
       <c r="F5">
-        <v>187</v>
+        <v>240</v>
       </c>
       <c r="G5">
-        <v>199</v>
+        <v>255</v>
       </c>
       <c r="H5">
-        <v>140.25</v>
+        <v>180</v>
       </c>
       <c r="I5">
-        <v>149.25</v>
+        <v>191.25</v>
       </c>
       <c r="J5" t="s">
-        <v>78</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="B6" t="s">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="C6" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="D6">
         <v>163.94</v>
       </c>
       <c r="E6">
-        <v>114.76</v>
+        <v>147.55</v>
       </c>
       <c r="F6">
-        <v>153</v>
+        <v>196</v>
       </c>
       <c r="G6">
-        <v>163</v>
+        <v>208</v>
       </c>
       <c r="H6">
-        <v>114.75</v>
+        <v>147</v>
       </c>
       <c r="I6">
-        <v>122.25</v>
+        <v>156</v>
       </c>
       <c r="J6" t="s">
-        <v>81</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>82</v>
+        <v>59</v>
       </c>
       <c r="B7" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="C7" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="D7">
         <v>163.3</v>
       </c>
       <c r="E7">
-        <v>114.31</v>
+        <v>146.97</v>
       </c>
       <c r="F7">
-        <v>152</v>
+        <v>195</v>
       </c>
       <c r="G7">
-        <v>162</v>
+        <v>207</v>
       </c>
       <c r="H7">
-        <v>114</v>
+        <v>146.25</v>
       </c>
       <c r="I7">
-        <v>121.5</v>
+        <v>155.25</v>
       </c>
       <c r="J7" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="B8" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="C8" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="D8">
         <v>76.33</v>
@@ -3027,18 +4231,18 @@
         <v>81</v>
       </c>
       <c r="J8" t="s">
-        <v>81</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>88</v>
+        <v>62</v>
       </c>
       <c r="B9" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="C9" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="D9">
         <v>65</v>
@@ -3059,18 +4263,18 @@
         <v>69</v>
       </c>
       <c r="J9" t="s">
-        <v>90</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="B10" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="C10" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="D10">
         <v>29.13</v>
@@ -3091,18 +4295,18 @@
         <v>30.75</v>
       </c>
       <c r="J10" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="B11" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="C11" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="D11">
         <v>28.67</v>
@@ -3123,18 +4327,18 @@
         <v>30.75</v>
       </c>
       <c r="J11" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>96</v>
+        <v>66</v>
       </c>
       <c r="B12" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="C12" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="D12">
         <v>24.25</v>
@@ -3155,18 +4359,18 @@
         <v>25.5</v>
       </c>
       <c r="J12" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="B13" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="C13" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="D13">
         <v>11.5</v>
@@ -3187,7 +4391,7 @@
         <v>12</v>
       </c>
       <c r="J13" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -3199,93 +4403,93 @@
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
       <c r="F14" s="3">
-        <v>802</v>
+        <v>941</v>
       </c>
       <c r="G14" s="3">
-        <v>856</v>
+        <v>1002</v>
       </c>
       <c r="H14" s="3">
-        <v>601.5</v>
+        <v>705.75</v>
       </c>
       <c r="I14" s="3">
-        <v>642</v>
+        <v>751.5</v>
       </c>
       <c r="J14" s="3"/>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="3" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="B18" t="s">
-        <v>101</v>
+        <v>63</v>
       </c>
       <c r="C18" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="D18">
         <v>200.83</v>
       </c>
       <c r="E18">
-        <v>140.58</v>
+        <v>180.75</v>
       </c>
       <c r="F18">
-        <v>187</v>
+        <v>240</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="B19" t="s">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="C19" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="D19">
         <v>163.94</v>
       </c>
       <c r="E19">
-        <v>114.76</v>
+        <v>147.55</v>
       </c>
       <c r="F19">
-        <v>153</v>
+        <v>196</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>82</v>
+        <v>59</v>
       </c>
       <c r="B20" t="s">
-        <v>102</v>
+        <v>58</v>
       </c>
       <c r="C20" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="D20">
         <v>163.3</v>
       </c>
       <c r="E20">
-        <v>114.31</v>
+        <v>146.97</v>
       </c>
       <c r="F20">
-        <v>152</v>
+        <v>195</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="B21" t="s">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="C21" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="D21">
         <v>76.33</v>
@@ -3299,13 +4503,13 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>88</v>
+        <v>62</v>
       </c>
       <c r="B22" t="s">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="C22" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="D22">
         <v>65</v>
@@ -3319,13 +4523,13 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="B23" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="C23" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="D23">
         <v>29.13</v>
@@ -3339,13 +4543,13 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="B24" t="s">
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="C24" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="D24">
         <v>28.67</v>
@@ -3359,13 +4563,13 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>96</v>
+        <v>66</v>
       </c>
       <c r="B25" t="s">
-        <v>96</v>
+        <v>66</v>
       </c>
       <c r="C25" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="D25">
         <v>24.25</v>
@@ -3379,13 +4583,13 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="B26" t="s">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="C26" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="D26">
         <v>11.5</v>

</xml_diff>

<commit_message>
Set LA VELA distribution to 400 und and limit production plan to 100 und in 5 colors
Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SHORT_PLAYA_CAB_Cantidades_Sugeridas_Proyecciones.xlsx
+++ b/SHORT_PLAYA_CAB_Cantidades_Sugeridas_Proyecciones.xlsx
@@ -19,12 +19,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="113">
   <si>
     <t>CANTIDADES POR COLORES</t>
   </si>
   <si>
-    <t>SHORT PLAYA CAB · S12 M25 L32 XL18 2XL13 · LA VELA 350 und · Habano/Azul Verdoso/Azul Pizzarra 90% tela · ≤50 und → S10 M24 L30 XL16 2XL20</t>
+    <t>SHORT PLAYA CAB · S12 M25 L32 XL18 2XL13 · LA VELA 400 und · plan prod. 100 und (5 colores) · Habano/Azul Verdoso/Azul Pizzarra 90% tela · ≤50 und → S10 M24 L30 XL16 2XL20</t>
   </si>
   <si>
     <t>Rango producción: 941 – 1002 und</t>
@@ -180,10 +180,10 @@
     <t>Short Playa · Aguamarina [PRODUCCIÓN · Tela Aguamarina (11.50 m usados) · curva lote chico S10 M24 L30 XL16 2XL20]</t>
   </si>
   <si>
-    <t>SHORT PLAYA CAB — PRODUCCIÓN LA VELA ★ (350 und)</t>
-  </si>
-  <si>
-    <t>Desglose color × talla para playa · prioridad por rotación y stock crítico VELA</t>
+    <t>SHORT PLAYA CAB — PRODUCCIÓN LA VELA ★ (100 und prioritarias)</t>
+  </si>
+  <si>
+    <t>Distribución total tienda LA VELA: 400 und · Plan producción = 100 und · Verde Pino · Azul Pizarra · Azul Verdoso · Marron · Cereza</t>
   </si>
   <si>
     <t>Color</t>
@@ -201,6 +201,12 @@
     <t>Azul Pizzarra</t>
   </si>
   <si>
+    <t>Marron</t>
+  </si>
+  <si>
+    <t>Habano</t>
+  </si>
+  <si>
     <t>Azul Verdoso</t>
   </si>
   <si>
@@ -210,148 +216,142 @@
     <t>Rojo</t>
   </si>
   <si>
-    <t>Marron</t>
-  </si>
-  <si>
-    <t>Habano</t>
-  </si>
-  <si>
     <t>Verde Pino</t>
   </si>
   <si>
+    <t>TOTAL VELA</t>
+  </si>
+  <si>
+    <t>Detalle línea a línea:</t>
+  </si>
+  <si>
+    <t>Und</t>
+  </si>
+  <si>
+    <t>Nota</t>
+  </si>
+  <si>
+    <t>lote chico</t>
+  </si>
+  <si>
+    <t>SHORT PLAYA CAB — DISTRIBUCIÓN POR TIENDA Y TALLA</t>
+  </si>
+  <si>
+    <t>★ LA VELA = 400 und mín · resto tiendas por peso ventas</t>
+  </si>
+  <si>
+    <t>Tienda</t>
+  </si>
+  <si>
+    <t>GRIETA</t>
+  </si>
+  <si>
+    <t>LA VELA ★</t>
+  </si>
+  <si>
+    <t>SAMBIL CHACAO</t>
+  </si>
+  <si>
+    <t>SAMBIL VALENCIA</t>
+  </si>
+  <si>
+    <t>CERRO VERDE</t>
+  </si>
+  <si>
+    <t>GRAND PLAZ</t>
+  </si>
+  <si>
+    <t>TOLON ★</t>
+  </si>
+  <si>
+    <t>SHORT PLAYA CAB — TELA EXISTENTE A AGOTAR (100%)</t>
+  </si>
+  <si>
+    <t>Consumo: 0.75 m/pieza · Habano/Azul Verdoso/Azul Pizzarra al 90% · ≤50 und → S10 M24 L30 XL16 2XL20</t>
+  </si>
+  <si>
+    <t>Producto</t>
+  </si>
+  <si>
+    <t>% Tela</t>
+  </si>
+  <si>
+    <t>Mts stock</t>
+  </si>
+  <si>
+    <t>Mts usados</t>
+  </si>
+  <si>
+    <t>Und Mín</t>
+  </si>
+  <si>
+    <t>Und Máx</t>
+  </si>
+  <si>
+    <t>Mts prod Mín</t>
+  </si>
+  <si>
+    <t>Mts prod Máx</t>
+  </si>
+  <si>
+    <t>Notas</t>
+  </si>
+  <si>
+    <t>Short Playa · Marron</t>
+  </si>
+  <si>
+    <t>90%</t>
+  </si>
+  <si>
+    <t>Curva global ventas · Tela HABANO</t>
+  </si>
+  <si>
+    <t>Short Playa · Azul Verdoso</t>
+  </si>
+  <si>
+    <t>Curva global ventas</t>
+  </si>
+  <si>
+    <t>Short Playa · Azul Pizarra</t>
+  </si>
+  <si>
+    <t>Curva global ventas · Tela AZUL PIZZARRA</t>
+  </si>
+  <si>
+    <t>Short Playa · Verde Pino</t>
+  </si>
+  <si>
+    <t>100%</t>
+  </si>
+  <si>
+    <t>Short Playa · Cereza</t>
+  </si>
+  <si>
+    <t>Curva global ventas · Tela ROJO</t>
+  </si>
+  <si>
+    <t>Verde Oliva</t>
+  </si>
+  <si>
+    <t>Short Playa · Verde Oliva</t>
+  </si>
+  <si>
+    <t>Curva global ventas · Lote chico → todas las tallas</t>
+  </si>
+  <si>
+    <t>Gris Azulado</t>
+  </si>
+  <si>
+    <t>Short Playa · Gris Azulado</t>
+  </si>
+  <si>
     <t>Azul Marino</t>
   </si>
   <si>
-    <t>Gris Azulado</t>
-  </si>
-  <si>
-    <t>Verde Oliva</t>
+    <t>Short Playa · Azul Marino</t>
   </si>
   <si>
     <t>Aguamarina</t>
-  </si>
-  <si>
-    <t>TOTAL VELA</t>
-  </si>
-  <si>
-    <t>Detalle línea a línea:</t>
-  </si>
-  <si>
-    <t>Und</t>
-  </si>
-  <si>
-    <t>Nota</t>
-  </si>
-  <si>
-    <t>lote chico</t>
-  </si>
-  <si>
-    <t>SHORT PLAYA CAB — DISTRIBUCIÓN POR TIENDA Y TALLA</t>
-  </si>
-  <si>
-    <t>★ LA VELA = 350 und mín · resto tiendas por peso ventas</t>
-  </si>
-  <si>
-    <t>Tienda</t>
-  </si>
-  <si>
-    <t>GRIETA</t>
-  </si>
-  <si>
-    <t>LA VELA ★</t>
-  </si>
-  <si>
-    <t>SAMBIL CHACAO</t>
-  </si>
-  <si>
-    <t>SAMBIL VALENCIA</t>
-  </si>
-  <si>
-    <t>CERRO VERDE</t>
-  </si>
-  <si>
-    <t>GRAND PLAZ</t>
-  </si>
-  <si>
-    <t>TOLON ★</t>
-  </si>
-  <si>
-    <t>SHORT PLAYA CAB — TELA EXISTENTE A AGOTAR (100%)</t>
-  </si>
-  <si>
-    <t>Consumo: 0.75 m/pieza · Habano/Azul Verdoso/Azul Pizzarra al 90% · ≤50 und → S10 M24 L30 XL16 2XL20</t>
-  </si>
-  <si>
-    <t>Producto</t>
-  </si>
-  <si>
-    <t>% Tela</t>
-  </si>
-  <si>
-    <t>Mts stock</t>
-  </si>
-  <si>
-    <t>Mts usados</t>
-  </si>
-  <si>
-    <t>Und Mín</t>
-  </si>
-  <si>
-    <t>Und Máx</t>
-  </si>
-  <si>
-    <t>Mts prod Mín</t>
-  </si>
-  <si>
-    <t>Mts prod Máx</t>
-  </si>
-  <si>
-    <t>Notas</t>
-  </si>
-  <si>
-    <t>Short Playa · Marron</t>
-  </si>
-  <si>
-    <t>90%</t>
-  </si>
-  <si>
-    <t>Curva global ventas · Tela HABANO</t>
-  </si>
-  <si>
-    <t>Short Playa · Azul Verdoso</t>
-  </si>
-  <si>
-    <t>Curva global ventas</t>
-  </si>
-  <si>
-    <t>Short Playa · Azul Pizarra</t>
-  </si>
-  <si>
-    <t>Curva global ventas · Tela AZUL PIZZARRA</t>
-  </si>
-  <si>
-    <t>Short Playa · Verde Pino</t>
-  </si>
-  <si>
-    <t>100%</t>
-  </si>
-  <si>
-    <t>Short Playa · Cereza</t>
-  </si>
-  <si>
-    <t>Curva global ventas · Tela ROJO</t>
-  </si>
-  <si>
-    <t>Short Playa · Verde Oliva</t>
-  </si>
-  <si>
-    <t>Curva global ventas · Lote chico → todas las tallas</t>
-  </si>
-  <si>
-    <t>Short Playa · Gris Azulado</t>
-  </si>
-  <si>
-    <t>Short Playa · Azul Marino</t>
   </si>
   <si>
     <t>Short Playa · Aguamarina</t>
@@ -2659,7 +2659,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -2706,22 +2706,22 @@
         <v>59</v>
       </c>
       <c r="C5">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D5">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="E5">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="F5">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H5">
-        <v>57</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -2729,51 +2729,51 @@
         <v>60</v>
       </c>
       <c r="B6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C6">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D6">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="E6">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="F6">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G6">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H6">
-        <v>56</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B7" t="s">
         <v>62</v>
       </c>
       <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>5</v>
+      </c>
+      <c r="E7">
         <v>6</v>
       </c>
-      <c r="D7">
-        <v>14</v>
-      </c>
-      <c r="E7">
-        <v>18</v>
-      </c>
       <c r="F7">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G7">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H7">
-        <v>55</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -2784,22 +2784,22 @@
         <v>64</v>
       </c>
       <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8">
+        <v>5</v>
+      </c>
+      <c r="E8">
         <v>6</v>
       </c>
-      <c r="D8">
-        <v>13</v>
-      </c>
-      <c r="E8">
-        <v>17</v>
-      </c>
       <c r="F8">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G8">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H8">
-        <v>53</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -2810,172 +2810,136 @@
         <v>65</v>
       </c>
       <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9">
+        <v>4</v>
+      </c>
+      <c r="E9">
         <v>6</v>
       </c>
-      <c r="D9">
-        <v>13</v>
-      </c>
-      <c r="E9">
-        <v>17</v>
-      </c>
       <c r="F9">
+        <v>3</v>
+      </c>
+      <c r="G9">
+        <v>4</v>
+      </c>
+      <c r="H9">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3">
+        <v>10</v>
+      </c>
+      <c r="D10" s="3">
+        <v>24</v>
+      </c>
+      <c r="E10" s="3">
+        <v>30</v>
+      </c>
+      <c r="F10" s="3">
+        <v>16</v>
+      </c>
+      <c r="G10" s="3">
+        <v>20</v>
+      </c>
+      <c r="H10" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14" t="s">
         <v>9</v>
       </c>
-      <c r="G9">
+      <c r="D14">
+        <v>4</v>
+      </c>
+      <c r="E14" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" t="s">
+        <v>58</v>
+      </c>
+      <c r="B15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" t="s">
         <v>7</v>
       </c>
-      <c r="H9">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" t="s">
-        <v>66</v>
-      </c>
-      <c r="B10" t="s">
-        <v>66</v>
-      </c>
-      <c r="C10">
-        <v>3</v>
-      </c>
-      <c r="D10">
-        <v>7</v>
-      </c>
-      <c r="E10">
-        <v>9</v>
-      </c>
-      <c r="F10">
+      <c r="D15">
+        <v>6</v>
+      </c>
+      <c r="E15" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16">
         <v>5</v>
       </c>
-      <c r="G10">
-        <v>6</v>
-      </c>
-      <c r="H10">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" t="s">
-        <v>67</v>
-      </c>
-      <c r="B11" t="s">
-        <v>67</v>
-      </c>
-      <c r="C11">
+      <c r="E16" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" t="s">
+        <v>58</v>
+      </c>
+      <c r="B17" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" t="s">
+        <v>5</v>
+      </c>
+      <c r="D17">
         <v>2</v>
       </c>
-      <c r="D11">
-        <v>5</v>
-      </c>
-      <c r="E11">
-        <v>6</v>
-      </c>
-      <c r="F11">
-        <v>4</v>
-      </c>
-      <c r="G11">
-        <v>4</v>
-      </c>
-      <c r="H11">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" t="s">
-        <v>68</v>
-      </c>
-      <c r="B12" t="s">
-        <v>68</v>
-      </c>
-      <c r="C12">
-        <v>2</v>
-      </c>
-      <c r="D12">
-        <v>4</v>
-      </c>
-      <c r="E12">
-        <v>4</v>
-      </c>
-      <c r="F12">
-        <v>2</v>
-      </c>
-      <c r="G12">
-        <v>3</v>
-      </c>
-      <c r="H12">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13" t="s">
-        <v>69</v>
-      </c>
-      <c r="B13" t="s">
-        <v>69</v>
-      </c>
-      <c r="C13">
-        <v>1</v>
-      </c>
-      <c r="D13">
-        <v>3</v>
-      </c>
-      <c r="E13">
-        <v>3</v>
-      </c>
-      <c r="F13">
-        <v>2</v>
-      </c>
-      <c r="G13">
-        <v>2</v>
-      </c>
-      <c r="H13">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="A14" s="3" t="s">
+      <c r="E17" t="s">
         <v>70</v>
-      </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3">
-        <v>40</v>
-      </c>
-      <c r="D14" s="3">
-        <v>87</v>
-      </c>
-      <c r="E14" s="3">
-        <v>110</v>
-      </c>
-      <c r="F14" s="3">
-        <v>62</v>
-      </c>
-      <c r="G14" s="3">
-        <v>51</v>
-      </c>
-      <c r="H14" s="3">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
-      <c r="A16" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="A17" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -2986,276 +2950,336 @@
         <v>59</v>
       </c>
       <c r="C18" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D18">
-        <v>8</v>
+        <v>4</v>
+      </c>
+      <c r="E18" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B19" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C19" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D19">
-        <v>18</v>
+        <v>4</v>
+      </c>
+      <c r="E19" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B20" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
         <v>6</v>
       </c>
-      <c r="D20">
-        <v>14</v>
+      <c r="E20" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B21" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D21">
         <v>5</v>
       </c>
-      <c r="D21">
-        <v>7</v>
+      <c r="E21" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B22" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C22" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D22">
-        <v>10</v>
+        <v>2</v>
+      </c>
+      <c r="E22" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B23" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C23" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D23">
-        <v>7</v>
+        <v>3</v>
+      </c>
+      <c r="E23" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B24" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C24" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D24">
-        <v>18</v>
+        <v>4</v>
+      </c>
+      <c r="E24" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B25" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C25" t="s">
+        <v>7</v>
+      </c>
+      <c r="D25">
         <v>6</v>
       </c>
-      <c r="D25">
-        <v>14</v>
+      <c r="E25" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B26" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C26" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26">
         <v>5</v>
       </c>
-      <c r="D26">
-        <v>7</v>
+      <c r="E26" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C27" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D27">
-        <v>10</v>
+        <v>2</v>
+      </c>
+      <c r="E27" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B28" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C28" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D28">
-        <v>7</v>
+        <v>3</v>
+      </c>
+      <c r="E28" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
+        <v>60</v>
+      </c>
+      <c r="B29" t="s">
         <v>61</v>
       </c>
-      <c r="B29" t="s">
-        <v>62</v>
-      </c>
       <c r="C29" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D29">
-        <v>18</v>
+        <v>4</v>
+      </c>
+      <c r="E29" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
+        <v>60</v>
+      </c>
+      <c r="B30" t="s">
         <v>61</v>
       </c>
-      <c r="B30" t="s">
-        <v>62</v>
-      </c>
       <c r="C30" t="s">
+        <v>7</v>
+      </c>
+      <c r="D30">
         <v>6</v>
       </c>
-      <c r="D30">
-        <v>14</v>
+      <c r="E30" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
+        <v>60</v>
+      </c>
+      <c r="B31" t="s">
         <v>61</v>
       </c>
-      <c r="B31" t="s">
-        <v>62</v>
-      </c>
       <c r="C31" t="s">
+        <v>6</v>
+      </c>
+      <c r="D31">
         <v>5</v>
       </c>
-      <c r="D31">
-        <v>6</v>
+      <c r="E31" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
+        <v>60</v>
+      </c>
+      <c r="B32" t="s">
         <v>61</v>
       </c>
-      <c r="B32" t="s">
-        <v>62</v>
-      </c>
       <c r="C32" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D32">
-        <v>10</v>
+        <v>2</v>
+      </c>
+      <c r="E32" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B33" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C33" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D33">
-        <v>7</v>
+        <v>3</v>
+      </c>
+      <c r="E33" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B34" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C34" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D34">
-        <v>17</v>
+        <v>4</v>
+      </c>
+      <c r="E34" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B35" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C35" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35">
         <v>6</v>
       </c>
-      <c r="D35">
-        <v>13</v>
+      <c r="E35" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B36" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C36" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D36">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="E36" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B37" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C37" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D37">
-        <v>10</v>
+        <v>2</v>
+      </c>
+      <c r="E37" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -3266,406 +3290,13 @@
         <v>65</v>
       </c>
       <c r="C38" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D38">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5">
-      <c r="A39" t="s">
-        <v>65</v>
-      </c>
-      <c r="B39" t="s">
-        <v>65</v>
-      </c>
-      <c r="C39" t="s">
-        <v>7</v>
-      </c>
-      <c r="D39">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5">
-      <c r="A40" t="s">
-        <v>65</v>
-      </c>
-      <c r="B40" t="s">
-        <v>65</v>
-      </c>
-      <c r="C40" t="s">
-        <v>6</v>
-      </c>
-      <c r="D40">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5">
-      <c r="A41" t="s">
-        <v>65</v>
-      </c>
-      <c r="B41" t="s">
-        <v>65</v>
-      </c>
-      <c r="C41" t="s">
-        <v>5</v>
-      </c>
-      <c r="D41">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5">
-      <c r="A42" t="s">
-        <v>65</v>
-      </c>
-      <c r="B42" t="s">
-        <v>65</v>
-      </c>
-      <c r="C42" t="s">
-        <v>8</v>
-      </c>
-      <c r="D42">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5">
-      <c r="A43" t="s">
-        <v>66</v>
-      </c>
-      <c r="B43" t="s">
-        <v>66</v>
-      </c>
-      <c r="C43" t="s">
-        <v>9</v>
-      </c>
-      <c r="D43">
-        <v>6</v>
-      </c>
-      <c r="E43" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5">
-      <c r="A44" t="s">
-        <v>66</v>
-      </c>
-      <c r="B44" t="s">
-        <v>66</v>
-      </c>
-      <c r="C44" t="s">
-        <v>7</v>
-      </c>
-      <c r="D44">
-        <v>9</v>
-      </c>
-      <c r="E44" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5">
-      <c r="A45" t="s">
-        <v>66</v>
-      </c>
-      <c r="B45" t="s">
-        <v>66</v>
-      </c>
-      <c r="C45" t="s">
-        <v>6</v>
-      </c>
-      <c r="D45">
-        <v>7</v>
-      </c>
-      <c r="E45" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5">
-      <c r="A46" t="s">
-        <v>66</v>
-      </c>
-      <c r="B46" t="s">
-        <v>66</v>
-      </c>
-      <c r="C46" t="s">
-        <v>5</v>
-      </c>
-      <c r="D46">
         <v>3</v>
       </c>
-      <c r="E46" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5">
-      <c r="A47" t="s">
-        <v>66</v>
-      </c>
-      <c r="B47" t="s">
-        <v>66</v>
-      </c>
-      <c r="C47" t="s">
-        <v>8</v>
-      </c>
-      <c r="D47">
-        <v>5</v>
-      </c>
-      <c r="E47" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5">
-      <c r="A48" t="s">
-        <v>67</v>
-      </c>
-      <c r="B48" t="s">
-        <v>67</v>
-      </c>
-      <c r="C48" t="s">
-        <v>9</v>
-      </c>
-      <c r="D48">
-        <v>4</v>
-      </c>
-      <c r="E48" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5">
-      <c r="A49" t="s">
-        <v>67</v>
-      </c>
-      <c r="B49" t="s">
-        <v>67</v>
-      </c>
-      <c r="C49" t="s">
-        <v>7</v>
-      </c>
-      <c r="D49">
-        <v>6</v>
-      </c>
-      <c r="E49" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5">
-      <c r="A50" t="s">
-        <v>67</v>
-      </c>
-      <c r="B50" t="s">
-        <v>67</v>
-      </c>
-      <c r="C50" t="s">
-        <v>6</v>
-      </c>
-      <c r="D50">
-        <v>5</v>
-      </c>
-      <c r="E50" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5">
-      <c r="A51" t="s">
-        <v>67</v>
-      </c>
-      <c r="B51" t="s">
-        <v>67</v>
-      </c>
-      <c r="C51" t="s">
-        <v>5</v>
-      </c>
-      <c r="D51">
-        <v>2</v>
-      </c>
-      <c r="E51" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5">
-      <c r="A52" t="s">
-        <v>67</v>
-      </c>
-      <c r="B52" t="s">
-        <v>67</v>
-      </c>
-      <c r="C52" t="s">
-        <v>8</v>
-      </c>
-      <c r="D52">
-        <v>4</v>
-      </c>
-      <c r="E52" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5">
-      <c r="A53" t="s">
-        <v>68</v>
-      </c>
-      <c r="B53" t="s">
-        <v>68</v>
-      </c>
-      <c r="C53" t="s">
-        <v>9</v>
-      </c>
-      <c r="D53">
-        <v>3</v>
-      </c>
-      <c r="E53" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5">
-      <c r="A54" t="s">
-        <v>68</v>
-      </c>
-      <c r="B54" t="s">
-        <v>68</v>
-      </c>
-      <c r="C54" t="s">
-        <v>7</v>
-      </c>
-      <c r="D54">
-        <v>4</v>
-      </c>
-      <c r="E54" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5">
-      <c r="A55" t="s">
-        <v>68</v>
-      </c>
-      <c r="B55" t="s">
-        <v>68</v>
-      </c>
-      <c r="C55" t="s">
-        <v>6</v>
-      </c>
-      <c r="D55">
-        <v>4</v>
-      </c>
-      <c r="E55" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5">
-      <c r="A56" t="s">
-        <v>68</v>
-      </c>
-      <c r="B56" t="s">
-        <v>68</v>
-      </c>
-      <c r="C56" t="s">
-        <v>5</v>
-      </c>
-      <c r="D56">
-        <v>2</v>
-      </c>
-      <c r="E56" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5">
-      <c r="A57" t="s">
-        <v>68</v>
-      </c>
-      <c r="B57" t="s">
-        <v>68</v>
-      </c>
-      <c r="C57" t="s">
-        <v>8</v>
-      </c>
-      <c r="D57">
-        <v>2</v>
-      </c>
-      <c r="E57" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5">
-      <c r="A58" t="s">
-        <v>69</v>
-      </c>
-      <c r="B58" t="s">
-        <v>69</v>
-      </c>
-      <c r="C58" t="s">
-        <v>9</v>
-      </c>
-      <c r="D58">
-        <v>2</v>
-      </c>
-      <c r="E58" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5">
-      <c r="A59" t="s">
-        <v>69</v>
-      </c>
-      <c r="B59" t="s">
-        <v>69</v>
-      </c>
-      <c r="C59" t="s">
-        <v>7</v>
-      </c>
-      <c r="D59">
-        <v>3</v>
-      </c>
-      <c r="E59" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5">
-      <c r="A60" t="s">
-        <v>69</v>
-      </c>
-      <c r="B60" t="s">
-        <v>69</v>
-      </c>
-      <c r="C60" t="s">
-        <v>6</v>
-      </c>
-      <c r="D60">
-        <v>3</v>
-      </c>
-      <c r="E60" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5">
-      <c r="A61" t="s">
-        <v>69</v>
-      </c>
-      <c r="B61" t="s">
-        <v>69</v>
-      </c>
-      <c r="C61" t="s">
-        <v>5</v>
-      </c>
-      <c r="D61">
-        <v>1</v>
-      </c>
-      <c r="E61" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5">
-      <c r="A62" t="s">
-        <v>69</v>
-      </c>
-      <c r="B62" t="s">
-        <v>69</v>
-      </c>
-      <c r="C62" t="s">
-        <v>8</v>
-      </c>
-      <c r="D62">
-        <v>2</v>
-      </c>
-      <c r="E62" t="s">
-        <v>74</v>
+      <c r="E38" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -3680,17 +3311,17 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="4" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>5</v>
@@ -3752,197 +3383,197 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B6">
+        <v>16</v>
+      </c>
+      <c r="C6">
         <v>17</v>
       </c>
-      <c r="C6">
+      <c r="D6">
+        <v>33</v>
+      </c>
+      <c r="E6">
+        <v>35</v>
+      </c>
+      <c r="F6">
+        <v>42</v>
+      </c>
+      <c r="G6">
+        <v>45</v>
+      </c>
+      <c r="H6">
+        <v>23</v>
+      </c>
+      <c r="I6">
+        <v>25</v>
+      </c>
+      <c r="J6">
+        <v>17</v>
+      </c>
+      <c r="K6">
         <v>18</v>
       </c>
-      <c r="D6">
-        <v>36</v>
-      </c>
-      <c r="E6">
-        <v>38</v>
-      </c>
-      <c r="F6">
-        <v>46</v>
-      </c>
-      <c r="G6">
-        <v>49</v>
-      </c>
-      <c r="H6">
-        <v>26</v>
-      </c>
-      <c r="I6">
-        <v>28</v>
-      </c>
-      <c r="J6">
-        <v>18</v>
-      </c>
-      <c r="K6">
-        <v>20</v>
-      </c>
       <c r="L6">
-        <v>143</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B7">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="C7">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="D7">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="E7">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="F7">
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="G7">
-        <v>119</v>
+        <v>136</v>
       </c>
       <c r="H7">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="I7">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="J7">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="K7">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L7">
-        <v>350</v>
+        <v>400</v>
       </c>
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B8">
+        <v>15</v>
+      </c>
+      <c r="C8">
+        <v>16</v>
+      </c>
+      <c r="D8">
+        <v>32</v>
+      </c>
+      <c r="E8">
+        <v>34</v>
+      </c>
+      <c r="F8">
+        <v>41</v>
+      </c>
+      <c r="G8">
+        <v>44</v>
+      </c>
+      <c r="H8">
+        <v>23</v>
+      </c>
+      <c r="I8">
+        <v>25</v>
+      </c>
+      <c r="J8">
         <v>17</v>
       </c>
-      <c r="C8">
+      <c r="K8">
         <v>18</v>
       </c>
-      <c r="D8">
-        <v>35</v>
-      </c>
-      <c r="E8">
-        <v>37</v>
-      </c>
-      <c r="F8">
-        <v>45</v>
-      </c>
-      <c r="G8">
-        <v>48</v>
-      </c>
-      <c r="H8">
-        <v>25</v>
-      </c>
-      <c r="I8">
-        <v>27</v>
-      </c>
-      <c r="J8">
-        <v>18</v>
-      </c>
-      <c r="K8">
-        <v>19</v>
-      </c>
       <c r="L8">
-        <v>140</v>
+        <v>128</v>
       </c>
     </row>
     <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B9">
+        <v>15</v>
+      </c>
+      <c r="C9">
         <v>16</v>
       </c>
-      <c r="C9">
+      <c r="D9">
+        <v>30</v>
+      </c>
+      <c r="E9">
+        <v>32</v>
+      </c>
+      <c r="F9">
+        <v>39</v>
+      </c>
+      <c r="G9">
+        <v>42</v>
+      </c>
+      <c r="H9">
+        <v>22</v>
+      </c>
+      <c r="I9">
+        <v>23</v>
+      </c>
+      <c r="J9">
+        <v>16</v>
+      </c>
+      <c r="K9">
         <v>17</v>
       </c>
-      <c r="D9">
-        <v>33</v>
-      </c>
-      <c r="E9">
-        <v>36</v>
-      </c>
-      <c r="F9">
-        <v>43</v>
-      </c>
-      <c r="G9">
-        <v>45</v>
-      </c>
-      <c r="H9">
-        <v>24</v>
-      </c>
-      <c r="I9">
-        <v>26</v>
-      </c>
-      <c r="J9">
-        <v>17</v>
-      </c>
-      <c r="K9">
-        <v>18</v>
-      </c>
       <c r="L9">
-        <v>133</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B10">
+        <v>15</v>
+      </c>
+      <c r="C10">
         <v>16</v>
       </c>
-      <c r="C10">
+      <c r="D10">
+        <v>30</v>
+      </c>
+      <c r="E10">
+        <v>33</v>
+      </c>
+      <c r="F10">
+        <v>39</v>
+      </c>
+      <c r="G10">
+        <v>42</v>
+      </c>
+      <c r="H10">
+        <v>22</v>
+      </c>
+      <c r="I10">
+        <v>23</v>
+      </c>
+      <c r="J10">
+        <v>16</v>
+      </c>
+      <c r="K10">
         <v>17</v>
       </c>
-      <c r="D10">
-        <v>34</v>
-      </c>
-      <c r="E10">
-        <v>36</v>
-      </c>
-      <c r="F10">
-        <v>43</v>
-      </c>
-      <c r="G10">
-        <v>46</v>
-      </c>
-      <c r="H10">
-        <v>24</v>
-      </c>
-      <c r="I10">
-        <v>26</v>
-      </c>
-      <c r="J10">
-        <v>17</v>
-      </c>
-      <c r="K10">
-        <v>18</v>
-      </c>
       <c r="L10">
-        <v>134</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B11">
         <v>2</v>
@@ -3954,19 +3585,19 @@
         <v>3</v>
       </c>
       <c r="E11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F11">
         <v>4</v>
       </c>
       <c r="G11">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H11">
+        <v>2</v>
+      </c>
+      <c r="I11">
         <v>3</v>
-      </c>
-      <c r="I11">
-        <v>2</v>
       </c>
       <c r="J11">
         <v>2</v>
@@ -3975,30 +3606,30 @@
         <v>2</v>
       </c>
       <c r="L11">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B12">
         <v>3</v>
       </c>
       <c r="C12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D12">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E12">
         <v>7</v>
       </c>
       <c r="F12">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G12">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H12">
         <v>5</v>
@@ -4010,10 +3641,10 @@
         <v>3</v>
       </c>
       <c r="K12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L12">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -4021,31 +3652,31 @@
         <v>35</v>
       </c>
       <c r="B13" s="3">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C13" s="3">
         <v>117</v>
       </c>
       <c r="D13" s="3">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E13" s="3">
         <v>250</v>
       </c>
       <c r="F13" s="3">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G13" s="3">
         <v>318</v>
       </c>
       <c r="H13" s="3">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="I13" s="3">
         <v>178</v>
       </c>
       <c r="J13" s="3">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="K13" s="3">
         <v>139</v>
@@ -4066,12 +3697,12 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="2" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -4079,42 +3710,42 @@
         <v>56</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="H4" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="I4" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="J4" s="4" t="s">
         <v>91</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B5" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C5" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D5">
         <v>200.83</v>
@@ -4135,18 +3766,18 @@
         <v>191.25</v>
       </c>
       <c r="J5" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B6" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C6" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D6">
         <v>163.94</v>
@@ -4167,7 +3798,7 @@
         <v>156</v>
       </c>
       <c r="J6" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -4175,10 +3806,10 @@
         <v>59</v>
       </c>
       <c r="B7" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C7" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D7">
         <v>163.3</v>
@@ -4199,7 +3830,7 @@
         <v>155.25</v>
       </c>
       <c r="J7" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -4207,10 +3838,10 @@
         <v>65</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C8" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D8">
         <v>76.33</v>
@@ -4231,18 +3862,18 @@
         <v>81</v>
       </c>
       <c r="J8" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B9" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D9">
         <v>65</v>
@@ -4263,18 +3894,18 @@
         <v>69</v>
       </c>
       <c r="J9" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>68</v>
+        <v>103</v>
       </c>
       <c r="B10" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C10" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D10">
         <v>29.13</v>
@@ -4295,18 +3926,18 @@
         <v>30.75</v>
       </c>
       <c r="J10" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="B11" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C11" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D11">
         <v>28.67</v>
@@ -4327,18 +3958,18 @@
         <v>30.75</v>
       </c>
       <c r="J11" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>66</v>
+        <v>108</v>
       </c>
       <c r="B12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C12" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D12">
         <v>24.25</v>
@@ -4359,18 +3990,18 @@
         <v>25.5</v>
       </c>
       <c r="J12" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>69</v>
+        <v>110</v>
       </c>
       <c r="B13" t="s">
         <v>111</v>
       </c>
       <c r="C13" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D13">
         <v>11.5</v>
@@ -4391,7 +4022,7 @@
         <v>12</v>
       </c>
       <c r="J13" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -4423,13 +4054,13 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B18" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C18" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D18">
         <v>200.83</v>
@@ -4443,13 +4074,13 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B19" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C19" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D19">
         <v>163.94</v>
@@ -4469,7 +4100,7 @@
         <v>58</v>
       </c>
       <c r="C20" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D20">
         <v>163.3</v>
@@ -4489,7 +4120,7 @@
         <v>65</v>
       </c>
       <c r="C21" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D21">
         <v>76.33</v>
@@ -4503,13 +4134,13 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B22" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C22" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D22">
         <v>65</v>
@@ -4523,13 +4154,13 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>68</v>
+        <v>103</v>
       </c>
       <c r="B23" t="s">
-        <v>68</v>
+        <v>103</v>
       </c>
       <c r="C23" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D23">
         <v>29.13</v>
@@ -4543,13 +4174,13 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="B24" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="C24" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D24">
         <v>28.67</v>
@@ -4563,13 +4194,13 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>66</v>
+        <v>108</v>
       </c>
       <c r="B25" t="s">
-        <v>66</v>
+        <v>108</v>
       </c>
       <c r="C25" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D25">
         <v>24.25</v>
@@ -4583,13 +4214,13 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>69</v>
+        <v>110</v>
       </c>
       <c r="B26" t="s">
-        <v>69</v>
+        <v>110</v>
       </c>
       <c r="C26" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D26">
         <v>11.5</v>

</xml_diff>

<commit_message>
Add Producción Satélite sheet as global minus VELA priority batch
Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SHORT_PLAYA_CAB_Cantidades_Sugeridas_Proyecciones.xlsx
+++ b/SHORT_PLAYA_CAB_Cantidades_Sugeridas_Proyecciones.xlsx
@@ -10,16 +10,17 @@
     <sheet name="Cantidades por Colores" sheetId="1" r:id="rId1"/>
     <sheet name="Producción por Talla" sheetId="2" r:id="rId2"/>
     <sheet name="Producción Color × Talla" sheetId="3" r:id="rId3"/>
-    <sheet name="Producción LA VELA" sheetId="4" r:id="rId4"/>
-    <sheet name="Distribución por Tienda" sheetId="5" r:id="rId5"/>
-    <sheet name="Uso de Tela Short Playa" sheetId="6" r:id="rId6"/>
+    <sheet name="Distribución por Tienda" sheetId="4" r:id="rId4"/>
+    <sheet name="Uso de Tela Short Playa" sheetId="5" r:id="rId5"/>
+    <sheet name="Producción LA VELA" sheetId="6" r:id="rId6"/>
+    <sheet name="Producción Satélite" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="117">
   <si>
     <t>CANTIDADES POR COLORES</t>
   </si>
@@ -180,6 +181,159 @@
     <t>Short Playa · Aguamarina [PRODUCCIÓN · Tela Aguamarina (11.50 m usados) · curva lote chico S10 M24 L30 XL16 2XL20]</t>
   </si>
   <si>
+    <t>SHORT PLAYA CAB — DISTRIBUCIÓN POR TIENDA Y TALLA</t>
+  </si>
+  <si>
+    <t>★ LA VELA = 400 und mín · resto tiendas por peso ventas</t>
+  </si>
+  <si>
+    <t>Tienda</t>
+  </si>
+  <si>
+    <t>GRIETA</t>
+  </si>
+  <si>
+    <t>LA VELA ★</t>
+  </si>
+  <si>
+    <t>SAMBIL CHACAO</t>
+  </si>
+  <si>
+    <t>SAMBIL VALENCIA</t>
+  </si>
+  <si>
+    <t>CERRO VERDE</t>
+  </si>
+  <si>
+    <t>GRAND PLAZ</t>
+  </si>
+  <si>
+    <t>TOLON ★</t>
+  </si>
+  <si>
+    <t>SHORT PLAYA CAB — TELA EXISTENTE A AGOTAR (100%)</t>
+  </si>
+  <si>
+    <t>Consumo: 0.75 m/pieza · Habano/Azul Verdoso/Azul Pizzarra al 90% · ≤50 und → S10 M24 L30 XL16 2XL20</t>
+  </si>
+  <si>
+    <t>Tela</t>
+  </si>
+  <si>
+    <t>Producto</t>
+  </si>
+  <si>
+    <t>% Tela</t>
+  </si>
+  <si>
+    <t>Mts stock</t>
+  </si>
+  <si>
+    <t>Mts usados</t>
+  </si>
+  <si>
+    <t>Und Mín</t>
+  </si>
+  <si>
+    <t>Und Máx</t>
+  </si>
+  <si>
+    <t>Mts prod Mín</t>
+  </si>
+  <si>
+    <t>Mts prod Máx</t>
+  </si>
+  <si>
+    <t>Notas</t>
+  </si>
+  <si>
+    <t>Habano</t>
+  </si>
+  <si>
+    <t>Short Playa · Marron</t>
+  </si>
+  <si>
+    <t>90%</t>
+  </si>
+  <si>
+    <t>Curva global ventas · Tela HABANO</t>
+  </si>
+  <si>
+    <t>Azul Verdoso</t>
+  </si>
+  <si>
+    <t>Short Playa · Azul Verdoso</t>
+  </si>
+  <si>
+    <t>Curva global ventas</t>
+  </si>
+  <si>
+    <t>Azul Pizzarra</t>
+  </si>
+  <si>
+    <t>Short Playa · Azul Pizarra</t>
+  </si>
+  <si>
+    <t>Curva global ventas · Tela AZUL PIZZARRA</t>
+  </si>
+  <si>
+    <t>Verde Pino</t>
+  </si>
+  <si>
+    <t>Short Playa · Verde Pino</t>
+  </si>
+  <si>
+    <t>100%</t>
+  </si>
+  <si>
+    <t>Rojo</t>
+  </si>
+  <si>
+    <t>Short Playa · Cereza</t>
+  </si>
+  <si>
+    <t>Curva global ventas · Tela ROJO</t>
+  </si>
+  <si>
+    <t>Verde Oliva</t>
+  </si>
+  <si>
+    <t>Short Playa · Verde Oliva</t>
+  </si>
+  <si>
+    <t>Curva global ventas · Lote chico → todas las tallas</t>
+  </si>
+  <si>
+    <t>Gris Azulado</t>
+  </si>
+  <si>
+    <t>Short Playa · Gris Azulado</t>
+  </si>
+  <si>
+    <t>Azul Marino</t>
+  </si>
+  <si>
+    <t>Short Playa · Azul Marino</t>
+  </si>
+  <si>
+    <t>Aguamarina</t>
+  </si>
+  <si>
+    <t>Short Playa · Aguamarina</t>
+  </si>
+  <si>
+    <t>Resumen tela stock vs usada:</t>
+  </si>
+  <si>
+    <t>Marron</t>
+  </si>
+  <si>
+    <t>Azul Pizarra</t>
+  </si>
+  <si>
+    <t>Cereza</t>
+  </si>
+  <si>
     <t>SHORT PLAYA CAB — PRODUCCIÓN LA VELA ★ (100 und prioritarias)</t>
   </si>
   <si>
@@ -189,36 +343,9 @@
     <t>Color</t>
   </si>
   <si>
-    <t>Tela</t>
-  </si>
-  <si>
     <t>Total</t>
   </si>
   <si>
-    <t>Azul Pizarra</t>
-  </si>
-  <si>
-    <t>Azul Pizzarra</t>
-  </si>
-  <si>
-    <t>Marron</t>
-  </si>
-  <si>
-    <t>Habano</t>
-  </si>
-  <si>
-    <t>Azul Verdoso</t>
-  </si>
-  <si>
-    <t>Cereza</t>
-  </si>
-  <si>
-    <t>Rojo</t>
-  </si>
-  <si>
-    <t>Verde Pino</t>
-  </si>
-  <si>
     <t>TOTAL VELA</t>
   </si>
   <si>
@@ -234,130 +361,16 @@
     <t>lote chico</t>
   </si>
   <si>
-    <t>SHORT PLAYA CAB — DISTRIBUCIÓN POR TIENDA Y TALLA</t>
-  </si>
-  <si>
-    <t>★ LA VELA = 400 und mín · resto tiendas por peso ventas</t>
-  </si>
-  <si>
-    <t>Tienda</t>
-  </si>
-  <si>
-    <t>GRIETA</t>
-  </si>
-  <si>
-    <t>LA VELA ★</t>
-  </si>
-  <si>
-    <t>SAMBIL CHACAO</t>
-  </si>
-  <si>
-    <t>SAMBIL VALENCIA</t>
-  </si>
-  <si>
-    <t>CERRO VERDE</t>
-  </si>
-  <si>
-    <t>GRAND PLAZ</t>
-  </si>
-  <si>
-    <t>TOLON ★</t>
-  </si>
-  <si>
-    <t>SHORT PLAYA CAB — TELA EXISTENTE A AGOTAR (100%)</t>
-  </si>
-  <si>
-    <t>Consumo: 0.75 m/pieza · Habano/Azul Verdoso/Azul Pizzarra al 90% · ≤50 und → S10 M24 L30 XL16 2XL20</t>
-  </si>
-  <si>
-    <t>Producto</t>
-  </si>
-  <si>
-    <t>% Tela</t>
-  </si>
-  <si>
-    <t>Mts stock</t>
-  </si>
-  <si>
-    <t>Mts usados</t>
-  </si>
-  <si>
-    <t>Und Mín</t>
-  </si>
-  <si>
-    <t>Und Máx</t>
-  </si>
-  <si>
-    <t>Mts prod Mín</t>
-  </si>
-  <si>
-    <t>Mts prod Máx</t>
-  </si>
-  <si>
-    <t>Notas</t>
-  </si>
-  <si>
-    <t>Short Playa · Marron</t>
-  </si>
-  <si>
-    <t>90%</t>
-  </si>
-  <si>
-    <t>Curva global ventas · Tela HABANO</t>
-  </si>
-  <si>
-    <t>Short Playa · Azul Verdoso</t>
-  </si>
-  <si>
-    <t>Curva global ventas</t>
-  </si>
-  <si>
-    <t>Short Playa · Azul Pizarra</t>
-  </si>
-  <si>
-    <t>Curva global ventas · Tela AZUL PIZZARRA</t>
-  </si>
-  <si>
-    <t>Short Playa · Verde Pino</t>
-  </si>
-  <si>
-    <t>100%</t>
-  </si>
-  <si>
-    <t>Short Playa · Cereza</t>
-  </si>
-  <si>
-    <t>Curva global ventas · Tela ROJO</t>
-  </si>
-  <si>
-    <t>Verde Oliva</t>
-  </si>
-  <si>
-    <t>Short Playa · Verde Oliva</t>
-  </si>
-  <si>
-    <t>Curva global ventas · Lote chico → todas las tallas</t>
-  </si>
-  <si>
-    <t>Gris Azulado</t>
-  </si>
-  <si>
-    <t>Short Playa · Gris Azulado</t>
-  </si>
-  <si>
-    <t>Azul Marino</t>
-  </si>
-  <si>
-    <t>Short Playa · Azul Marino</t>
-  </si>
-  <si>
-    <t>Aguamarina</t>
-  </si>
-  <si>
-    <t>Short Playa · Aguamarina</t>
-  </si>
-  <si>
-    <t>Resumen tela stock vs usada:</t>
+    <t>SHORT PLAYA CAB — PRODUCCIÓN SATÉLITE (841 und)</t>
+  </si>
+  <si>
+    <t>Global 941 und − VELA prioritario 100 und = 841 und · resto tiendas (GRIETA, SAMBIL, CERRO VERDE, GRAND PLAZ, TOLON)</t>
+  </si>
+  <si>
+    <t>TOTAL SATÉLITE</t>
+  </si>
+  <si>
+    <t>Resta VELA</t>
   </si>
 </sst>
 </file>
@@ -2659,644 +2672,383 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:12">
       <c r="A2" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:12">
       <c r="A4" s="4" t="s">
         <v>55</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C4" s="4" t="s">
         <v>5</v>
       </c>
+      <c r="C4" s="4"/>
       <c r="D4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="4"/>
+      <c r="F4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="G4" s="4"/>
+      <c r="H4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="I4" s="4"/>
+      <c r="J4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="K4" s="4"/>
+      <c r="L4" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="L5" s="4"/>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6">
+        <v>16</v>
+      </c>
+      <c r="C6">
+        <v>17</v>
+      </c>
+      <c r="D6">
+        <v>33</v>
+      </c>
+      <c r="E6">
+        <v>35</v>
+      </c>
+      <c r="F6">
+        <v>42</v>
+      </c>
+      <c r="G6">
+        <v>45</v>
+      </c>
+      <c r="H6">
+        <v>23</v>
+      </c>
+      <c r="I6">
+        <v>25</v>
+      </c>
+      <c r="J6">
+        <v>17</v>
+      </c>
+      <c r="K6">
+        <v>18</v>
+      </c>
+      <c r="L6">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" t="s">
+      <c r="B7">
+        <v>48</v>
+      </c>
+      <c r="C7">
+        <v>51</v>
+      </c>
+      <c r="D7">
+        <v>100</v>
+      </c>
+      <c r="E7">
+        <v>106</v>
+      </c>
+      <c r="F7">
+        <v>128</v>
+      </c>
+      <c r="G7">
+        <v>136</v>
+      </c>
+      <c r="H7">
+        <v>72</v>
+      </c>
+      <c r="I7">
+        <v>76</v>
+      </c>
+      <c r="J7">
+        <v>52</v>
+      </c>
+      <c r="K7">
+        <v>55</v>
+      </c>
+      <c r="L7">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" t="s">
         <v>58</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B8">
+        <v>15</v>
+      </c>
+      <c r="C8">
+        <v>16</v>
+      </c>
+      <c r="D8">
+        <v>32</v>
+      </c>
+      <c r="E8">
+        <v>34</v>
+      </c>
+      <c r="F8">
+        <v>41</v>
+      </c>
+      <c r="G8">
+        <v>44</v>
+      </c>
+      <c r="H8">
+        <v>23</v>
+      </c>
+      <c r="I8">
+        <v>25</v>
+      </c>
+      <c r="J8">
+        <v>17</v>
+      </c>
+      <c r="K8">
+        <v>18</v>
+      </c>
+      <c r="L8">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" t="s">
         <v>59</v>
       </c>
-      <c r="C5">
+      <c r="B9">
+        <v>15</v>
+      </c>
+      <c r="C9">
+        <v>16</v>
+      </c>
+      <c r="D9">
+        <v>30</v>
+      </c>
+      <c r="E9">
+        <v>32</v>
+      </c>
+      <c r="F9">
+        <v>39</v>
+      </c>
+      <c r="G9">
+        <v>42</v>
+      </c>
+      <c r="H9">
+        <v>22</v>
+      </c>
+      <c r="I9">
+        <v>23</v>
+      </c>
+      <c r="J9">
+        <v>16</v>
+      </c>
+      <c r="K9">
+        <v>17</v>
+      </c>
+      <c r="L9">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10">
+        <v>15</v>
+      </c>
+      <c r="C10">
+        <v>16</v>
+      </c>
+      <c r="D10">
+        <v>30</v>
+      </c>
+      <c r="E10">
+        <v>33</v>
+      </c>
+      <c r="F10">
+        <v>39</v>
+      </c>
+      <c r="G10">
+        <v>42</v>
+      </c>
+      <c r="H10">
+        <v>22</v>
+      </c>
+      <c r="I10">
+        <v>23</v>
+      </c>
+      <c r="J10">
+        <v>16</v>
+      </c>
+      <c r="K10">
+        <v>17</v>
+      </c>
+      <c r="L10">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11">
         <v>2</v>
       </c>
-      <c r="D5">
+      <c r="C11">
+        <v>2</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>3</v>
+      </c>
+      <c r="F11">
+        <v>4</v>
+      </c>
+      <c r="G11">
+        <v>4</v>
+      </c>
+      <c r="H11">
+        <v>2</v>
+      </c>
+      <c r="I11">
+        <v>3</v>
+      </c>
+      <c r="J11">
+        <v>2</v>
+      </c>
+      <c r="K11">
+        <v>2</v>
+      </c>
+      <c r="L11">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="D12">
+        <v>6</v>
+      </c>
+      <c r="E12">
+        <v>7</v>
+      </c>
+      <c r="F12">
+        <v>8</v>
+      </c>
+      <c r="G12">
+        <v>8</v>
+      </c>
+      <c r="H12">
         <v>5</v>
       </c>
-      <c r="E5">
-        <v>6</v>
-      </c>
-      <c r="F5">
-        <v>4</v>
-      </c>
-      <c r="G5">
-        <v>4</v>
-      </c>
-      <c r="H5">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C6">
-        <v>2</v>
-      </c>
-      <c r="D6">
+      <c r="I12">
         <v>5</v>
       </c>
-      <c r="E6">
-        <v>6</v>
-      </c>
-      <c r="F6">
+      <c r="J12">
         <v>3</v>
       </c>
-      <c r="G6">
-        <v>4</v>
-      </c>
-      <c r="H6">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" t="s">
-        <v>62</v>
-      </c>
-      <c r="B7" t="s">
-        <v>62</v>
-      </c>
-      <c r="C7">
-        <v>2</v>
-      </c>
-      <c r="D7">
-        <v>5</v>
-      </c>
-      <c r="E7">
-        <v>6</v>
-      </c>
-      <c r="F7">
+      <c r="K12">
         <v>3</v>
       </c>
-      <c r="G7">
-        <v>4</v>
-      </c>
-      <c r="H7">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" t="s">
-        <v>63</v>
-      </c>
-      <c r="B8" t="s">
-        <v>64</v>
-      </c>
-      <c r="C8">
-        <v>2</v>
-      </c>
-      <c r="D8">
-        <v>5</v>
-      </c>
-      <c r="E8">
-        <v>6</v>
-      </c>
-      <c r="F8">
-        <v>3</v>
-      </c>
-      <c r="G8">
-        <v>4</v>
-      </c>
-      <c r="H8">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" t="s">
-        <v>65</v>
-      </c>
-      <c r="B9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C9">
-        <v>2</v>
-      </c>
-      <c r="D9">
-        <v>4</v>
-      </c>
-      <c r="E9">
-        <v>6</v>
-      </c>
-      <c r="F9">
-        <v>3</v>
-      </c>
-      <c r="G9">
-        <v>4</v>
-      </c>
-      <c r="H9">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3">
-        <v>10</v>
-      </c>
-      <c r="D10" s="3">
-        <v>24</v>
-      </c>
-      <c r="E10" s="3">
-        <v>30</v>
-      </c>
-      <c r="F10" s="3">
-        <v>16</v>
-      </c>
-      <c r="G10" s="3">
-        <v>20</v>
-      </c>
-      <c r="H10" s="3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="A14" t="s">
-        <v>58</v>
-      </c>
-      <c r="B14" t="s">
-        <v>59</v>
-      </c>
-      <c r="C14" t="s">
-        <v>9</v>
-      </c>
-      <c r="D14">
-        <v>4</v>
-      </c>
-      <c r="E14" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
-      <c r="A15" t="s">
-        <v>58</v>
-      </c>
-      <c r="B15" t="s">
-        <v>59</v>
-      </c>
-      <c r="C15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15">
-        <v>6</v>
-      </c>
-      <c r="E15" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
-      <c r="A16" t="s">
-        <v>58</v>
-      </c>
-      <c r="B16" t="s">
-        <v>59</v>
-      </c>
-      <c r="C16" t="s">
-        <v>6</v>
-      </c>
-      <c r="D16">
-        <v>5</v>
-      </c>
-      <c r="E16" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="A17" t="s">
-        <v>58</v>
-      </c>
-      <c r="B17" t="s">
-        <v>59</v>
-      </c>
-      <c r="C17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D17">
-        <v>2</v>
-      </c>
-      <c r="E17" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" t="s">
-        <v>58</v>
-      </c>
-      <c r="B18" t="s">
-        <v>59</v>
-      </c>
-      <c r="C18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18">
-        <v>4</v>
-      </c>
-      <c r="E18" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" t="s">
-        <v>62</v>
-      </c>
-      <c r="B19" t="s">
-        <v>62</v>
-      </c>
-      <c r="C19" t="s">
-        <v>9</v>
-      </c>
-      <c r="D19">
-        <v>4</v>
-      </c>
-      <c r="E19" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" t="s">
-        <v>62</v>
-      </c>
-      <c r="B20" t="s">
-        <v>62</v>
-      </c>
-      <c r="C20" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20">
-        <v>6</v>
-      </c>
-      <c r="E20" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5">
-      <c r="A21" t="s">
-        <v>62</v>
-      </c>
-      <c r="B21" t="s">
-        <v>62</v>
-      </c>
-      <c r="C21" t="s">
-        <v>6</v>
-      </c>
-      <c r="D21">
-        <v>5</v>
-      </c>
-      <c r="E21" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22" t="s">
-        <v>62</v>
-      </c>
-      <c r="B22" t="s">
-        <v>62</v>
-      </c>
-      <c r="C22" t="s">
-        <v>5</v>
-      </c>
-      <c r="D22">
-        <v>2</v>
-      </c>
-      <c r="E22" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5">
-      <c r="A23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B23" t="s">
-        <v>62</v>
-      </c>
-      <c r="C23" t="s">
-        <v>8</v>
-      </c>
-      <c r="D23">
-        <v>3</v>
-      </c>
-      <c r="E23" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="A24" t="s">
-        <v>63</v>
-      </c>
-      <c r="B24" t="s">
-        <v>64</v>
-      </c>
-      <c r="C24" t="s">
-        <v>9</v>
-      </c>
-      <c r="D24">
-        <v>4</v>
-      </c>
-      <c r="E24" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5">
-      <c r="A25" t="s">
-        <v>63</v>
-      </c>
-      <c r="B25" t="s">
-        <v>64</v>
-      </c>
-      <c r="C25" t="s">
-        <v>7</v>
-      </c>
-      <c r="D25">
-        <v>6</v>
-      </c>
-      <c r="E25" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="A26" t="s">
-        <v>63</v>
-      </c>
-      <c r="B26" t="s">
-        <v>64</v>
-      </c>
-      <c r="C26" t="s">
-        <v>6</v>
-      </c>
-      <c r="D26">
-        <v>5</v>
-      </c>
-      <c r="E26" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="A27" t="s">
-        <v>63</v>
-      </c>
-      <c r="B27" t="s">
-        <v>64</v>
-      </c>
-      <c r="C27" t="s">
-        <v>5</v>
-      </c>
-      <c r="D27">
-        <v>2</v>
-      </c>
-      <c r="E27" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5">
-      <c r="A28" t="s">
-        <v>63</v>
-      </c>
-      <c r="B28" t="s">
-        <v>64</v>
-      </c>
-      <c r="C28" t="s">
-        <v>8</v>
-      </c>
-      <c r="D28">
-        <v>3</v>
-      </c>
-      <c r="E28" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5">
-      <c r="A29" t="s">
-        <v>60</v>
-      </c>
-      <c r="B29" t="s">
-        <v>61</v>
-      </c>
-      <c r="C29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D29">
-        <v>4</v>
-      </c>
-      <c r="E29" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5">
-      <c r="A30" t="s">
-        <v>60</v>
-      </c>
-      <c r="B30" t="s">
-        <v>61</v>
-      </c>
-      <c r="C30" t="s">
-        <v>7</v>
-      </c>
-      <c r="D30">
-        <v>6</v>
-      </c>
-      <c r="E30" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5">
-      <c r="A31" t="s">
-        <v>60</v>
-      </c>
-      <c r="B31" t="s">
-        <v>61</v>
-      </c>
-      <c r="C31" t="s">
-        <v>6</v>
-      </c>
-      <c r="D31">
-        <v>5</v>
-      </c>
-      <c r="E31" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5">
-      <c r="A32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B32" t="s">
-        <v>61</v>
-      </c>
-      <c r="C32" t="s">
-        <v>5</v>
-      </c>
-      <c r="D32">
-        <v>2</v>
-      </c>
-      <c r="E32" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5">
-      <c r="A33" t="s">
-        <v>60</v>
-      </c>
-      <c r="B33" t="s">
-        <v>61</v>
-      </c>
-      <c r="C33" t="s">
-        <v>8</v>
-      </c>
-      <c r="D33">
-        <v>3</v>
-      </c>
-      <c r="E33" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5">
-      <c r="A34" t="s">
-        <v>65</v>
-      </c>
-      <c r="B34" t="s">
-        <v>65</v>
-      </c>
-      <c r="C34" t="s">
-        <v>9</v>
-      </c>
-      <c r="D34">
-        <v>4</v>
-      </c>
-      <c r="E34" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5">
-      <c r="A35" t="s">
-        <v>65</v>
-      </c>
-      <c r="B35" t="s">
-        <v>65</v>
-      </c>
-      <c r="C35" t="s">
-        <v>7</v>
-      </c>
-      <c r="D35">
-        <v>6</v>
-      </c>
-      <c r="E35" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5">
-      <c r="A36" t="s">
-        <v>65</v>
-      </c>
-      <c r="B36" t="s">
-        <v>65</v>
-      </c>
-      <c r="C36" t="s">
-        <v>6</v>
-      </c>
-      <c r="D36">
-        <v>4</v>
-      </c>
-      <c r="E36" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5">
-      <c r="A37" t="s">
-        <v>65</v>
-      </c>
-      <c r="B37" t="s">
-        <v>65</v>
-      </c>
-      <c r="C37" t="s">
-        <v>5</v>
-      </c>
-      <c r="D37">
-        <v>2</v>
-      </c>
-      <c r="E37" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5">
-      <c r="A38" t="s">
-        <v>65</v>
-      </c>
-      <c r="B38" t="s">
-        <v>65</v>
-      </c>
-      <c r="C38" t="s">
-        <v>8</v>
-      </c>
-      <c r="D38">
-        <v>3</v>
-      </c>
-      <c r="E38" t="s">
-        <v>70</v>
+      <c r="L12">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="3">
+        <v>114</v>
+      </c>
+      <c r="C13" s="3">
+        <v>117</v>
+      </c>
+      <c r="D13" s="3">
+        <v>234</v>
+      </c>
+      <c r="E13" s="3">
+        <v>250</v>
+      </c>
+      <c r="F13" s="3">
+        <v>301</v>
+      </c>
+      <c r="G13" s="3">
+        <v>318</v>
+      </c>
+      <c r="H13" s="3">
+        <v>169</v>
+      </c>
+      <c r="I13" s="3">
+        <v>178</v>
+      </c>
+      <c r="J13" s="3">
+        <v>123</v>
+      </c>
+      <c r="K13" s="3">
+        <v>139</v>
+      </c>
+      <c r="L13" s="3">
+        <v>941</v>
       </c>
     </row>
   </sheetData>
@@ -3306,383 +3058,544 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="2" spans="1:12">
-      <c r="A2" s="2" t="s">
+      <c r="H4" s="4" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="4" spans="1:12">
-      <c r="A4" s="4" t="s">
+      <c r="I4" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="I4" s="4"/>
       <c r="J4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="L5" s="4"/>
-    </row>
-    <row r="6" spans="1:12">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C5" t="s">
+        <v>77</v>
+      </c>
+      <c r="D5">
+        <v>200.83</v>
+      </c>
+      <c r="E5">
+        <v>180.75</v>
+      </c>
+      <c r="F5">
+        <v>240</v>
+      </c>
+      <c r="G5">
+        <v>255</v>
+      </c>
+      <c r="H5">
+        <v>180</v>
+      </c>
+      <c r="I5">
+        <v>191.25</v>
+      </c>
+      <c r="J5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>74</v>
-      </c>
-      <c r="B6">
+        <v>79</v>
+      </c>
+      <c r="B6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D6">
+        <v>163.94</v>
+      </c>
+      <c r="E6">
+        <v>147.55</v>
+      </c>
+      <c r="F6">
+        <v>196</v>
+      </c>
+      <c r="G6">
+        <v>208</v>
+      </c>
+      <c r="H6">
+        <v>147</v>
+      </c>
+      <c r="I6">
+        <v>156</v>
+      </c>
+      <c r="J6" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7">
+        <v>163.3</v>
+      </c>
+      <c r="E7">
+        <v>146.97</v>
+      </c>
+      <c r="F7">
+        <v>195</v>
+      </c>
+      <c r="G7">
+        <v>207</v>
+      </c>
+      <c r="H7">
+        <v>146.25</v>
+      </c>
+      <c r="I7">
+        <v>155.25</v>
+      </c>
+      <c r="J7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B8" t="s">
+        <v>86</v>
+      </c>
+      <c r="C8" t="s">
+        <v>87</v>
+      </c>
+      <c r="D8">
+        <v>76.33</v>
+      </c>
+      <c r="E8">
+        <v>76.33</v>
+      </c>
+      <c r="F8">
+        <v>101</v>
+      </c>
+      <c r="G8">
+        <v>108</v>
+      </c>
+      <c r="H8">
+        <v>75.75</v>
+      </c>
+      <c r="I8">
+        <v>81</v>
+      </c>
+      <c r="J8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" t="s">
+        <v>88</v>
+      </c>
+      <c r="B9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C9" t="s">
+        <v>87</v>
+      </c>
+      <c r="D9">
+        <v>65</v>
+      </c>
+      <c r="E9">
+        <v>65</v>
+      </c>
+      <c r="F9">
+        <v>86</v>
+      </c>
+      <c r="G9">
+        <v>92</v>
+      </c>
+      <c r="H9">
+        <v>64.5</v>
+      </c>
+      <c r="I9">
+        <v>69</v>
+      </c>
+      <c r="J9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" t="s">
+        <v>87</v>
+      </c>
+      <c r="D10">
+        <v>29.13</v>
+      </c>
+      <c r="E10">
+        <v>29.13</v>
+      </c>
+      <c r="F10">
+        <v>38</v>
+      </c>
+      <c r="G10">
+        <v>41</v>
+      </c>
+      <c r="H10">
+        <v>28.5</v>
+      </c>
+      <c r="I10">
+        <v>30.75</v>
+      </c>
+      <c r="J10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" t="s">
+        <v>95</v>
+      </c>
+      <c r="C11" t="s">
+        <v>87</v>
+      </c>
+      <c r="D11">
+        <v>28.67</v>
+      </c>
+      <c r="E11">
+        <v>28.67</v>
+      </c>
+      <c r="F11">
+        <v>38</v>
+      </c>
+      <c r="G11">
+        <v>41</v>
+      </c>
+      <c r="H11">
+        <v>28.5</v>
+      </c>
+      <c r="I11">
+        <v>30.75</v>
+      </c>
+      <c r="J11" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="A12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" t="s">
+        <v>97</v>
+      </c>
+      <c r="C12" t="s">
+        <v>87</v>
+      </c>
+      <c r="D12">
+        <v>24.25</v>
+      </c>
+      <c r="E12">
+        <v>24.25</v>
+      </c>
+      <c r="F12">
+        <v>32</v>
+      </c>
+      <c r="G12">
+        <v>34</v>
+      </c>
+      <c r="H12">
+        <v>24</v>
+      </c>
+      <c r="I12">
+        <v>25.5</v>
+      </c>
+      <c r="J12" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="A13" t="s">
+        <v>98</v>
+      </c>
+      <c r="B13" t="s">
+        <v>99</v>
+      </c>
+      <c r="C13" t="s">
+        <v>87</v>
+      </c>
+      <c r="D13">
+        <v>11.5</v>
+      </c>
+      <c r="E13">
+        <v>11.5</v>
+      </c>
+      <c r="F13">
+        <v>15</v>
+      </c>
+      <c r="G13">
         <v>16</v>
       </c>
-      <c r="C6">
-        <v>17</v>
-      </c>
-      <c r="D6">
-        <v>33</v>
-      </c>
-      <c r="E6">
+      <c r="H13">
+        <v>11.25</v>
+      </c>
+      <c r="I13">
+        <v>12</v>
+      </c>
+      <c r="J13" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="A14" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="F6">
-        <v>42</v>
-      </c>
-      <c r="G6">
-        <v>45</v>
-      </c>
-      <c r="H6">
-        <v>23</v>
-      </c>
-      <c r="I6">
-        <v>25</v>
-      </c>
-      <c r="J6">
-        <v>17</v>
-      </c>
-      <c r="K6">
-        <v>18</v>
-      </c>
-      <c r="L6">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
-      <c r="A7" t="s">
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3">
+        <v>941</v>
+      </c>
+      <c r="G14" s="3">
+        <v>1002</v>
+      </c>
+      <c r="H14" s="3">
+        <v>705.75</v>
+      </c>
+      <c r="I14" s="3">
+        <v>751.5</v>
+      </c>
+      <c r="J14" s="3"/>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" t="s">
         <v>75</v>
       </c>
-      <c r="B7">
-        <v>48</v>
-      </c>
-      <c r="C7">
-        <v>51</v>
-      </c>
-      <c r="D7">
-        <v>100</v>
-      </c>
-      <c r="E7">
-        <v>106</v>
-      </c>
-      <c r="F7">
-        <v>128</v>
-      </c>
-      <c r="G7">
-        <v>136</v>
-      </c>
-      <c r="H7">
-        <v>72</v>
-      </c>
-      <c r="I7">
-        <v>76</v>
-      </c>
-      <c r="J7">
-        <v>52</v>
-      </c>
-      <c r="K7">
-        <v>55</v>
-      </c>
-      <c r="L7">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
-      <c r="A8" t="s">
-        <v>76</v>
-      </c>
-      <c r="B8">
+      <c r="B18" t="s">
+        <v>101</v>
+      </c>
+      <c r="C18" t="s">
+        <v>77</v>
+      </c>
+      <c r="D18">
+        <v>200.83</v>
+      </c>
+      <c r="E18">
+        <v>180.75</v>
+      </c>
+      <c r="F18">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" t="s">
+        <v>79</v>
+      </c>
+      <c r="B19" t="s">
+        <v>79</v>
+      </c>
+      <c r="C19" t="s">
+        <v>77</v>
+      </c>
+      <c r="D19">
+        <v>163.94</v>
+      </c>
+      <c r="E19">
+        <v>147.55</v>
+      </c>
+      <c r="F19">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" t="s">
+        <v>82</v>
+      </c>
+      <c r="B20" t="s">
+        <v>102</v>
+      </c>
+      <c r="C20" t="s">
+        <v>77</v>
+      </c>
+      <c r="D20">
+        <v>163.3</v>
+      </c>
+      <c r="E20">
+        <v>146.97</v>
+      </c>
+      <c r="F20">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" t="s">
+        <v>85</v>
+      </c>
+      <c r="B21" t="s">
+        <v>85</v>
+      </c>
+      <c r="C21" t="s">
+        <v>87</v>
+      </c>
+      <c r="D21">
+        <v>76.33</v>
+      </c>
+      <c r="E21">
+        <v>76.33</v>
+      </c>
+      <c r="F21">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" t="s">
+        <v>88</v>
+      </c>
+      <c r="B22" t="s">
+        <v>103</v>
+      </c>
+      <c r="C22" t="s">
+        <v>87</v>
+      </c>
+      <c r="D22">
+        <v>65</v>
+      </c>
+      <c r="E22">
+        <v>65</v>
+      </c>
+      <c r="F22">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" t="s">
+        <v>91</v>
+      </c>
+      <c r="B23" t="s">
+        <v>91</v>
+      </c>
+      <c r="C23" t="s">
+        <v>87</v>
+      </c>
+      <c r="D23">
+        <v>29.13</v>
+      </c>
+      <c r="E23">
+        <v>29.13</v>
+      </c>
+      <c r="F23">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" t="s">
+        <v>94</v>
+      </c>
+      <c r="B24" t="s">
+        <v>94</v>
+      </c>
+      <c r="C24" t="s">
+        <v>87</v>
+      </c>
+      <c r="D24">
+        <v>28.67</v>
+      </c>
+      <c r="E24">
+        <v>28.67</v>
+      </c>
+      <c r="F24">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" t="s">
+        <v>96</v>
+      </c>
+      <c r="B25" t="s">
+        <v>96</v>
+      </c>
+      <c r="C25" t="s">
+        <v>87</v>
+      </c>
+      <c r="D25">
+        <v>24.25</v>
+      </c>
+      <c r="E25">
+        <v>24.25</v>
+      </c>
+      <c r="F25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" t="s">
+        <v>98</v>
+      </c>
+      <c r="B26" t="s">
+        <v>98</v>
+      </c>
+      <c r="C26" t="s">
+        <v>87</v>
+      </c>
+      <c r="D26">
+        <v>11.5</v>
+      </c>
+      <c r="E26">
+        <v>11.5</v>
+      </c>
+      <c r="F26">
         <v>15</v>
-      </c>
-      <c r="C8">
-        <v>16</v>
-      </c>
-      <c r="D8">
-        <v>32</v>
-      </c>
-      <c r="E8">
-        <v>34</v>
-      </c>
-      <c r="F8">
-        <v>41</v>
-      </c>
-      <c r="G8">
-        <v>44</v>
-      </c>
-      <c r="H8">
-        <v>23</v>
-      </c>
-      <c r="I8">
-        <v>25</v>
-      </c>
-      <c r="J8">
-        <v>17</v>
-      </c>
-      <c r="K8">
-        <v>18</v>
-      </c>
-      <c r="L8">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
-      <c r="A9" t="s">
-        <v>77</v>
-      </c>
-      <c r="B9">
-        <v>15</v>
-      </c>
-      <c r="C9">
-        <v>16</v>
-      </c>
-      <c r="D9">
-        <v>30</v>
-      </c>
-      <c r="E9">
-        <v>32</v>
-      </c>
-      <c r="F9">
-        <v>39</v>
-      </c>
-      <c r="G9">
-        <v>42</v>
-      </c>
-      <c r="H9">
-        <v>22</v>
-      </c>
-      <c r="I9">
-        <v>23</v>
-      </c>
-      <c r="J9">
-        <v>16</v>
-      </c>
-      <c r="K9">
-        <v>17</v>
-      </c>
-      <c r="L9">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
-      <c r="A10" t="s">
-        <v>78</v>
-      </c>
-      <c r="B10">
-        <v>15</v>
-      </c>
-      <c r="C10">
-        <v>16</v>
-      </c>
-      <c r="D10">
-        <v>30</v>
-      </c>
-      <c r="E10">
-        <v>33</v>
-      </c>
-      <c r="F10">
-        <v>39</v>
-      </c>
-      <c r="G10">
-        <v>42</v>
-      </c>
-      <c r="H10">
-        <v>22</v>
-      </c>
-      <c r="I10">
-        <v>23</v>
-      </c>
-      <c r="J10">
-        <v>16</v>
-      </c>
-      <c r="K10">
-        <v>17</v>
-      </c>
-      <c r="L10">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12">
-      <c r="A11" t="s">
-        <v>79</v>
-      </c>
-      <c r="B11">
-        <v>2</v>
-      </c>
-      <c r="C11">
-        <v>2</v>
-      </c>
-      <c r="D11">
-        <v>3</v>
-      </c>
-      <c r="E11">
-        <v>3</v>
-      </c>
-      <c r="F11">
-        <v>4</v>
-      </c>
-      <c r="G11">
-        <v>4</v>
-      </c>
-      <c r="H11">
-        <v>2</v>
-      </c>
-      <c r="I11">
-        <v>3</v>
-      </c>
-      <c r="J11">
-        <v>2</v>
-      </c>
-      <c r="K11">
-        <v>2</v>
-      </c>
-      <c r="L11">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12">
-      <c r="A12" t="s">
-        <v>80</v>
-      </c>
-      <c r="B12">
-        <v>3</v>
-      </c>
-      <c r="C12">
-        <v>3</v>
-      </c>
-      <c r="D12">
-        <v>6</v>
-      </c>
-      <c r="E12">
-        <v>7</v>
-      </c>
-      <c r="F12">
-        <v>8</v>
-      </c>
-      <c r="G12">
-        <v>8</v>
-      </c>
-      <c r="H12">
-        <v>5</v>
-      </c>
-      <c r="I12">
-        <v>5</v>
-      </c>
-      <c r="J12">
-        <v>3</v>
-      </c>
-      <c r="K12">
-        <v>3</v>
-      </c>
-      <c r="L12">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12">
-      <c r="A13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="3">
-        <v>114</v>
-      </c>
-      <c r="C13" s="3">
-        <v>117</v>
-      </c>
-      <c r="D13" s="3">
-        <v>234</v>
-      </c>
-      <c r="E13" s="3">
-        <v>250</v>
-      </c>
-      <c r="F13" s="3">
-        <v>301</v>
-      </c>
-      <c r="G13" s="3">
-        <v>318</v>
-      </c>
-      <c r="H13" s="3">
-        <v>169</v>
-      </c>
-      <c r="I13" s="3">
-        <v>178</v>
-      </c>
-      <c r="J13" s="3">
-        <v>123</v>
-      </c>
-      <c r="K13" s="3">
-        <v>139</v>
-      </c>
-      <c r="L13" s="3">
-        <v>941</v>
       </c>
     </row>
   </sheetData>
@@ -3692,544 +3605,1798 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B5" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="4" spans="1:10">
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>6</v>
+      </c>
+      <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
+      <c r="H5">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>6</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+      <c r="G6">
+        <v>4</v>
+      </c>
+      <c r="H6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>5</v>
+      </c>
+      <c r="E7">
+        <v>6</v>
+      </c>
+      <c r="F7">
+        <v>3</v>
+      </c>
+      <c r="G7">
+        <v>4</v>
+      </c>
+      <c r="H7">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" t="s">
+        <v>88</v>
+      </c>
+      <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8">
+        <v>5</v>
+      </c>
+      <c r="E8">
+        <v>6</v>
+      </c>
+      <c r="F8">
+        <v>3</v>
+      </c>
+      <c r="G8">
+        <v>4</v>
+      </c>
+      <c r="H8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
+        <v>85</v>
+      </c>
+      <c r="B9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9">
+        <v>4</v>
+      </c>
+      <c r="E9">
+        <v>6</v>
+      </c>
+      <c r="F9">
+        <v>3</v>
+      </c>
+      <c r="G9">
+        <v>4</v>
+      </c>
+      <c r="H9">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3">
+        <v>10</v>
+      </c>
+      <c r="D10" s="3">
+        <v>24</v>
+      </c>
+      <c r="E10" s="3">
+        <v>30</v>
+      </c>
+      <c r="F10" s="3">
+        <v>16</v>
+      </c>
+      <c r="G10" s="3">
+        <v>20</v>
+      </c>
+      <c r="H10" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" t="s">
+        <v>102</v>
+      </c>
+      <c r="B14" t="s">
+        <v>82</v>
+      </c>
+      <c r="C14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14">
+        <v>4</v>
+      </c>
+      <c r="E14" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" t="s">
+        <v>102</v>
+      </c>
+      <c r="B15" t="s">
+        <v>82</v>
+      </c>
+      <c r="C15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15">
+        <v>6</v>
+      </c>
+      <c r="E15" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" t="s">
+        <v>102</v>
+      </c>
+      <c r="B16" t="s">
+        <v>82</v>
+      </c>
+      <c r="C16" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16">
+        <v>5</v>
+      </c>
+      <c r="E16" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" t="s">
+        <v>102</v>
+      </c>
+      <c r="B17" t="s">
+        <v>82</v>
+      </c>
+      <c r="C17" t="s">
+        <v>5</v>
+      </c>
+      <c r="D17">
+        <v>2</v>
+      </c>
+      <c r="E17" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" t="s">
+        <v>102</v>
+      </c>
+      <c r="B18" t="s">
+        <v>82</v>
+      </c>
+      <c r="C18" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18">
+        <v>4</v>
+      </c>
+      <c r="E18" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" t="s">
+        <v>79</v>
+      </c>
+      <c r="B19" t="s">
+        <v>79</v>
+      </c>
+      <c r="C19" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19">
+        <v>4</v>
+      </c>
+      <c r="E19" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" t="s">
+        <v>79</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>6</v>
+      </c>
+      <c r="E20" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" t="s">
+        <v>79</v>
+      </c>
+      <c r="B21" t="s">
+        <v>79</v>
+      </c>
+      <c r="C21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D21">
+        <v>5</v>
+      </c>
+      <c r="E21" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" t="s">
+        <v>79</v>
+      </c>
+      <c r="B22" t="s">
+        <v>79</v>
+      </c>
+      <c r="C22" t="s">
+        <v>5</v>
+      </c>
+      <c r="D22">
+        <v>2</v>
+      </c>
+      <c r="E22" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" t="s">
+        <v>79</v>
+      </c>
+      <c r="C23" t="s">
+        <v>8</v>
+      </c>
+      <c r="D23">
+        <v>3</v>
+      </c>
+      <c r="E23" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" t="s">
+        <v>103</v>
+      </c>
+      <c r="B24" t="s">
+        <v>88</v>
+      </c>
+      <c r="C24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D24">
+        <v>4</v>
+      </c>
+      <c r="E24" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" t="s">
+        <v>103</v>
+      </c>
+      <c r="B25" t="s">
+        <v>88</v>
+      </c>
+      <c r="C25" t="s">
+        <v>7</v>
+      </c>
+      <c r="D25">
+        <v>6</v>
+      </c>
+      <c r="E25" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" t="s">
+        <v>103</v>
+      </c>
+      <c r="B26" t="s">
+        <v>88</v>
+      </c>
+      <c r="C26" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26">
+        <v>5</v>
+      </c>
+      <c r="E26" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" t="s">
+        <v>103</v>
+      </c>
+      <c r="B27" t="s">
+        <v>88</v>
+      </c>
+      <c r="C27" t="s">
+        <v>5</v>
+      </c>
+      <c r="D27">
+        <v>2</v>
+      </c>
+      <c r="E27" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" t="s">
+        <v>103</v>
+      </c>
+      <c r="B28" t="s">
+        <v>88</v>
+      </c>
+      <c r="C28" t="s">
+        <v>8</v>
+      </c>
+      <c r="D28">
+        <v>3</v>
+      </c>
+      <c r="E28" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" t="s">
+        <v>101</v>
+      </c>
+      <c r="B29" t="s">
+        <v>75</v>
+      </c>
+      <c r="C29" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29">
+        <v>4</v>
+      </c>
+      <c r="E29" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" t="s">
+        <v>101</v>
+      </c>
+      <c r="B30" t="s">
+        <v>75</v>
+      </c>
+      <c r="C30" t="s">
+        <v>7</v>
+      </c>
+      <c r="D30">
+        <v>6</v>
+      </c>
+      <c r="E30" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" t="s">
+        <v>101</v>
+      </c>
+      <c r="B31" t="s">
+        <v>75</v>
+      </c>
+      <c r="C31" t="s">
+        <v>6</v>
+      </c>
+      <c r="D31">
+        <v>5</v>
+      </c>
+      <c r="E31" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" t="s">
+        <v>101</v>
+      </c>
+      <c r="B32" t="s">
+        <v>75</v>
+      </c>
+      <c r="C32" t="s">
+        <v>5</v>
+      </c>
+      <c r="D32">
+        <v>2</v>
+      </c>
+      <c r="E32" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" t="s">
+        <v>101</v>
+      </c>
+      <c r="B33" t="s">
+        <v>75</v>
+      </c>
+      <c r="C33" t="s">
+        <v>8</v>
+      </c>
+      <c r="D33">
+        <v>3</v>
+      </c>
+      <c r="E33" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" t="s">
+        <v>85</v>
+      </c>
+      <c r="B34" t="s">
+        <v>85</v>
+      </c>
+      <c r="C34" t="s">
+        <v>9</v>
+      </c>
+      <c r="D34">
+        <v>4</v>
+      </c>
+      <c r="E34" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" t="s">
+        <v>85</v>
+      </c>
+      <c r="B35" t="s">
+        <v>85</v>
+      </c>
+      <c r="C35" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35">
+        <v>6</v>
+      </c>
+      <c r="E35" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36" t="s">
+        <v>85</v>
+      </c>
+      <c r="B36" t="s">
+        <v>85</v>
+      </c>
+      <c r="C36" t="s">
+        <v>6</v>
+      </c>
+      <c r="D36">
+        <v>4</v>
+      </c>
+      <c r="E36" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" t="s">
+        <v>85</v>
+      </c>
+      <c r="B37" t="s">
+        <v>85</v>
+      </c>
+      <c r="C37" t="s">
+        <v>5</v>
+      </c>
+      <c r="D37">
+        <v>2</v>
+      </c>
+      <c r="E37" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38" t="s">
+        <v>85</v>
+      </c>
+      <c r="B38" t="s">
+        <v>85</v>
+      </c>
+      <c r="C38" t="s">
+        <v>8</v>
+      </c>
+      <c r="D38">
+        <v>3</v>
+      </c>
+      <c r="E38" t="s">
+        <v>112</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H62"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C5">
+        <v>26</v>
+      </c>
+      <c r="D5">
+        <v>55</v>
+      </c>
+      <c r="E5">
+        <v>70</v>
+      </c>
+      <c r="F5">
+        <v>40</v>
+      </c>
+      <c r="G5">
+        <v>29</v>
+      </c>
+      <c r="H5">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6">
+        <v>21</v>
+      </c>
+      <c r="D6">
+        <v>44</v>
+      </c>
+      <c r="E6">
         <v>56</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="F6">
+        <v>32</v>
+      </c>
+      <c r="G6">
+        <v>23</v>
+      </c>
+      <c r="H6">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B7" t="s">
+        <v>82</v>
+      </c>
+      <c r="C7">
+        <v>21</v>
+      </c>
+      <c r="D7">
+        <v>43</v>
+      </c>
+      <c r="E7">
+        <v>56</v>
+      </c>
+      <c r="F7">
+        <v>31</v>
+      </c>
+      <c r="G7">
+        <v>23</v>
+      </c>
+      <c r="H7">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
         <v>85</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G4" s="4" t="s">
+      <c r="B8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8">
+        <v>10</v>
+      </c>
+      <c r="D8">
+        <v>20</v>
+      </c>
+      <c r="E8">
+        <v>26</v>
+      </c>
+      <c r="F8">
+        <v>15</v>
+      </c>
+      <c r="G8">
+        <v>11</v>
+      </c>
+      <c r="H8">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
+        <v>103</v>
+      </c>
+      <c r="B9" t="s">
         <v>88</v>
       </c>
-      <c r="H4" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="J4" s="4" t="s">
+      <c r="C9">
+        <v>8</v>
+      </c>
+      <c r="D9">
+        <v>16</v>
+      </c>
+      <c r="E9">
+        <v>21</v>
+      </c>
+      <c r="F9">
+        <v>12</v>
+      </c>
+      <c r="G9">
+        <v>9</v>
+      </c>
+      <c r="H9">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="5" spans="1:10">
-      <c r="A5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" t="s">
-        <v>92</v>
-      </c>
-      <c r="C5" t="s">
-        <v>93</v>
-      </c>
-      <c r="D5">
-        <v>200.83</v>
-      </c>
-      <c r="E5">
-        <v>180.75</v>
-      </c>
-      <c r="F5">
-        <v>240</v>
-      </c>
-      <c r="G5">
-        <v>255</v>
-      </c>
-      <c r="H5">
-        <v>180</v>
-      </c>
-      <c r="I5">
-        <v>191.25</v>
-      </c>
-      <c r="J5" t="s">
+      <c r="B10" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10">
+        <v>4</v>
+      </c>
+      <c r="D10">
+        <v>9</v>
+      </c>
+      <c r="E10">
+        <v>11</v>
+      </c>
+      <c r="F10">
+        <v>6</v>
+      </c>
+      <c r="G10">
+        <v>8</v>
+      </c>
+      <c r="H10">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="6" spans="1:10">
-      <c r="A6" t="s">
-        <v>62</v>
-      </c>
-      <c r="B6" t="s">
-        <v>95</v>
-      </c>
-      <c r="C6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D6">
-        <v>163.94</v>
-      </c>
-      <c r="E6">
-        <v>147.55</v>
-      </c>
-      <c r="F6">
-        <v>196</v>
-      </c>
-      <c r="G6">
+      <c r="B11" t="s">
+        <v>94</v>
+      </c>
+      <c r="C11">
+        <v>4</v>
+      </c>
+      <c r="D11">
+        <v>9</v>
+      </c>
+      <c r="E11">
+        <v>11</v>
+      </c>
+      <c r="F11">
+        <v>6</v>
+      </c>
+      <c r="G11">
+        <v>8</v>
+      </c>
+      <c r="H11">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" t="s">
+        <v>96</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="D12">
+        <v>8</v>
+      </c>
+      <c r="E12">
+        <v>10</v>
+      </c>
+      <c r="F12">
+        <v>5</v>
+      </c>
+      <c r="G12">
+        <v>6</v>
+      </c>
+      <c r="H12">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" t="s">
+        <v>98</v>
+      </c>
+      <c r="B13" t="s">
+        <v>98</v>
+      </c>
+      <c r="C13">
+        <v>2</v>
+      </c>
+      <c r="D13">
+        <v>4</v>
+      </c>
+      <c r="E13">
+        <v>4</v>
+      </c>
+      <c r="F13">
+        <v>2</v>
+      </c>
+      <c r="G13">
+        <v>3</v>
+      </c>
+      <c r="H13">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3">
+        <v>99</v>
+      </c>
+      <c r="D14" s="3">
         <v>208</v>
       </c>
-      <c r="H6">
-        <v>147</v>
-      </c>
-      <c r="I6">
-        <v>156</v>
-      </c>
-      <c r="J6" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
-      <c r="A7" t="s">
-        <v>59</v>
-      </c>
-      <c r="B7" t="s">
-        <v>97</v>
-      </c>
-      <c r="C7" t="s">
-        <v>93</v>
-      </c>
-      <c r="D7">
-        <v>163.3</v>
-      </c>
-      <c r="E7">
-        <v>146.97</v>
-      </c>
-      <c r="F7">
-        <v>195</v>
-      </c>
-      <c r="G7">
-        <v>207</v>
-      </c>
-      <c r="H7">
-        <v>146.25</v>
-      </c>
-      <c r="I7">
-        <v>155.25</v>
-      </c>
-      <c r="J7" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
-      <c r="A8" t="s">
+      <c r="E14" s="3">
+        <v>265</v>
+      </c>
+      <c r="F14" s="3">
+        <v>149</v>
+      </c>
+      <c r="G14" s="3">
+        <v>120</v>
+      </c>
+      <c r="H14" s="3">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B8" t="s">
-        <v>99</v>
-      </c>
-      <c r="C8" t="s">
-        <v>100</v>
-      </c>
-      <c r="D8">
-        <v>76.33</v>
-      </c>
-      <c r="E8">
-        <v>76.33</v>
-      </c>
-      <c r="F8">
-        <v>101</v>
-      </c>
-      <c r="G8">
-        <v>108</v>
-      </c>
-      <c r="H8">
-        <v>75.75</v>
-      </c>
-      <c r="I8">
-        <v>81</v>
-      </c>
-      <c r="J8" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
-      <c r="A9" t="s">
-        <v>64</v>
-      </c>
-      <c r="B9" t="s">
-        <v>101</v>
-      </c>
-      <c r="C9" t="s">
-        <v>100</v>
-      </c>
-      <c r="D9">
-        <v>65</v>
-      </c>
-      <c r="E9">
-        <v>65</v>
-      </c>
-      <c r="F9">
-        <v>86</v>
-      </c>
-      <c r="G9">
-        <v>92</v>
-      </c>
-      <c r="H9">
-        <v>64.5</v>
-      </c>
-      <c r="I9">
-        <v>69</v>
-      </c>
-      <c r="J9" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
-      <c r="A10" t="s">
-        <v>103</v>
-      </c>
-      <c r="B10" t="s">
-        <v>104</v>
-      </c>
-      <c r="C10" t="s">
-        <v>100</v>
-      </c>
-      <c r="D10">
-        <v>29.13</v>
-      </c>
-      <c r="E10">
-        <v>29.13</v>
-      </c>
-      <c r="F10">
-        <v>38</v>
-      </c>
-      <c r="G10">
-        <v>41</v>
-      </c>
-      <c r="H10">
-        <v>28.5</v>
-      </c>
-      <c r="I10">
-        <v>30.75</v>
-      </c>
-      <c r="J10" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
-      <c r="A11" t="s">
-        <v>106</v>
-      </c>
-      <c r="B11" t="s">
-        <v>107</v>
-      </c>
-      <c r="C11" t="s">
-        <v>100</v>
-      </c>
-      <c r="D11">
-        <v>28.67</v>
-      </c>
-      <c r="E11">
-        <v>28.67</v>
-      </c>
-      <c r="F11">
-        <v>38</v>
-      </c>
-      <c r="G11">
-        <v>41</v>
-      </c>
-      <c r="H11">
-        <v>28.5</v>
-      </c>
-      <c r="I11">
-        <v>30.75</v>
-      </c>
-      <c r="J11" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
-      <c r="A12" t="s">
-        <v>108</v>
-      </c>
-      <c r="B12" t="s">
-        <v>109</v>
-      </c>
-      <c r="C12" t="s">
-        <v>100</v>
-      </c>
-      <c r="D12">
-        <v>24.25</v>
-      </c>
-      <c r="E12">
-        <v>24.25</v>
-      </c>
-      <c r="F12">
-        <v>32</v>
-      </c>
-      <c r="G12">
-        <v>34</v>
-      </c>
-      <c r="H12">
-        <v>24</v>
-      </c>
-      <c r="I12">
-        <v>25.5</v>
-      </c>
-      <c r="J12" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
-      <c r="A13" t="s">
+      <c r="C17" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="B13" t="s">
+      <c r="E17" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="F17" s="4" t="s">
         <v>111</v>
-      </c>
-      <c r="C13" t="s">
-        <v>100</v>
-      </c>
-      <c r="D13">
-        <v>11.5</v>
-      </c>
-      <c r="E13">
-        <v>11.5</v>
-      </c>
-      <c r="F13">
-        <v>15</v>
-      </c>
-      <c r="G13">
-        <v>16</v>
-      </c>
-      <c r="H13">
-        <v>11.25</v>
-      </c>
-      <c r="I13">
-        <v>12</v>
-      </c>
-      <c r="J13" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10">
-      <c r="A14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3">
-        <v>941</v>
-      </c>
-      <c r="G14" s="3">
-        <v>1002</v>
-      </c>
-      <c r="H14" s="3">
-        <v>705.75</v>
-      </c>
-      <c r="I14" s="3">
-        <v>751.5</v>
-      </c>
-      <c r="J14" s="3"/>
-    </row>
-    <row r="17" spans="1:6">
-      <c r="A17" s="3" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>61</v>
+        <v>101</v>
       </c>
       <c r="B18" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="C18" t="s">
-        <v>93</v>
+        <v>9</v>
       </c>
       <c r="D18">
-        <v>200.83</v>
+        <v>29</v>
       </c>
       <c r="E18">
-        <v>180.75</v>
-      </c>
-      <c r="F18">
-        <v>240</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>62</v>
+        <v>101</v>
       </c>
       <c r="B19" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="C19" t="s">
-        <v>93</v>
+        <v>7</v>
       </c>
       <c r="D19">
-        <v>163.94</v>
+        <v>70</v>
       </c>
       <c r="E19">
-        <v>147.55</v>
-      </c>
-      <c r="F19">
-        <v>196</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>59</v>
+        <v>101</v>
       </c>
       <c r="B20" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="C20" t="s">
-        <v>93</v>
+        <v>6</v>
       </c>
       <c r="D20">
-        <v>163.3</v>
+        <v>55</v>
       </c>
       <c r="E20">
-        <v>146.97</v>
-      </c>
-      <c r="F20">
-        <v>195</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>65</v>
+        <v>101</v>
       </c>
       <c r="B21" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="C21" t="s">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="D21">
-        <v>76.33</v>
+        <v>26</v>
       </c>
       <c r="E21">
-        <v>76.33</v>
-      </c>
-      <c r="F21">
-        <v>101</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
       <c r="B22" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="C22" t="s">
-        <v>100</v>
+        <v>8</v>
       </c>
       <c r="D22">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="E22">
-        <v>65</v>
-      </c>
-      <c r="F22">
-        <v>86</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>103</v>
+        <v>79</v>
       </c>
       <c r="B23" t="s">
-        <v>103</v>
+        <v>79</v>
       </c>
       <c r="C23" t="s">
-        <v>100</v>
+        <v>9</v>
       </c>
       <c r="D23">
-        <v>29.13</v>
+        <v>23</v>
       </c>
       <c r="E23">
-        <v>29.13</v>
-      </c>
-      <c r="F23">
-        <v>38</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="B24" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="C24" t="s">
-        <v>100</v>
+        <v>7</v>
       </c>
       <c r="D24">
-        <v>28.67</v>
+        <v>56</v>
       </c>
       <c r="E24">
-        <v>28.67</v>
-      </c>
-      <c r="F24">
-        <v>38</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>108</v>
+        <v>79</v>
       </c>
       <c r="B25" t="s">
-        <v>108</v>
+        <v>79</v>
       </c>
       <c r="C25" t="s">
-        <v>100</v>
+        <v>6</v>
       </c>
       <c r="D25">
-        <v>24.25</v>
+        <v>44</v>
       </c>
       <c r="E25">
-        <v>24.25</v>
-      </c>
-      <c r="F25">
-        <v>32</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="B26" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="C26" t="s">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="D26">
-        <v>11.5</v>
+        <v>21</v>
       </c>
       <c r="E26">
-        <v>11.5</v>
-      </c>
-      <c r="F26">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" t="s">
+        <v>79</v>
+      </c>
+      <c r="B27" t="s">
+        <v>79</v>
+      </c>
+      <c r="C27" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27">
+        <v>32</v>
+      </c>
+      <c r="E27">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" t="s">
+        <v>102</v>
+      </c>
+      <c r="B28" t="s">
+        <v>82</v>
+      </c>
+      <c r="C28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28">
+        <v>23</v>
+      </c>
+      <c r="E28">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" t="s">
+        <v>102</v>
+      </c>
+      <c r="B29" t="s">
+        <v>82</v>
+      </c>
+      <c r="C29" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29">
+        <v>56</v>
+      </c>
+      <c r="E29">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" t="s">
+        <v>102</v>
+      </c>
+      <c r="B30" t="s">
+        <v>82</v>
+      </c>
+      <c r="C30" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30">
+        <v>43</v>
+      </c>
+      <c r="E30">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" t="s">
+        <v>102</v>
+      </c>
+      <c r="B31" t="s">
+        <v>82</v>
+      </c>
+      <c r="C31" t="s">
+        <v>5</v>
+      </c>
+      <c r="D31">
+        <v>21</v>
+      </c>
+      <c r="E31">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" t="s">
+        <v>102</v>
+      </c>
+      <c r="B32" t="s">
+        <v>82</v>
+      </c>
+      <c r="C32" t="s">
+        <v>8</v>
+      </c>
+      <c r="D32">
+        <v>31</v>
+      </c>
+      <c r="E32">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" t="s">
+        <v>85</v>
+      </c>
+      <c r="B33" t="s">
+        <v>85</v>
+      </c>
+      <c r="C33" t="s">
+        <v>9</v>
+      </c>
+      <c r="D33">
+        <v>11</v>
+      </c>
+      <c r="E33">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" t="s">
+        <v>85</v>
+      </c>
+      <c r="B34" t="s">
+        <v>85</v>
+      </c>
+      <c r="C34" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34">
+        <v>26</v>
+      </c>
+      <c r="E34">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" t="s">
+        <v>85</v>
+      </c>
+      <c r="B35" t="s">
+        <v>85</v>
+      </c>
+      <c r="C35" t="s">
+        <v>6</v>
+      </c>
+      <c r="D35">
+        <v>20</v>
+      </c>
+      <c r="E35">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" t="s">
+        <v>85</v>
+      </c>
+      <c r="B36" t="s">
+        <v>85</v>
+      </c>
+      <c r="C36" t="s">
+        <v>5</v>
+      </c>
+      <c r="D36">
+        <v>10</v>
+      </c>
+      <c r="E36">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" t="s">
+        <v>85</v>
+      </c>
+      <c r="B37" t="s">
+        <v>85</v>
+      </c>
+      <c r="C37" t="s">
+        <v>8</v>
+      </c>
+      <c r="D37">
         <v>15</v>
+      </c>
+      <c r="E37">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" t="s">
+        <v>103</v>
+      </c>
+      <c r="B38" t="s">
+        <v>88</v>
+      </c>
+      <c r="C38" t="s">
+        <v>9</v>
+      </c>
+      <c r="D38">
+        <v>9</v>
+      </c>
+      <c r="E38">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" t="s">
+        <v>103</v>
+      </c>
+      <c r="B39" t="s">
+        <v>88</v>
+      </c>
+      <c r="C39" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39">
+        <v>21</v>
+      </c>
+      <c r="E39">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" t="s">
+        <v>103</v>
+      </c>
+      <c r="B40" t="s">
+        <v>88</v>
+      </c>
+      <c r="C40" t="s">
+        <v>6</v>
+      </c>
+      <c r="D40">
+        <v>16</v>
+      </c>
+      <c r="E40">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41" t="s">
+        <v>103</v>
+      </c>
+      <c r="B41" t="s">
+        <v>88</v>
+      </c>
+      <c r="C41" t="s">
+        <v>5</v>
+      </c>
+      <c r="D41">
+        <v>8</v>
+      </c>
+      <c r="E41">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" t="s">
+        <v>103</v>
+      </c>
+      <c r="B42" t="s">
+        <v>88</v>
+      </c>
+      <c r="C42" t="s">
+        <v>8</v>
+      </c>
+      <c r="D42">
+        <v>12</v>
+      </c>
+      <c r="E42">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" t="s">
+        <v>94</v>
+      </c>
+      <c r="B43" t="s">
+        <v>94</v>
+      </c>
+      <c r="C43" t="s">
+        <v>9</v>
+      </c>
+      <c r="D43">
+        <v>8</v>
+      </c>
+      <c r="E43">
+        <v>0</v>
+      </c>
+      <c r="F43" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44" t="s">
+        <v>94</v>
+      </c>
+      <c r="B44" t="s">
+        <v>94</v>
+      </c>
+      <c r="C44" t="s">
+        <v>7</v>
+      </c>
+      <c r="D44">
+        <v>11</v>
+      </c>
+      <c r="E44">
+        <v>0</v>
+      </c>
+      <c r="F44" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45" t="s">
+        <v>94</v>
+      </c>
+      <c r="B45" t="s">
+        <v>94</v>
+      </c>
+      <c r="C45" t="s">
+        <v>6</v>
+      </c>
+      <c r="D45">
+        <v>9</v>
+      </c>
+      <c r="E45">
+        <v>0</v>
+      </c>
+      <c r="F45" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46" t="s">
+        <v>94</v>
+      </c>
+      <c r="B46" t="s">
+        <v>94</v>
+      </c>
+      <c r="C46" t="s">
+        <v>5</v>
+      </c>
+      <c r="D46">
+        <v>4</v>
+      </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
+      <c r="F46" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
+      <c r="A47" t="s">
+        <v>94</v>
+      </c>
+      <c r="B47" t="s">
+        <v>94</v>
+      </c>
+      <c r="C47" t="s">
+        <v>8</v>
+      </c>
+      <c r="D47">
+        <v>6</v>
+      </c>
+      <c r="E47">
+        <v>0</v>
+      </c>
+      <c r="F47" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
+      <c r="A48" t="s">
+        <v>91</v>
+      </c>
+      <c r="B48" t="s">
+        <v>91</v>
+      </c>
+      <c r="C48" t="s">
+        <v>9</v>
+      </c>
+      <c r="D48">
+        <v>8</v>
+      </c>
+      <c r="E48">
+        <v>0</v>
+      </c>
+      <c r="F48" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49" t="s">
+        <v>91</v>
+      </c>
+      <c r="B49" t="s">
+        <v>91</v>
+      </c>
+      <c r="C49" t="s">
+        <v>7</v>
+      </c>
+      <c r="D49">
+        <v>11</v>
+      </c>
+      <c r="E49">
+        <v>0</v>
+      </c>
+      <c r="F49" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
+      <c r="A50" t="s">
+        <v>91</v>
+      </c>
+      <c r="B50" t="s">
+        <v>91</v>
+      </c>
+      <c r="C50" t="s">
+        <v>6</v>
+      </c>
+      <c r="D50">
+        <v>9</v>
+      </c>
+      <c r="E50">
+        <v>0</v>
+      </c>
+      <c r="F50" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51" t="s">
+        <v>91</v>
+      </c>
+      <c r="B51" t="s">
+        <v>91</v>
+      </c>
+      <c r="C51" t="s">
+        <v>5</v>
+      </c>
+      <c r="D51">
+        <v>4</v>
+      </c>
+      <c r="E51">
+        <v>0</v>
+      </c>
+      <c r="F51" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52" t="s">
+        <v>91</v>
+      </c>
+      <c r="B52" t="s">
+        <v>91</v>
+      </c>
+      <c r="C52" t="s">
+        <v>8</v>
+      </c>
+      <c r="D52">
+        <v>6</v>
+      </c>
+      <c r="E52">
+        <v>0</v>
+      </c>
+      <c r="F52" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="A53" t="s">
+        <v>96</v>
+      </c>
+      <c r="B53" t="s">
+        <v>96</v>
+      </c>
+      <c r="C53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D53">
+        <v>6</v>
+      </c>
+      <c r="E53">
+        <v>0</v>
+      </c>
+      <c r="F53" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54" t="s">
+        <v>96</v>
+      </c>
+      <c r="B54" t="s">
+        <v>96</v>
+      </c>
+      <c r="C54" t="s">
+        <v>7</v>
+      </c>
+      <c r="D54">
+        <v>10</v>
+      </c>
+      <c r="E54">
+        <v>0</v>
+      </c>
+      <c r="F54" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55" t="s">
+        <v>96</v>
+      </c>
+      <c r="B55" t="s">
+        <v>96</v>
+      </c>
+      <c r="C55" t="s">
+        <v>6</v>
+      </c>
+      <c r="D55">
+        <v>8</v>
+      </c>
+      <c r="E55">
+        <v>0</v>
+      </c>
+      <c r="F55" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
+      <c r="A56" t="s">
+        <v>96</v>
+      </c>
+      <c r="B56" t="s">
+        <v>96</v>
+      </c>
+      <c r="C56" t="s">
+        <v>5</v>
+      </c>
+      <c r="D56">
+        <v>3</v>
+      </c>
+      <c r="E56">
+        <v>0</v>
+      </c>
+      <c r="F56" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
+      <c r="A57" t="s">
+        <v>96</v>
+      </c>
+      <c r="B57" t="s">
+        <v>96</v>
+      </c>
+      <c r="C57" t="s">
+        <v>8</v>
+      </c>
+      <c r="D57">
+        <v>5</v>
+      </c>
+      <c r="E57">
+        <v>0</v>
+      </c>
+      <c r="F57" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
+      <c r="A58" t="s">
+        <v>98</v>
+      </c>
+      <c r="B58" t="s">
+        <v>98</v>
+      </c>
+      <c r="C58" t="s">
+        <v>9</v>
+      </c>
+      <c r="D58">
+        <v>3</v>
+      </c>
+      <c r="E58">
+        <v>0</v>
+      </c>
+      <c r="F58" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
+      <c r="A59" t="s">
+        <v>98</v>
+      </c>
+      <c r="B59" t="s">
+        <v>98</v>
+      </c>
+      <c r="C59" t="s">
+        <v>7</v>
+      </c>
+      <c r="D59">
+        <v>4</v>
+      </c>
+      <c r="E59">
+        <v>0</v>
+      </c>
+      <c r="F59" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
+      <c r="A60" t="s">
+        <v>98</v>
+      </c>
+      <c r="B60" t="s">
+        <v>98</v>
+      </c>
+      <c r="C60" t="s">
+        <v>6</v>
+      </c>
+      <c r="D60">
+        <v>4</v>
+      </c>
+      <c r="E60">
+        <v>0</v>
+      </c>
+      <c r="F60" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="A61" t="s">
+        <v>98</v>
+      </c>
+      <c r="B61" t="s">
+        <v>98</v>
+      </c>
+      <c r="C61" t="s">
+        <v>5</v>
+      </c>
+      <c r="D61">
+        <v>2</v>
+      </c>
+      <c r="E61">
+        <v>0</v>
+      </c>
+      <c r="F61" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
+      <c r="A62" t="s">
+        <v>98</v>
+      </c>
+      <c r="B62" t="s">
+        <v>98</v>
+      </c>
+      <c r="C62" t="s">
+        <v>8</v>
+      </c>
+      <c r="D62">
+        <v>2</v>
+      </c>
+      <c r="E62">
+        <v>0</v>
+      </c>
+      <c r="F62" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Show satellite production as min-max range like global plan
Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SHORT_PLAYA_CAB_Cantidades_Sugeridas_Proyecciones.xlsx
+++ b/SHORT_PLAYA_CAB_Cantidades_Sugeridas_Proyecciones.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="122">
   <si>
     <t>CANTIDADES POR COLORES</t>
   </si>
@@ -361,16 +361,31 @@
     <t>lote chico</t>
   </si>
   <si>
-    <t>SHORT PLAYA CAB — PRODUCCIÓN SATÉLITE (841 und)</t>
-  </si>
-  <si>
-    <t>Global 941 und − VELA prioritario 100 und = 841 und · resto tiendas (GRIETA, SAMBIL, CERRO VERDE, GRAND PLAZ, TOLON)</t>
+    <t>SHORT PLAYA CAB — PRODUCCIÓN SATÉLITE (841 – 896 und)</t>
+  </si>
+  <si>
+    <t>Global 941–1002 und − VELA prioritario 100 und = 841–896 und · resto tiendas (GRIETA, SAMBIL, CERRO VERDE, GRAND PLAZ, TOLON)</t>
+  </si>
+  <si>
+    <t>Rango producción: 841 – 896 und</t>
+  </si>
+  <si>
+    <t>MÍNIMO — 841 und</t>
   </si>
   <si>
     <t>TOTAL SATÉLITE</t>
   </si>
   <si>
-    <t>Resta VELA</t>
+    <t>MÁXIMO — 896 und (tope)</t>
+  </si>
+  <si>
+    <t>Detalle línea a línea (Mín / Máx):</t>
+  </si>
+  <si>
+    <t>Resta VELA mín</t>
+  </si>
+  <si>
+    <t>Resta VELA máx</t>
   </si>
 </sst>
 </file>
@@ -4252,7 +4267,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -4265,1137 +4280,1712 @@
         <v>114</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="4" t="s">
+    <row r="3" spans="1:8">
+      <c r="A3" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B6" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="G4" s="4" t="s">
+      <c r="F6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="4" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" t="s">
-        <v>101</v>
-      </c>
-      <c r="B5" t="s">
-        <v>75</v>
-      </c>
-      <c r="C5">
-        <v>26</v>
-      </c>
-      <c r="D5">
-        <v>55</v>
-      </c>
-      <c r="E5">
-        <v>70</v>
-      </c>
-      <c r="F5">
-        <v>40</v>
-      </c>
-      <c r="G5">
-        <v>29</v>
-      </c>
-      <c r="H5">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" t="s">
-        <v>79</v>
-      </c>
-      <c r="B6" t="s">
-        <v>79</v>
-      </c>
-      <c r="C6">
-        <v>21</v>
-      </c>
-      <c r="D6">
-        <v>44</v>
-      </c>
-      <c r="E6">
-        <v>56</v>
-      </c>
-      <c r="F6">
-        <v>32</v>
-      </c>
-      <c r="G6">
-        <v>23</v>
-      </c>
-      <c r="H6">
-        <v>176</v>
+      <c r="H6" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B7" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="C7">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D7">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="E7">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="F7">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="G7">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="H7">
-        <v>174</v>
+        <v>220</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B8" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="C8">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="D8">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="E8">
-        <v>26</v>
+        <v>56</v>
       </c>
       <c r="F8">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="G8">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="H8">
-        <v>82</v>
+        <v>176</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B9" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="C9">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D9">
-        <v>16</v>
+        <v>43</v>
       </c>
       <c r="E9">
-        <v>21</v>
+        <v>56</v>
       </c>
       <c r="F9">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="G9">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="H9">
-        <v>66</v>
+        <v>174</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B10" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="C10">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D10">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="E10">
+        <v>26</v>
+      </c>
+      <c r="F10">
+        <v>15</v>
+      </c>
+      <c r="G10">
         <v>11</v>
       </c>
-      <c r="F10">
-        <v>6</v>
-      </c>
-      <c r="G10">
-        <v>8</v>
-      </c>
       <c r="H10">
-        <v>38</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="B11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="C11">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D11">
+        <v>16</v>
+      </c>
+      <c r="E11">
+        <v>21</v>
+      </c>
+      <c r="F11">
+        <v>12</v>
+      </c>
+      <c r="G11">
         <v>9</v>
       </c>
-      <c r="E11">
-        <v>11</v>
-      </c>
-      <c r="F11">
-        <v>6</v>
-      </c>
-      <c r="G11">
-        <v>8</v>
-      </c>
       <c r="H11">
-        <v>38</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B12" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="C12">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D12">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E12">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G12">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H12">
-        <v>32</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
+        <v>94</v>
+      </c>
+      <c r="B13" t="s">
+        <v>94</v>
+      </c>
+      <c r="C13">
+        <v>4</v>
+      </c>
+      <c r="D13">
+        <v>9</v>
+      </c>
+      <c r="E13">
+        <v>11</v>
+      </c>
+      <c r="F13">
+        <v>6</v>
+      </c>
+      <c r="G13">
+        <v>8</v>
+      </c>
+      <c r="H13">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" t="s">
+        <v>96</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14">
+        <v>8</v>
+      </c>
+      <c r="E14">
+        <v>10</v>
+      </c>
+      <c r="F14">
+        <v>5</v>
+      </c>
+      <c r="G14">
+        <v>6</v>
+      </c>
+      <c r="H14">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" t="s">
         <v>98</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B15" t="s">
         <v>98</v>
       </c>
-      <c r="C13">
+      <c r="C15">
         <v>2</v>
       </c>
-      <c r="D13">
+      <c r="D15">
         <v>4</v>
       </c>
-      <c r="E13">
+      <c r="E15">
         <v>4</v>
       </c>
-      <c r="F13">
+      <c r="F15">
         <v>2</v>
       </c>
-      <c r="G13">
+      <c r="G15">
         <v>3</v>
       </c>
-      <c r="H13">
+      <c r="H15">
         <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="A14" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3">
-        <v>99</v>
-      </c>
-      <c r="D14" s="3">
-        <v>208</v>
-      </c>
-      <c r="E14" s="3">
-        <v>265</v>
-      </c>
-      <c r="F14" s="3">
-        <v>149</v>
-      </c>
-      <c r="G14" s="3">
-        <v>120</v>
-      </c>
-      <c r="H14" s="3">
-        <v>841</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="3" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
-      <c r="A17" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3">
+        <v>99</v>
+      </c>
+      <c r="D16" s="3">
+        <v>208</v>
+      </c>
+      <c r="E16" s="3">
+        <v>265</v>
+      </c>
+      <c r="F16" s="3">
+        <v>149</v>
+      </c>
+      <c r="G16" s="3">
+        <v>120</v>
+      </c>
+      <c r="H16" s="3">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B19" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" t="s">
-        <v>101</v>
-      </c>
-      <c r="B18" t="s">
-        <v>75</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="C19" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G19" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D18">
-        <v>29</v>
-      </c>
-      <c r="E18">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6">
-      <c r="A19" t="s">
-        <v>101</v>
-      </c>
-      <c r="B19" t="s">
-        <v>75</v>
-      </c>
-      <c r="C19" t="s">
-        <v>7</v>
-      </c>
-      <c r="D19">
-        <v>70</v>
-      </c>
-      <c r="E19">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6">
+      <c r="H19" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20" t="s">
         <v>101</v>
       </c>
       <c r="B20" t="s">
         <v>75</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20">
+        <v>28</v>
+      </c>
+      <c r="D20">
+        <v>59</v>
+      </c>
+      <c r="E20">
+        <v>75</v>
+      </c>
+      <c r="F20">
+        <v>42</v>
+      </c>
+      <c r="G20">
+        <v>30</v>
+      </c>
+      <c r="H20">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" t="s">
+        <v>79</v>
+      </c>
+      <c r="B21" t="s">
+        <v>79</v>
+      </c>
+      <c r="C21">
+        <v>22</v>
+      </c>
+      <c r="D21">
+        <v>47</v>
+      </c>
+      <c r="E21">
+        <v>60</v>
+      </c>
+      <c r="F21">
+        <v>33</v>
+      </c>
+      <c r="G21">
+        <v>24</v>
+      </c>
+      <c r="H21">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" t="s">
+        <v>102</v>
+      </c>
+      <c r="B22" t="s">
+        <v>82</v>
+      </c>
+      <c r="C22">
+        <v>22</v>
+      </c>
+      <c r="D22">
+        <v>46</v>
+      </c>
+      <c r="E22">
+        <v>59</v>
+      </c>
+      <c r="F22">
+        <v>34</v>
+      </c>
+      <c r="G22">
+        <v>24</v>
+      </c>
+      <c r="H22">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" t="s">
+        <v>85</v>
+      </c>
+      <c r="B23" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23">
+        <v>11</v>
+      </c>
+      <c r="D23">
+        <v>22</v>
+      </c>
+      <c r="E23">
+        <v>28</v>
+      </c>
+      <c r="F23">
+        <v>16</v>
+      </c>
+      <c r="G23">
+        <v>11</v>
+      </c>
+      <c r="H23">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" t="s">
+        <v>103</v>
+      </c>
+      <c r="B24" t="s">
+        <v>88</v>
+      </c>
+      <c r="C24">
+        <v>8</v>
+      </c>
+      <c r="D24">
+        <v>18</v>
+      </c>
+      <c r="E24">
+        <v>23</v>
+      </c>
+      <c r="F24">
+        <v>13</v>
+      </c>
+      <c r="G24">
+        <v>9</v>
+      </c>
+      <c r="H24">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" t="s">
+        <v>91</v>
+      </c>
+      <c r="B25" t="s">
+        <v>91</v>
+      </c>
+      <c r="C25">
+        <v>4</v>
+      </c>
+      <c r="D25">
+        <v>10</v>
+      </c>
+      <c r="E25">
+        <v>12</v>
+      </c>
+      <c r="F25">
+        <v>7</v>
+      </c>
+      <c r="G25">
+        <v>8</v>
+      </c>
+      <c r="H25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" t="s">
+        <v>94</v>
+      </c>
+      <c r="B26" t="s">
+        <v>94</v>
+      </c>
+      <c r="C26">
+        <v>4</v>
+      </c>
+      <c r="D26">
+        <v>10</v>
+      </c>
+      <c r="E26">
+        <v>12</v>
+      </c>
+      <c r="F26">
+        <v>7</v>
+      </c>
+      <c r="G26">
+        <v>8</v>
+      </c>
+      <c r="H26">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27" t="s">
+        <v>96</v>
+      </c>
+      <c r="B27" t="s">
+        <v>96</v>
+      </c>
+      <c r="C27">
+        <v>3</v>
+      </c>
+      <c r="D27">
+        <v>8</v>
+      </c>
+      <c r="E27">
+        <v>10</v>
+      </c>
+      <c r="F27">
         <v>6</v>
       </c>
-      <c r="D20">
-        <v>55</v>
-      </c>
-      <c r="E20">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21" t="s">
+      <c r="G27">
+        <v>7</v>
+      </c>
+      <c r="H27">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
+      <c r="A28" t="s">
+        <v>98</v>
+      </c>
+      <c r="B28" t="s">
+        <v>98</v>
+      </c>
+      <c r="C28">
+        <v>2</v>
+      </c>
+      <c r="D28">
+        <v>4</v>
+      </c>
+      <c r="E28">
+        <v>5</v>
+      </c>
+      <c r="F28">
+        <v>2</v>
+      </c>
+      <c r="G28">
+        <v>3</v>
+      </c>
+      <c r="H28">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
+      <c r="A29" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3">
+        <v>104</v>
+      </c>
+      <c r="D29" s="3">
+        <v>224</v>
+      </c>
+      <c r="E29" s="3">
+        <v>284</v>
+      </c>
+      <c r="F29" s="3">
+        <v>160</v>
+      </c>
+      <c r="G29" s="3">
+        <v>124</v>
+      </c>
+      <c r="H29" s="3">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
+      <c r="A31" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="A32" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33" t="s">
         <v>101</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B33" t="s">
         <v>75</v>
-      </c>
-      <c r="C21" t="s">
-        <v>5</v>
-      </c>
-      <c r="D21">
-        <v>26</v>
-      </c>
-      <c r="E21">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6">
-      <c r="A22" t="s">
-        <v>101</v>
-      </c>
-      <c r="B22" t="s">
-        <v>75</v>
-      </c>
-      <c r="C22" t="s">
-        <v>8</v>
-      </c>
-      <c r="D22">
-        <v>40</v>
-      </c>
-      <c r="E22">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6">
-      <c r="A23" t="s">
-        <v>79</v>
-      </c>
-      <c r="B23" t="s">
-        <v>79</v>
-      </c>
-      <c r="C23" t="s">
-        <v>9</v>
-      </c>
-      <c r="D23">
-        <v>23</v>
-      </c>
-      <c r="E23">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6">
-      <c r="A24" t="s">
-        <v>79</v>
-      </c>
-      <c r="B24" t="s">
-        <v>79</v>
-      </c>
-      <c r="C24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24">
-        <v>56</v>
-      </c>
-      <c r="E24">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6">
-      <c r="A25" t="s">
-        <v>79</v>
-      </c>
-      <c r="B25" t="s">
-        <v>79</v>
-      </c>
-      <c r="C25" t="s">
-        <v>6</v>
-      </c>
-      <c r="D25">
-        <v>44</v>
-      </c>
-      <c r="E25">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6">
-      <c r="A26" t="s">
-        <v>79</v>
-      </c>
-      <c r="B26" t="s">
-        <v>79</v>
-      </c>
-      <c r="C26" t="s">
-        <v>5</v>
-      </c>
-      <c r="D26">
-        <v>21</v>
-      </c>
-      <c r="E26">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6">
-      <c r="A27" t="s">
-        <v>79</v>
-      </c>
-      <c r="B27" t="s">
-        <v>79</v>
-      </c>
-      <c r="C27" t="s">
-        <v>8</v>
-      </c>
-      <c r="D27">
-        <v>32</v>
-      </c>
-      <c r="E27">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6">
-      <c r="A28" t="s">
-        <v>102</v>
-      </c>
-      <c r="B28" t="s">
-        <v>82</v>
-      </c>
-      <c r="C28" t="s">
-        <v>9</v>
-      </c>
-      <c r="D28">
-        <v>23</v>
-      </c>
-      <c r="E28">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6">
-      <c r="A29" t="s">
-        <v>102</v>
-      </c>
-      <c r="B29" t="s">
-        <v>82</v>
-      </c>
-      <c r="C29" t="s">
-        <v>7</v>
-      </c>
-      <c r="D29">
-        <v>56</v>
-      </c>
-      <c r="E29">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6">
-      <c r="A30" t="s">
-        <v>102</v>
-      </c>
-      <c r="B30" t="s">
-        <v>82</v>
-      </c>
-      <c r="C30" t="s">
-        <v>6</v>
-      </c>
-      <c r="D30">
-        <v>43</v>
-      </c>
-      <c r="E30">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6">
-      <c r="A31" t="s">
-        <v>102</v>
-      </c>
-      <c r="B31" t="s">
-        <v>82</v>
-      </c>
-      <c r="C31" t="s">
-        <v>5</v>
-      </c>
-      <c r="D31">
-        <v>21</v>
-      </c>
-      <c r="E31">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6">
-      <c r="A32" t="s">
-        <v>102</v>
-      </c>
-      <c r="B32" t="s">
-        <v>82</v>
-      </c>
-      <c r="C32" t="s">
-        <v>8</v>
-      </c>
-      <c r="D32">
-        <v>31</v>
-      </c>
-      <c r="E32">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6">
-      <c r="A33" t="s">
-        <v>85</v>
-      </c>
-      <c r="B33" t="s">
-        <v>85</v>
       </c>
       <c r="C33" t="s">
         <v>9</v>
       </c>
       <c r="D33">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="E33">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6">
+        <v>30</v>
+      </c>
+      <c r="F33">
+        <v>20</v>
+      </c>
+      <c r="G33">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
       <c r="A34" t="s">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="B34" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="C34" t="s">
         <v>7</v>
       </c>
       <c r="D34">
-        <v>26</v>
+        <v>70</v>
       </c>
       <c r="E34">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6">
+        <v>75</v>
+      </c>
+      <c r="F34">
+        <v>20</v>
+      </c>
+      <c r="G34">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="B35" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="C35" t="s">
         <v>6</v>
       </c>
       <c r="D35">
+        <v>55</v>
+      </c>
+      <c r="E35">
+        <v>59</v>
+      </c>
+      <c r="F35">
         <v>20</v>
       </c>
-      <c r="E35">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6">
+      <c r="G35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
       <c r="A36" t="s">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="B36" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="C36" t="s">
         <v>5</v>
       </c>
       <c r="D36">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="E36">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6">
+        <v>28</v>
+      </c>
+      <c r="F36">
+        <v>20</v>
+      </c>
+      <c r="G36">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
       <c r="A37" t="s">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="B37" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="C37" t="s">
         <v>8</v>
       </c>
       <c r="D37">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="E37">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6">
+        <v>42</v>
+      </c>
+      <c r="F37">
+        <v>20</v>
+      </c>
+      <c r="G37">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
       <c r="A38" t="s">
-        <v>103</v>
+        <v>79</v>
       </c>
       <c r="B38" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="C38" t="s">
         <v>9</v>
       </c>
       <c r="D38">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="E38">
+        <v>24</v>
+      </c>
+      <c r="F38">
         <v>20</v>
       </c>
-    </row>
-    <row r="39" spans="1:6">
+      <c r="G38">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
       <c r="A39" t="s">
-        <v>103</v>
+        <v>79</v>
       </c>
       <c r="B39" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="C39" t="s">
         <v>7</v>
       </c>
       <c r="D39">
-        <v>21</v>
+        <v>56</v>
       </c>
       <c r="E39">
+        <v>60</v>
+      </c>
+      <c r="F39">
         <v>20</v>
       </c>
-    </row>
-    <row r="40" spans="1:6">
+      <c r="G39">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
       <c r="A40" t="s">
-        <v>103</v>
+        <v>79</v>
       </c>
       <c r="B40" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="C40" t="s">
         <v>6</v>
       </c>
       <c r="D40">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="E40">
+        <v>47</v>
+      </c>
+      <c r="F40">
         <v>20</v>
       </c>
-    </row>
-    <row r="41" spans="1:6">
+      <c r="G40">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
       <c r="A41" t="s">
-        <v>103</v>
+        <v>79</v>
       </c>
       <c r="B41" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="C41" t="s">
         <v>5</v>
       </c>
       <c r="D41">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="E41">
+        <v>22</v>
+      </c>
+      <c r="F41">
         <v>20</v>
       </c>
-    </row>
-    <row r="42" spans="1:6">
+      <c r="G41">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
       <c r="A42" t="s">
-        <v>103</v>
+        <v>79</v>
       </c>
       <c r="B42" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="C42" t="s">
         <v>8</v>
       </c>
       <c r="D42">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="E42">
+        <v>33</v>
+      </c>
+      <c r="F42">
         <v>20</v>
       </c>
-    </row>
-    <row r="43" spans="1:6">
+      <c r="G42">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
       <c r="A43" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="B43" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="C43" t="s">
         <v>9</v>
       </c>
       <c r="D43">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="E43">
-        <v>0</v>
-      </c>
-      <c r="F43" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6">
+        <v>24</v>
+      </c>
+      <c r="F43">
+        <v>21</v>
+      </c>
+      <c r="G43">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="B44" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="C44" t="s">
         <v>7</v>
       </c>
       <c r="D44">
-        <v>11</v>
+        <v>56</v>
       </c>
       <c r="E44">
-        <v>0</v>
-      </c>
-      <c r="F44" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6">
+        <v>59</v>
+      </c>
+      <c r="F44">
+        <v>21</v>
+      </c>
+      <c r="G44">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
       <c r="A45" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="B45" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="C45" t="s">
         <v>6</v>
       </c>
       <c r="D45">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="E45">
-        <v>0</v>
-      </c>
-      <c r="F45" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6">
+        <v>46</v>
+      </c>
+      <c r="F45">
+        <v>21</v>
+      </c>
+      <c r="G45">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
       <c r="A46" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="B46" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="C46" t="s">
         <v>5</v>
       </c>
       <c r="D46">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="E46">
-        <v>0</v>
-      </c>
-      <c r="F46" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6">
+        <v>22</v>
+      </c>
+      <c r="F46">
+        <v>21</v>
+      </c>
+      <c r="G46">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
       <c r="A47" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="B47" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="C47" t="s">
         <v>8</v>
       </c>
       <c r="D47">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="E47">
-        <v>0</v>
-      </c>
-      <c r="F47" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6">
+        <v>34</v>
+      </c>
+      <c r="F47">
+        <v>21</v>
+      </c>
+      <c r="G47">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
       <c r="A48" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B48" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="C48" t="s">
         <v>9</v>
       </c>
       <c r="D48">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E48">
-        <v>0</v>
-      </c>
-      <c r="F48" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6">
+        <v>11</v>
+      </c>
+      <c r="F48">
+        <v>19</v>
+      </c>
+      <c r="G48">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
       <c r="A49" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B49" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="C49" t="s">
         <v>7</v>
       </c>
       <c r="D49">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="E49">
-        <v>0</v>
-      </c>
-      <c r="F49" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6">
+        <v>28</v>
+      </c>
+      <c r="F49">
+        <v>19</v>
+      </c>
+      <c r="G49">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
       <c r="A50" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B50" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="C50" t="s">
         <v>6</v>
       </c>
       <c r="D50">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="E50">
-        <v>0</v>
-      </c>
-      <c r="F50" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6">
+        <v>22</v>
+      </c>
+      <c r="F50">
+        <v>19</v>
+      </c>
+      <c r="G50">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
       <c r="A51" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B51" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="C51" t="s">
         <v>5</v>
       </c>
       <c r="D51">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E51">
-        <v>0</v>
-      </c>
-      <c r="F51" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6">
+        <v>11</v>
+      </c>
+      <c r="F51">
+        <v>19</v>
+      </c>
+      <c r="G51">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
       <c r="A52" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B52" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="C52" t="s">
         <v>8</v>
       </c>
       <c r="D52">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E52">
-        <v>0</v>
-      </c>
-      <c r="F52" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6">
+        <v>16</v>
+      </c>
+      <c r="F52">
+        <v>19</v>
+      </c>
+      <c r="G52">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
       <c r="A53" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="B53" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C53" t="s">
         <v>9</v>
       </c>
       <c r="D53">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E53">
-        <v>0</v>
-      </c>
-      <c r="F53" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6">
+        <v>9</v>
+      </c>
+      <c r="F53">
+        <v>20</v>
+      </c>
+      <c r="G53">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
       <c r="A54" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="B54" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C54" t="s">
         <v>7</v>
       </c>
       <c r="D54">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E54">
-        <v>0</v>
-      </c>
-      <c r="F54" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6">
+        <v>23</v>
+      </c>
+      <c r="F54">
+        <v>20</v>
+      </c>
+      <c r="G54">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
       <c r="A55" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="B55" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C55" t="s">
         <v>6</v>
       </c>
       <c r="D55">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E55">
-        <v>0</v>
-      </c>
-      <c r="F55" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6">
+        <v>18</v>
+      </c>
+      <c r="F55">
+        <v>20</v>
+      </c>
+      <c r="G55">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8">
       <c r="A56" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="B56" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C56" t="s">
         <v>5</v>
       </c>
       <c r="D56">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E56">
-        <v>0</v>
-      </c>
-      <c r="F56" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="F56">
+        <v>20</v>
+      </c>
+      <c r="G56">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
       <c r="A57" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="B57" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C57" t="s">
         <v>8</v>
       </c>
       <c r="D57">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E57">
-        <v>0</v>
-      </c>
-      <c r="F57" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6">
+        <v>13</v>
+      </c>
+      <c r="F57">
+        <v>20</v>
+      </c>
+      <c r="G57">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
       <c r="A58" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B58" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C58" t="s">
         <v>9</v>
       </c>
       <c r="D58">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E58">
-        <v>0</v>
-      </c>
-      <c r="F58" t="s">
+        <v>8</v>
+      </c>
+      <c r="F58">
+        <v>0</v>
+      </c>
+      <c r="G58">
+        <v>0</v>
+      </c>
+      <c r="H58" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="59" spans="1:6">
+    <row r="59" spans="1:8">
       <c r="A59" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B59" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C59" t="s">
         <v>7</v>
       </c>
       <c r="D59">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E59">
-        <v>0</v>
-      </c>
-      <c r="F59" t="s">
+        <v>12</v>
+      </c>
+      <c r="F59">
+        <v>0</v>
+      </c>
+      <c r="G59">
+        <v>0</v>
+      </c>
+      <c r="H59" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="60" spans="1:6">
+    <row r="60" spans="1:8">
       <c r="A60" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B60" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C60" t="s">
         <v>6</v>
       </c>
       <c r="D60">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E60">
-        <v>0</v>
-      </c>
-      <c r="F60" t="s">
+        <v>10</v>
+      </c>
+      <c r="F60">
+        <v>0</v>
+      </c>
+      <c r="G60">
+        <v>0</v>
+      </c>
+      <c r="H60" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="61" spans="1:6">
+    <row r="61" spans="1:8">
       <c r="A61" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B61" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C61" t="s">
         <v>5</v>
       </c>
       <c r="D61">
+        <v>4</v>
+      </c>
+      <c r="E61">
+        <v>4</v>
+      </c>
+      <c r="F61">
+        <v>0</v>
+      </c>
+      <c r="G61">
+        <v>0</v>
+      </c>
+      <c r="H61" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8">
+      <c r="A62" t="s">
+        <v>94</v>
+      </c>
+      <c r="B62" t="s">
+        <v>94</v>
+      </c>
+      <c r="C62" t="s">
+        <v>8</v>
+      </c>
+      <c r="D62">
+        <v>6</v>
+      </c>
+      <c r="E62">
+        <v>7</v>
+      </c>
+      <c r="F62">
+        <v>0</v>
+      </c>
+      <c r="G62">
+        <v>0</v>
+      </c>
+      <c r="H62" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8">
+      <c r="A63" t="s">
+        <v>91</v>
+      </c>
+      <c r="B63" t="s">
+        <v>91</v>
+      </c>
+      <c r="C63" t="s">
+        <v>9</v>
+      </c>
+      <c r="D63">
+        <v>8</v>
+      </c>
+      <c r="E63">
+        <v>8</v>
+      </c>
+      <c r="F63">
+        <v>0</v>
+      </c>
+      <c r="G63">
+        <v>0</v>
+      </c>
+      <c r="H63" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64" t="s">
+        <v>91</v>
+      </c>
+      <c r="C64" t="s">
+        <v>7</v>
+      </c>
+      <c r="D64">
+        <v>11</v>
+      </c>
+      <c r="E64">
+        <v>12</v>
+      </c>
+      <c r="F64">
+        <v>0</v>
+      </c>
+      <c r="G64">
+        <v>0</v>
+      </c>
+      <c r="H64" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8">
+      <c r="A65" t="s">
+        <v>91</v>
+      </c>
+      <c r="B65" t="s">
+        <v>91</v>
+      </c>
+      <c r="C65" t="s">
+        <v>6</v>
+      </c>
+      <c r="D65">
+        <v>9</v>
+      </c>
+      <c r="E65">
+        <v>10</v>
+      </c>
+      <c r="F65">
+        <v>0</v>
+      </c>
+      <c r="G65">
+        <v>0</v>
+      </c>
+      <c r="H65" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8">
+      <c r="A66" t="s">
+        <v>91</v>
+      </c>
+      <c r="B66" t="s">
+        <v>91</v>
+      </c>
+      <c r="C66" t="s">
+        <v>5</v>
+      </c>
+      <c r="D66">
+        <v>4</v>
+      </c>
+      <c r="E66">
+        <v>4</v>
+      </c>
+      <c r="F66">
+        <v>0</v>
+      </c>
+      <c r="G66">
+        <v>0</v>
+      </c>
+      <c r="H66" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8">
+      <c r="A67" t="s">
+        <v>91</v>
+      </c>
+      <c r="B67" t="s">
+        <v>91</v>
+      </c>
+      <c r="C67" t="s">
+        <v>8</v>
+      </c>
+      <c r="D67">
+        <v>6</v>
+      </c>
+      <c r="E67">
+        <v>7</v>
+      </c>
+      <c r="F67">
+        <v>0</v>
+      </c>
+      <c r="G67">
+        <v>0</v>
+      </c>
+      <c r="H67" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8">
+      <c r="A68" t="s">
+        <v>96</v>
+      </c>
+      <c r="B68" t="s">
+        <v>96</v>
+      </c>
+      <c r="C68" t="s">
+        <v>9</v>
+      </c>
+      <c r="D68">
+        <v>6</v>
+      </c>
+      <c r="E68">
+        <v>7</v>
+      </c>
+      <c r="F68">
+        <v>0</v>
+      </c>
+      <c r="G68">
+        <v>0</v>
+      </c>
+      <c r="H68" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69" t="s">
+        <v>96</v>
+      </c>
+      <c r="C69" t="s">
+        <v>7</v>
+      </c>
+      <c r="D69">
+        <v>10</v>
+      </c>
+      <c r="E69">
+        <v>10</v>
+      </c>
+      <c r="F69">
+        <v>0</v>
+      </c>
+      <c r="G69">
+        <v>0</v>
+      </c>
+      <c r="H69" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8">
+      <c r="A70" t="s">
+        <v>96</v>
+      </c>
+      <c r="B70" t="s">
+        <v>96</v>
+      </c>
+      <c r="C70" t="s">
+        <v>6</v>
+      </c>
+      <c r="D70">
+        <v>8</v>
+      </c>
+      <c r="E70">
+        <v>8</v>
+      </c>
+      <c r="F70">
+        <v>0</v>
+      </c>
+      <c r="G70">
+        <v>0</v>
+      </c>
+      <c r="H70" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8">
+      <c r="A71" t="s">
+        <v>96</v>
+      </c>
+      <c r="B71" t="s">
+        <v>96</v>
+      </c>
+      <c r="C71" t="s">
+        <v>5</v>
+      </c>
+      <c r="D71">
+        <v>3</v>
+      </c>
+      <c r="E71">
+        <v>3</v>
+      </c>
+      <c r="F71">
+        <v>0</v>
+      </c>
+      <c r="G71">
+        <v>0</v>
+      </c>
+      <c r="H71" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8">
+      <c r="A72" t="s">
+        <v>96</v>
+      </c>
+      <c r="B72" t="s">
+        <v>96</v>
+      </c>
+      <c r="C72" t="s">
+        <v>8</v>
+      </c>
+      <c r="D72">
+        <v>5</v>
+      </c>
+      <c r="E72">
+        <v>6</v>
+      </c>
+      <c r="F72">
+        <v>0</v>
+      </c>
+      <c r="G72">
+        <v>0</v>
+      </c>
+      <c r="H72" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8">
+      <c r="A73" t="s">
+        <v>98</v>
+      </c>
+      <c r="B73" t="s">
+        <v>98</v>
+      </c>
+      <c r="C73" t="s">
+        <v>9</v>
+      </c>
+      <c r="D73">
+        <v>3</v>
+      </c>
+      <c r="E73">
+        <v>3</v>
+      </c>
+      <c r="F73">
+        <v>0</v>
+      </c>
+      <c r="G73">
+        <v>0</v>
+      </c>
+      <c r="H73" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8">
+      <c r="A74" t="s">
+        <v>98</v>
+      </c>
+      <c r="B74" t="s">
+        <v>98</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>4</v>
+      </c>
+      <c r="E74">
+        <v>5</v>
+      </c>
+      <c r="F74">
+        <v>0</v>
+      </c>
+      <c r="G74">
+        <v>0</v>
+      </c>
+      <c r="H74" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8">
+      <c r="A75" t="s">
+        <v>98</v>
+      </c>
+      <c r="B75" t="s">
+        <v>98</v>
+      </c>
+      <c r="C75" t="s">
+        <v>6</v>
+      </c>
+      <c r="D75">
+        <v>4</v>
+      </c>
+      <c r="E75">
+        <v>4</v>
+      </c>
+      <c r="F75">
+        <v>0</v>
+      </c>
+      <c r="G75">
+        <v>0</v>
+      </c>
+      <c r="H75" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8">
+      <c r="A76" t="s">
+        <v>98</v>
+      </c>
+      <c r="B76" t="s">
+        <v>98</v>
+      </c>
+      <c r="C76" t="s">
+        <v>5</v>
+      </c>
+      <c r="D76">
         <v>2</v>
       </c>
-      <c r="E61">
-        <v>0</v>
-      </c>
-      <c r="F61" t="s">
+      <c r="E76">
+        <v>2</v>
+      </c>
+      <c r="F76">
+        <v>0</v>
+      </c>
+      <c r="G76">
+        <v>0</v>
+      </c>
+      <c r="H76" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="62" spans="1:6">
-      <c r="A62" t="s">
+    <row r="77" spans="1:8">
+      <c r="A77" t="s">
         <v>98</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B77" t="s">
         <v>98</v>
       </c>
-      <c r="C62" t="s">
-        <v>8</v>
-      </c>
-      <c r="D62">
+      <c r="C77" t="s">
+        <v>8</v>
+      </c>
+      <c r="D77">
         <v>2</v>
       </c>
-      <c r="E62">
-        <v>0</v>
-      </c>
-      <c r="F62" t="s">
+      <c r="E77">
+        <v>2</v>
+      </c>
+      <c r="F77">
+        <v>0</v>
+      </c>
+      <c r="G77">
+        <v>0</v>
+      </c>
+      <c r="H77" t="s">
         <v>112</v>
       </c>
     </row>

</xml_diff>